<commit_message>
Publish Latest checklists 2026-03-18
Updates based on OWASP/wstg@ae3e640
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3817,7 +3817,7 @@
         </is>
       </c>
       <c r="C105" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Encryption", "Testing for Weak Encryption")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -4595,38 +4595,63 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="66" customHeight="1" s="82">
+    <row r="139" ht="132" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-03</t>
+        </is>
+      </c>
+      <c r="C139" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
+        <v/>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>- Identify API responses that contain more data than what the client application displays or requires.
+- Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
+- Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="66" customHeight="1" s="82">
+      <c r="A140" s="19" t="n"/>
+      <c r="B140" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C140" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="82">
-      <c r="A140" s="97" t="n"/>
-      <c r="B140" s="98" t="n"/>
-      <c r="C140" s="99" t="n"/>
-      <c r="D140" s="99" t="n"/>
-      <c r="E140" s="99" t="n"/>
-      <c r="F140" s="99" t="n"/>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="82">
+      <c r="A141" s="97" t="n"/>
+      <c r="B141" s="98" t="n"/>
+      <c r="C141" s="99" t="n"/>
+      <c r="D141" s="99" t="n"/>
+      <c r="E141" s="99" t="n"/>
+      <c r="F141" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4643,7 +4668,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F140">
+  <conditionalFormatting sqref="B4:F141">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4655,7 +4680,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-03-18 (#1369)
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3817,7 +3817,7 @@
         </is>
       </c>
       <c r="C105" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Encryption", "Testing for Weak Encryption")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -4595,38 +4595,63 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="66" customHeight="1" s="82">
+    <row r="139" ht="132" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-03</t>
+        </is>
+      </c>
+      <c r="C139" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
+        <v/>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>- Identify API responses that contain more data than what the client application displays or requires.
+- Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
+- Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="66" customHeight="1" s="82">
+      <c r="A140" s="19" t="n"/>
+      <c r="B140" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C140" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="82">
-      <c r="A140" s="97" t="n"/>
-      <c r="B140" s="98" t="n"/>
-      <c r="C140" s="99" t="n"/>
-      <c r="D140" s="99" t="n"/>
-      <c r="E140" s="99" t="n"/>
-      <c r="F140" s="99" t="n"/>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="82">
+      <c r="A141" s="97" t="n"/>
+      <c r="B141" s="98" t="n"/>
+      <c r="C141" s="99" t="n"/>
+      <c r="D141" s="99" t="n"/>
+      <c r="E141" s="99" t="n"/>
+      <c r="F141" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4643,7 +4668,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F140">
+  <conditionalFormatting sqref="B4:F141">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4655,7 +4680,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-04-10
Updates based on OWASP/wstg@bfc7be7
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -4620,38 +4620,61 @@
       </c>
       <c r="F139" s="18" t="n"/>
     </row>
-    <row r="140" ht="66" customHeight="1" s="82">
+    <row r="140" ht="82.5" customHeight="1" s="82">
       <c r="A140" s="19" t="n"/>
       <c r="B140" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-03</t>
+        </is>
+      </c>
+      <c r="C140" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D140" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="66" customHeight="1" s="82">
+      <c r="A141" s="19" t="n"/>
+      <c r="B141" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C140" s="15">
+      <c r="C141" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D140" s="16" t="inlineStr">
+      <c r="D141" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="82">
-      <c r="A141" s="97" t="n"/>
-      <c r="B141" s="98" t="n"/>
-      <c r="C141" s="99" t="n"/>
-      <c r="D141" s="99" t="n"/>
-      <c r="E141" s="99" t="n"/>
-      <c r="F141" s="99" t="n"/>
+      <c r="E141" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F141" s="18" t="n"/>
+    </row>
+    <row r="142" ht="15" customHeight="1" s="82">
+      <c r="A142" s="97" t="n"/>
+      <c r="B142" s="98" t="n"/>
+      <c r="C142" s="99" t="n"/>
+      <c r="D142" s="99" t="n"/>
+      <c r="E142" s="99" t="n"/>
+      <c r="F142" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4668,7 +4691,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F141">
+  <conditionalFormatting sqref="B4:F142">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4680,7 +4703,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-04-10 (#1398)
Updates based on OWASP/wstg@bfc7be7
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -4620,38 +4620,61 @@
       </c>
       <c r="F139" s="18" t="n"/>
     </row>
-    <row r="140" ht="66" customHeight="1" s="82">
+    <row r="140" ht="82.5" customHeight="1" s="82">
       <c r="A140" s="19" t="n"/>
       <c r="B140" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-03</t>
+        </is>
+      </c>
+      <c r="C140" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D140" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="66" customHeight="1" s="82">
+      <c r="A141" s="19" t="n"/>
+      <c r="B141" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C140" s="15">
+      <c r="C141" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D140" s="16" t="inlineStr">
+      <c r="D141" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="82">
-      <c r="A141" s="97" t="n"/>
-      <c r="B141" s="98" t="n"/>
-      <c r="C141" s="99" t="n"/>
-      <c r="D141" s="99" t="n"/>
-      <c r="E141" s="99" t="n"/>
-      <c r="F141" s="99" t="n"/>
+      <c r="E141" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F141" s="18" t="n"/>
+    </row>
+    <row r="142" ht="15" customHeight="1" s="82">
+      <c r="A142" s="97" t="n"/>
+      <c r="B142" s="98" t="n"/>
+      <c r="C142" s="99" t="n"/>
+      <c r="D142" s="99" t="n"/>
+      <c r="E142" s="99" t="n"/>
+      <c r="F142" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4668,7 +4691,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F141">
+  <conditionalFormatting sqref="B4:F142">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4680,7 +4703,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-04-22
Updates based on OWASP/wstg@2ec67f9
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -1983,16 +1983,16 @@
       <c r="A25" s="19" t="n"/>
       <c r="B25" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-08</t>
+          <t>WSTG-CONF-09</t>
         </is>
       </c>
       <c r="C25" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/08-Test_RIA_Cross_Domain_Policy", "Test RIA Cross Domain Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/09-Test_File_Permission", "Test File Permission")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- Review and identify any rogue file permissions.</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -2002,20 +2002,21 @@
       </c>
       <c r="F25" s="18" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="82">
+    <row r="26" ht="33" customHeight="1" s="82">
       <c r="A26" s="19" t="n"/>
       <c r="B26" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-09</t>
+          <t>WSTG-CONF-10</t>
         </is>
       </c>
       <c r="C26" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/09-Test_File_Permission", "Test File Permission")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/10-Test_for_Subdomain_Takeover", "Test for Subdomain Takeover")</f>
         <v/>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>- Review and identify any rogue file permissions.</t>
+          <t>- Enumerate all possible domains (previous and current).
+- Identify any forgotten or misconfigured domains.</t>
         </is>
       </c>
       <c r="E26" s="18" t="inlineStr">
@@ -2029,17 +2030,16 @@
       <c r="A27" s="19" t="n"/>
       <c r="B27" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-10</t>
+          <t>WSTG-CONF-11</t>
         </is>
       </c>
       <c r="C27" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/10-Test_for_Subdomain_Takeover", "Test for Subdomain Takeover")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/11-Test_Cloud_Storage", "Test Cloud Storage")</f>
         <v/>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>- Enumerate all possible domains (previous and current).
-- Identify any forgotten or misconfigured domains.</t>
+          <t>- Assess that the access control configuration for the storage services is properly in place.</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
@@ -2053,16 +2053,16 @@
       <c r="A28" s="19" t="n"/>
       <c r="B28" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-11</t>
+          <t>WSTG-CONF-12</t>
         </is>
       </c>
       <c r="C28" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/11-Test_Cloud_Storage", "Test Cloud Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Testing for Content Security Policy")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>- Assess that the access control configuration for the storage services is properly in place.</t>
+          <t>- Review the Content-Security-Policy header or meta element to identify misconfigurations.</t>
         </is>
       </c>
       <c r="E28" s="18" t="inlineStr">
@@ -2072,20 +2072,20 @@
       </c>
       <c r="F28" s="18" t="n"/>
     </row>
-    <row r="29" ht="33" customHeight="1" s="82">
+    <row r="29" ht="16.5" customHeight="1" s="82">
       <c r="A29" s="19" t="n"/>
       <c r="B29" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-12</t>
+          <t>WSTG-CONF-13</t>
         </is>
       </c>
       <c r="C29" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Testing for Content Security Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/13-Test_for_Path_Confusion", "Test Path Confusion")</f>
         <v/>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>- Review the Content-Security-Policy header or meta element to identify misconfigurations.</t>
+          <t>- Make sure application paths are configured correctly.</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">
@@ -2095,108 +2095,109 @@
       </c>
       <c r="F29" s="18" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="82">
+    <row r="30" ht="66" customHeight="1" s="82">
       <c r="A30" s="19" t="n"/>
       <c r="B30" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-13</t>
+          <t>WSTG-CONF-14</t>
         </is>
       </c>
       <c r="C30" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/13-Test_for_Path_Confusion", "Test Path Confusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/14-Test_Other_HTTP_Security_Header_Misconfigurations", "Test Other HTTP Security Header Misconfigurations")</f>
         <v/>
       </c>
       <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>- Make sure application paths are configured correctly.</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="n"/>
-    </row>
-    <row r="31" ht="66" customHeight="1" s="82">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CONF-14</t>
-        </is>
-      </c>
-      <c r="C31" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/14-Test_Other_HTTP_Security_Header_Misconfigurations", "Test Other HTTP Security Header Misconfigurations")</f>
-        <v/>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>- Identify improperly configured security headers.
 - Assess the impact of misconfigured security headers.
 - Validate the correct implementation of required security headers.</t>
         </is>
       </c>
-      <c r="E31" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F31" s="18" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="82">
-      <c r="A32" s="97" t="n"/>
-      <c r="B32" s="98" t="n"/>
-      <c r="C32" s="99" t="n"/>
-      <c r="D32" s="99" t="n"/>
-      <c r="E32" s="99" t="n"/>
-      <c r="F32" s="99" t="n"/>
-    </row>
-    <row r="33" ht="47.25" customHeight="1" s="82">
-      <c r="A33" s="9" t="n"/>
-      <c r="B33" s="100" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="82">
+      <c r="A31" s="97" t="n"/>
+      <c r="B31" s="98" t="n"/>
+      <c r="C31" s="99" t="n"/>
+      <c r="D31" s="99" t="n"/>
+      <c r="E31" s="99" t="n"/>
+      <c r="F31" s="99" t="n"/>
+    </row>
+    <row r="32" ht="47.25" customHeight="1" s="82">
+      <c r="A32" s="9" t="n"/>
+      <c r="B32" s="100" t="inlineStr">
         <is>
           <t>Identity Management Testing</t>
         </is>
       </c>
-      <c r="C33" s="101" t="inlineStr">
+      <c r="C32" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D33" s="101" t="inlineStr">
+      <c r="D32" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E33" s="101" t="inlineStr">
+      <c r="E32" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F33" s="101" t="inlineStr">
+      <c r="F32" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="66" customHeight="1" s="82">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="34" t="inlineStr">
+    <row r="33" ht="66" customHeight="1" s="82">
+      <c r="A33" s="19" t="n"/>
+      <c r="B33" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-01</t>
         </is>
       </c>
-      <c r="C34" s="15">
+      <c r="C33" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/01-Test_Role_Definitions", "Test Role Definitions")</f>
         <v/>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>- Identify and document roles used by the application.
 - Attempt to switch, change, or access another role.
 - Review the granularity of the roles and the needs behind the permissions given.</t>
         </is>
       </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F33" s="18" t="n"/>
+    </row>
+    <row r="34" ht="49.5" customHeight="1" s="82">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-IDNT-02</t>
+        </is>
+      </c>
+      <c r="C34" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/02-Test_User_Registration_Process", "Test User Registration Process")</f>
+        <v/>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>- Verify that the identity requirements for user registration are aligned with business and security requirements.
+- Validate the registration process.</t>
+        </is>
+      </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2204,21 +2205,20 @@
       </c>
       <c r="F34" s="18" t="n"/>
     </row>
-    <row r="35" ht="49.5" customHeight="1" s="82">
+    <row r="35" ht="33" customHeight="1" s="82">
       <c r="A35" s="19" t="n"/>
       <c r="B35" s="34" t="inlineStr">
         <is>
-          <t>WSTG-IDNT-02</t>
+          <t>WSTG-IDNT-03</t>
         </is>
       </c>
       <c r="C35" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/02-Test_User_Registration_Process", "Test User Registration Process")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/03-Test_Account_Provisioning_Process", "Test Account Provisioning Process")</f>
         <v/>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>- Verify that the identity requirements for user registration are aligned with business and security requirements.
-- Validate the registration process.</t>
+          <t>- Verify which accounts may provision other accounts and of what type.</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
@@ -2228,20 +2228,21 @@
       </c>
       <c r="F35" s="18" t="n"/>
     </row>
-    <row r="36" ht="33" customHeight="1" s="82">
+    <row r="36" ht="49.5" customHeight="1" s="82">
       <c r="A36" s="19" t="n"/>
       <c r="B36" s="34" t="inlineStr">
         <is>
-          <t>WSTG-IDNT-03</t>
+          <t>WSTG-IDNT-04</t>
         </is>
       </c>
       <c r="C36" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/03-Test_Account_Provisioning_Process", "Test Account Provisioning Process")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/04-Testing_for_Account_Enumeration_and_Guessable_User_Account", "Testing for Account Enumeration and Guessable User Account")</f>
         <v/>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>- Verify which accounts may provision other accounts and of what type.</t>
+          <t>- Review processes that pertain to user identification (*e.g.* registration, login, etc.).
+- Enumerate users where possible through response analysis.</t>
         </is>
       </c>
       <c r="E36" s="18" t="inlineStr">
@@ -2251,21 +2252,20 @@
       </c>
       <c r="F36" s="18" t="n"/>
     </row>
-    <row r="37" ht="49.5" customHeight="1" s="82">
+    <row r="37" ht="33" customHeight="1" s="82">
       <c r="A37" s="19" t="n"/>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>WSTG-IDNT-04</t>
+          <t>WSTG-IDNT-05</t>
         </is>
       </c>
       <c r="C37" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/04-Testing_for_Account_Enumeration_and_Guessable_User_Account", "Testing for Account Enumeration and Guessable User Account")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/05-Testing_for_Weak_or_Unenforced_Username_Policy", "Testing for Weak or Unenforced Username Policy")</f>
         <v/>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>- Review processes that pertain to user identification (*e.g.* registration, login, etc.).
-- Enumerate users where possible through response analysis.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E37" s="18" t="inlineStr">
@@ -2275,79 +2275,80 @@
       </c>
       <c r="F37" s="18" t="n"/>
     </row>
-    <row r="38" ht="33" customHeight="1" s="82">
-      <c r="A38" s="19" t="n"/>
-      <c r="B38" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-IDNT-05</t>
-        </is>
-      </c>
-      <c r="C38" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/05-Testing_for_Weak_or_Unenforced_Username_Policy", "Testing for Weak or Unenforced Username Policy")</f>
-        <v/>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+    <row r="38" ht="15" customHeight="1" s="82">
+      <c r="A38" s="97" t="n"/>
+      <c r="B38" s="98" t="n"/>
+      <c r="C38" s="99" t="n"/>
+      <c r="D38" s="99" t="n"/>
+      <c r="E38" s="99" t="n"/>
+      <c r="F38" s="99" t="n"/>
+    </row>
+    <row r="39" ht="47.25" customHeight="1" s="82">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="100" t="inlineStr">
+        <is>
+          <t>Authentication Testing</t>
+        </is>
+      </c>
+      <c r="C39" s="101" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="D39" s="101" t="inlineStr">
+        <is>
+          <t>Objectives</t>
+        </is>
+      </c>
+      <c r="E39" s="101" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F39" s="101" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="33" customHeight="1" s="82">
+      <c r="A40" s="19" t="n"/>
+      <c r="B40" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-ATHN-01</t>
+        </is>
+      </c>
+      <c r="C40" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/01-Testing_for_Credentials_Transported_over_an_Encrypted_Channel", "Testing for Credentials Transported over an Encrypted Channel")</f>
+        <v/>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F38" s="18" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="82">
-      <c r="A39" s="97" t="n"/>
-      <c r="B39" s="98" t="n"/>
-      <c r="C39" s="99" t="n"/>
-      <c r="D39" s="99" t="n"/>
-      <c r="E39" s="99" t="n"/>
-      <c r="F39" s="99" t="n"/>
-    </row>
-    <row r="40" ht="47.25" customHeight="1" s="82">
-      <c r="A40" s="9" t="n"/>
-      <c r="B40" s="100" t="inlineStr">
-        <is>
-          <t>Authentication Testing</t>
-        </is>
-      </c>
-      <c r="C40" s="101" t="inlineStr">
-        <is>
-          <t>Test Name</t>
-        </is>
-      </c>
-      <c r="D40" s="101" t="inlineStr">
-        <is>
-          <t>Objectives</t>
-        </is>
-      </c>
-      <c r="E40" s="101" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F40" s="101" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="33" customHeight="1" s="82">
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F40" s="18" t="n"/>
+    </row>
+    <row r="41" ht="66" customHeight="1" s="82">
       <c r="A41" s="19" t="n"/>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-01</t>
+          <t>WSTG-ATHN-02</t>
         </is>
       </c>
       <c r="C41" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/01-Testing_for_Credentials_Transported_over_an_Encrypted_Channel", "Testing for Credentials Transported over an Encrypted Channel")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/02-Testing_for_Default_Credentials", "Testing for Default Credentials")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- Determine whether the application has any user accounts with default passwords.
+- Review whether new user accounts are created with weak or predictable passwords.</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">
@@ -2361,17 +2362,17 @@
       <c r="A42" s="19" t="n"/>
       <c r="B42" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-02</t>
+          <t>WSTG-ATHN-03</t>
         </is>
       </c>
       <c r="C42" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/02-Testing_for_Default_Credentials", "Testing for Default Credentials")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/03-Testing_for_Weak_Lock_Out_Mechanism", "Testing for Weak Lock Out Mechanism")</f>
         <v/>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the application has any user accounts with default passwords.
-- Review whether new user accounts are created with weak or predictable passwords.</t>
+          <t>- Evaluate the account lockout mechanism's ability to mitigate brute force password guessing.
+- Evaluate the unlock mechanism's resistance to unauthorized account unlocking.</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
@@ -2381,21 +2382,20 @@
       </c>
       <c r="F42" s="18" t="n"/>
     </row>
-    <row r="43" ht="66" customHeight="1" s="82">
+    <row r="43" ht="33" customHeight="1" s="82">
       <c r="A43" s="19" t="n"/>
       <c r="B43" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-03</t>
+          <t>WSTG-ATHN-04</t>
         </is>
       </c>
       <c r="C43" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/03-Testing_for_Weak_Lock_Out_Mechanism", "Testing for Weak Lock Out Mechanism")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/04-Testing_for_Bypassing_Authentication_Schema", "Testing for Bypassing Authentication Schema")</f>
         <v/>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>- Evaluate the account lockout mechanism's ability to mitigate brute force password guessing.
-- Evaluate the unlock mechanism's resistance to unauthorized account unlocking.</t>
+          <t>- Ensure that authentication is applied across all services that require it.</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
@@ -2409,16 +2409,16 @@
       <c r="A44" s="19" t="n"/>
       <c r="B44" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-04</t>
+          <t>WSTG-ATHN-05</t>
         </is>
       </c>
       <c r="C44" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/04-Testing_for_Bypassing_Authentication_Schema", "Testing for Bypassing Authentication Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/05-Testing_for_Vulnerable_Remember_Password", "Testing for Vulnerable Remember Password")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>- Ensure that authentication is applied across all services that require it.</t>
+          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
         </is>
       </c>
       <c r="E44" s="18" t="inlineStr">
@@ -2428,20 +2428,21 @@
       </c>
       <c r="F44" s="18" t="n"/>
     </row>
-    <row r="45" ht="33" customHeight="1" s="82">
+    <row r="45" ht="49.5" customHeight="1" s="82">
       <c r="A45" s="19" t="n"/>
       <c r="B45" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-05</t>
+          <t>WSTG-ATHN-06</t>
         </is>
       </c>
       <c r="C45" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/05-Testing_for_Vulnerable_Remember_Password", "Testing for Vulnerable Remember Password")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/06-Testing_for_Browser_Cache_Weaknesses", "Testing for Browser Cache Weaknesses")</f>
         <v/>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
+          <t>- Review if the application stores sensitive information on the client-side.
+- Review if access can occur without authorization.</t>
         </is>
       </c>
       <c r="E45" s="18" t="inlineStr">
@@ -2451,21 +2452,20 @@
       </c>
       <c r="F45" s="18" t="n"/>
     </row>
-    <row r="46" ht="49.5" customHeight="1" s="82">
+    <row r="46" ht="66" customHeight="1" s="82">
       <c r="A46" s="19" t="n"/>
       <c r="B46" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-06</t>
+          <t>WSTG-ATHN-07</t>
         </is>
       </c>
       <c r="C46" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/06-Testing_for_Browser_Cache_Weaknesses", "Testing for Browser Cache Weaknesses")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/07-Testing_for_Weak_Authentication_Methods", "Testing for Weak Authentication Methods")</f>
         <v/>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>- Review if the application stores sensitive information on the client-side.
-- Review if access can occur without authorization.</t>
+          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
         </is>
       </c>
       <c r="E46" s="18" t="inlineStr">
@@ -2475,20 +2475,21 @@
       </c>
       <c r="F46" s="18" t="n"/>
     </row>
-    <row r="47" ht="66" customHeight="1" s="82">
+    <row r="47" ht="49.5" customHeight="1" s="82">
       <c r="A47" s="19" t="n"/>
       <c r="B47" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-07</t>
+          <t>WSTG-ATHN-08</t>
         </is>
       </c>
       <c r="C47" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/07-Testing_for_Weak_Authentication_Methods", "Testing for Weak Authentication Methods")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/08-Testing_for_Weak_Security_Question_Answer", "Testing for Weak Security Question Answer")</f>
         <v/>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
+          <t>- Determine the complexity and how straight-forward the questions are.
+- Assess possible user answers and brute force capabilities.</t>
         </is>
       </c>
       <c r="E47" s="18" t="inlineStr">
@@ -2498,21 +2499,20 @@
       </c>
       <c r="F47" s="18" t="n"/>
     </row>
-    <row r="48" ht="49.5" customHeight="1" s="82">
+    <row r="48" ht="33" customHeight="1" s="82">
       <c r="A48" s="19" t="n"/>
       <c r="B48" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-08</t>
+          <t>WSTG-ATHN-09</t>
         </is>
       </c>
       <c r="C48" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/08-Testing_for_Weak_Security_Question_Answer", "Testing for Weak Security Question Answer")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/09-Testing_for_Weak_Password_Change_or_Reset_Functionalities", "Testing for Weak Password Change or Reset Functionalities")</f>
         <v/>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>- Determine the complexity and how straight-forward the questions are.
-- Assess possible user answers and brute force capabilities.</t>
+          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
         </is>
       </c>
       <c r="E48" s="18" t="inlineStr">
@@ -2522,20 +2522,21 @@
       </c>
       <c r="F48" s="18" t="n"/>
     </row>
-    <row r="49" ht="33" customHeight="1" s="82">
+    <row r="49" ht="49.5" customHeight="1" s="82">
       <c r="A49" s="19" t="n"/>
       <c r="B49" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-09</t>
+          <t>WSTG-ATHN-10</t>
         </is>
       </c>
       <c r="C49" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/09-Testing_for_Weak_Password_Change_or_Reset_Functionalities", "Testing for Weak Password Change or Reset Functionalities")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/10-Testing_for_Weaker_Authentication_in_Alternative_Channel", "Testing for Weaker Authentication in Alternative Channel")</f>
         <v/>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
+          <t>- Identify alternative authentication channels.
+- Assess the security measures used and if any bypasses exists on the alternative channels.</t>
         </is>
       </c>
       <c r="E49" s="18" t="inlineStr">
@@ -2545,106 +2546,105 @@
       </c>
       <c r="F49" s="18" t="n"/>
     </row>
-    <row r="50" ht="49.5" customHeight="1" s="82">
+    <row r="50" ht="66" customHeight="1" s="82">
       <c r="A50" s="19" t="n"/>
       <c r="B50" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-10</t>
+          <t>WSTG-ATHN-11</t>
         </is>
       </c>
       <c r="C50" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/10-Testing_for_Weaker_Authentication_in_Alternative_Channel", "Testing for Weaker Authentication in Alternative Channel")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/11-Testing_Multi-Factor_Authentication", "Testing Multi-Factor Authentication (MFA)")</f>
         <v/>
       </c>
       <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>- Identify alternative authentication channels.
-- Assess the security measures used and if any bypasses exists on the alternative channels.</t>
-        </is>
-      </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="n"/>
-    </row>
-    <row r="51" ht="66" customHeight="1" s="82">
-      <c r="A51" s="19" t="n"/>
-      <c r="B51" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-11</t>
-        </is>
-      </c>
-      <c r="C51" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/11-Testing_Multi-Factor_Authentication", "Testing Multi-Factor Authentication (MFA)")</f>
-        <v/>
-      </c>
-      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>- Identify the type of MFA used by the application.
 - Determine whether the MFA implementation is robust and secure.
 - Attempt to bypass the MFA.</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="82">
-      <c r="A52" s="97" t="n"/>
-      <c r="B52" s="98" t="n"/>
-      <c r="C52" s="99" t="n"/>
-      <c r="D52" s="99" t="n"/>
-      <c r="E52" s="99" t="n"/>
-      <c r="F52" s="99" t="n"/>
-    </row>
-    <row r="53" ht="47.25" customHeight="1" s="82">
-      <c r="A53" s="9" t="n"/>
-      <c r="B53" s="100" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="n"/>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="82">
+      <c r="A51" s="97" t="n"/>
+      <c r="B51" s="98" t="n"/>
+      <c r="C51" s="99" t="n"/>
+      <c r="D51" s="99" t="n"/>
+      <c r="E51" s="99" t="n"/>
+      <c r="F51" s="99" t="n"/>
+    </row>
+    <row r="52" ht="47.25" customHeight="1" s="82">
+      <c r="A52" s="9" t="n"/>
+      <c r="B52" s="100" t="inlineStr">
         <is>
           <t>Authorization Testing</t>
         </is>
       </c>
-      <c r="C53" s="101" t="inlineStr">
+      <c r="C52" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D53" s="101" t="inlineStr">
+      <c r="D52" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E53" s="101" t="inlineStr">
+      <c r="E52" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F53" s="101" t="inlineStr">
+      <c r="F52" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="49.5" customHeight="1" s="82">
+    <row r="53" ht="49.5" customHeight="1" s="82">
+      <c r="A53" s="19" t="n"/>
+      <c r="B53" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-ATHZ-01</t>
+        </is>
+      </c>
+      <c r="C53" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/01-Testing_Directory_Traversal_File_Include", "Testing Directory Traversal File Include")</f>
+        <v/>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>- Identify injection points that pertain to path traversal.
+- Assess bypassing techniques and identify the extent of path traversal.</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="n"/>
+    </row>
+    <row r="54" ht="33" customHeight="1" s="82">
       <c r="A54" s="19" t="n"/>
       <c r="B54" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-01</t>
+          <t>WSTG-ATHZ-02</t>
         </is>
       </c>
       <c r="C54" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/01-Testing_Directory_Traversal_File_Include", "Testing Directory Traversal File Include")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/02-Testing_for_Bypassing_Authorization_Schema", "Testing for Bypassing Authorization Schema")</f>
         <v/>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that pertain to path traversal.
-- Assess bypassing techniques and identify the extent of path traversal.</t>
+          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
         </is>
       </c>
       <c r="E54" s="18" t="inlineStr">
@@ -2654,20 +2654,21 @@
       </c>
       <c r="F54" s="18" t="n"/>
     </row>
-    <row r="55" ht="33" customHeight="1" s="82">
+    <row r="55" ht="49.5" customHeight="1" s="82">
       <c r="A55" s="19" t="n"/>
       <c r="B55" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-02</t>
+          <t>WSTG-ATHZ-03</t>
         </is>
       </c>
       <c r="C55" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/02-Testing_for_Bypassing_Authorization_Schema", "Testing for Bypassing Authorization Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/03-Testing_for_Privilege_Escalation", "Testing for Privilege Escalation")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
+          <t>- Identify injection points related to privilege manipulation.
+- Fuzz or otherwise attempt to bypass security measures.</t>
         </is>
       </c>
       <c r="E55" s="18" t="inlineStr">
@@ -2681,17 +2682,17 @@
       <c r="A56" s="19" t="n"/>
       <c r="B56" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-03</t>
+          <t>WSTG-ATHZ-04</t>
         </is>
       </c>
       <c r="C56" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/03-Testing_for_Privilege_Escalation", "Testing for Privilege Escalation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/04-Testing_for_Insecure_Direct_Object_References", "Testing for Insecure Direct Object References")</f>
         <v/>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points related to privilege manipulation.
-- Fuzz or otherwise attempt to bypass security measures.</t>
+          <t>- Identify points where object references may occur.
+- Assess the access control measures and if they're vulnerable to IDOR.</t>
         </is>
       </c>
       <c r="E56" s="18" t="inlineStr">
@@ -2701,21 +2702,20 @@
       </c>
       <c r="F56" s="18" t="n"/>
     </row>
-    <row r="57" ht="49.5" customHeight="1" s="82">
+    <row r="57" ht="33" customHeight="1" s="82">
       <c r="A57" s="19" t="n"/>
       <c r="B57" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-04</t>
+          <t>WSTG-ATHZ-05</t>
         </is>
       </c>
       <c r="C57" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/04-Testing_for_Insecure_Direct_Object_References", "Testing for Insecure Direct Object References")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/05-Testing_for_OAuth_Weaknesses", "Testing for OAuth Weaknesses")</f>
         <v/>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>- Identify points where object references may occur.
-- Assess the access control measures and if they're vulnerable to IDOR.</t>
+          <t>- Determine if OAuth2 implementation is vulnerable or using a deprecated or custom implementation.</t>
         </is>
       </c>
       <c r="E57" s="18" t="inlineStr">
@@ -2725,83 +2725,83 @@
       </c>
       <c r="F57" s="18" t="n"/>
     </row>
-    <row r="58" ht="33" customHeight="1" s="82">
-      <c r="A58" s="19" t="n"/>
-      <c r="B58" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHZ-05</t>
-        </is>
-      </c>
-      <c r="C58" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/05-Testing_for_OAuth_Weaknesses", "Testing for OAuth Weaknesses")</f>
-        <v/>
-      </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>- Determine if OAuth2 implementation is vulnerable or using a deprecated or custom implementation.</t>
-        </is>
-      </c>
-      <c r="E58" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F58" s="18" t="n"/>
-    </row>
-    <row r="59" ht="15" customHeight="1" s="82">
-      <c r="A59" s="97" t="n"/>
-      <c r="B59" s="98" t="n"/>
-      <c r="C59" s="99" t="n"/>
-      <c r="D59" s="99" t="n"/>
-      <c r="E59" s="99" t="n"/>
-      <c r="F59" s="99" t="n"/>
-    </row>
-    <row r="60" ht="47.25" customHeight="1" s="82">
-      <c r="A60" s="9" t="n"/>
-      <c r="B60" s="100" t="inlineStr">
+    <row r="58" ht="15" customHeight="1" s="82">
+      <c r="A58" s="97" t="n"/>
+      <c r="B58" s="98" t="n"/>
+      <c r="C58" s="99" t="n"/>
+      <c r="D58" s="99" t="n"/>
+      <c r="E58" s="99" t="n"/>
+      <c r="F58" s="99" t="n"/>
+    </row>
+    <row r="59" ht="47.25" customHeight="1" s="82">
+      <c r="A59" s="9" t="n"/>
+      <c r="B59" s="100" t="inlineStr">
         <is>
           <t>Session Management Testing</t>
         </is>
       </c>
-      <c r="C60" s="101" t="inlineStr">
+      <c r="C59" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D60" s="101" t="inlineStr">
+      <c r="D59" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E60" s="101" t="inlineStr">
+      <c r="E59" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F60" s="101" t="inlineStr">
+      <c r="F59" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="99" customHeight="1" s="82">
-      <c r="A61" s="19" t="n"/>
-      <c r="B61" s="34" t="inlineStr">
+    <row r="60" ht="99" customHeight="1" s="82">
+      <c r="A60" s="19" t="n"/>
+      <c r="B60" s="34" t="inlineStr">
         <is>
           <t>WSTG-SESS-01</t>
         </is>
       </c>
-      <c r="C61" s="15">
+      <c r="C60" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/01-Testing_for_Session_Management_Schema", "Testing for Session Management Schema")</f>
         <v/>
       </c>
-      <c r="D61" s="16" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
         <is>
           <t>- Gather session tokens, for the same user and for different users where possible.
 - Analyze and ensure that enough randomness exists to stop session forging attacks.
 - Modify cookies that are not signed and contain information that can be manipulated.</t>
         </is>
       </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="n"/>
+    </row>
+    <row r="61" ht="33" customHeight="1" s="82">
+      <c r="A61" s="19" t="n"/>
+      <c r="B61" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-SESS-02</t>
+        </is>
+      </c>
+      <c r="C61" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/02-Testing_for_Cookies_Attributes", "Testing for Cookies Attributes")</f>
+        <v/>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>- Ensure that the proper security configuration is set for cookies.</t>
+        </is>
+      </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2813,16 +2813,17 @@
       <c r="A62" s="19" t="n"/>
       <c r="B62" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-02</t>
+          <t>WSTG-SESS-03</t>
         </is>
       </c>
       <c r="C62" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/02-Testing_for_Cookies_Attributes", "Testing for Cookies Attributes")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/03-Testing_for_Session_Fixation", "Testing for Session Fixation")</f>
         <v/>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>- Ensure that the proper security configuration is set for cookies.</t>
+          <t>- Analyze the authentication mechanism and its flow.
+- Force cookies and assess the impact.</t>
         </is>
       </c>
       <c r="E62" s="18" t="inlineStr">
@@ -2832,48 +2833,47 @@
       </c>
       <c r="F62" s="18" t="n"/>
     </row>
-    <row r="63" ht="33" customHeight="1" s="82">
+    <row r="63" ht="49.5" customHeight="1" s="82">
       <c r="A63" s="19" t="n"/>
       <c r="B63" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-03</t>
+          <t>WSTG-SESS-04</t>
         </is>
       </c>
       <c r="C63" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/03-Testing_for_Session_Fixation", "Testing for Session Fixation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/04-Testing_for_Exposed_Session_Variables", "Testing for Exposed Session Variables")</f>
         <v/>
       </c>
       <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>- Analyze the authentication mechanism and its flow.
-- Force cookies and assess the impact.</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F63" s="18" t="n"/>
-    </row>
-    <row r="64" ht="49.5" customHeight="1" s="82">
-      <c r="A64" s="19" t="n"/>
-      <c r="B64" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-04</t>
-        </is>
-      </c>
-      <c r="C64" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/04-Testing_for_Exposed_Session_Variables", "Testing for Exposed Session Variables")</f>
-        <v/>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>- Ensure that proper encryption is implemented.
 - Review the caching configuration.
 - Assess the channel and methods' security.</t>
         </is>
       </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="n"/>
+    </row>
+    <row r="64" ht="33" customHeight="1" s="82">
+      <c r="A64" s="19" t="n"/>
+      <c r="B64" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-SESS-05</t>
+        </is>
+      </c>
+      <c r="C64" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/05-Testing_for_Cross_Site_Request_Forgery", "Testing for Cross Site Request Forgery")</f>
+        <v/>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
+        </is>
+      </c>
       <c r="E64" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2881,20 +2881,21 @@
       </c>
       <c r="F64" s="18" t="n"/>
     </row>
-    <row r="65" ht="33" customHeight="1" s="82">
+    <row r="65" ht="49.5" customHeight="1" s="82">
       <c r="A65" s="19" t="n"/>
       <c r="B65" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-05</t>
+          <t>WSTG-SESS-06</t>
         </is>
       </c>
       <c r="C65" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/05-Testing_for_Cross_Site_Request_Forgery", "Testing for Cross Site Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/06-Testing_for_Logout_Functionality", "Testing for Logout Functionality")</f>
         <v/>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
+          <t>- Assess the logout UI.
+- Analyze the session timeout and if the session is properly killed after logout.</t>
         </is>
       </c>
       <c r="E65" s="18" t="inlineStr">
@@ -2904,21 +2905,20 @@
       </c>
       <c r="F65" s="18" t="n"/>
     </row>
-    <row r="66" ht="49.5" customHeight="1" s="82">
+    <row r="66" ht="16.5" customHeight="1" s="82">
       <c r="A66" s="19" t="n"/>
       <c r="B66" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-06</t>
+          <t>WSTG-SESS-07</t>
         </is>
       </c>
       <c r="C66" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/06-Testing_for_Logout_Functionality", "Testing for Logout Functionality")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/07-Testing_Session_Timeout", "Testing Session Timeout")</f>
         <v/>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>- Assess the logout UI.
-- Analyze the session timeout and if the session is properly killed after logout.</t>
+          <t>- Validate that a hard session timeout exists.</t>
         </is>
       </c>
       <c r="E66" s="18" t="inlineStr">
@@ -2928,20 +2928,21 @@
       </c>
       <c r="F66" s="18" t="n"/>
     </row>
-    <row r="67" ht="16.5" customHeight="1" s="82">
+    <row r="67" ht="33" customHeight="1" s="82">
       <c r="A67" s="19" t="n"/>
       <c r="B67" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-07</t>
+          <t>WSTG-SESS-08</t>
         </is>
       </c>
       <c r="C67" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/07-Testing_Session_Timeout", "Testing Session Timeout")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/08-Testing_for_Session_Puzzling", "Testing for Session Puzzling")</f>
         <v/>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>- Validate that a hard session timeout exists.</t>
+          <t>- Identify all session variables.
+- Break the logical flow of session generation.</t>
         </is>
       </c>
       <c r="E67" s="18" t="inlineStr">
@@ -2955,17 +2956,17 @@
       <c r="A68" s="19" t="n"/>
       <c r="B68" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-08</t>
+          <t>WSTG-SESS-09</t>
         </is>
       </c>
       <c r="C68" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/08-Testing_for_Session_Puzzling", "Testing for Session Puzzling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/09-Testing_for_Session_Hijacking", "Testing for Session Hijacking")</f>
         <v/>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>- Identify all session variables.
-- Break the logical flow of session generation.</t>
+          <t>- Identify vulnerable session cookies.
+- Hijack vulnerable cookies and assess the risk level.</t>
         </is>
       </c>
       <c r="E68" s="18" t="inlineStr">
@@ -2975,21 +2976,21 @@
       </c>
       <c r="F68" s="18" t="n"/>
     </row>
-    <row r="69" ht="33" customHeight="1" s="82">
+    <row r="69" ht="49.5" customHeight="1" s="82">
       <c r="A69" s="19" t="n"/>
       <c r="B69" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-09</t>
+          <t>WSTG-SESS-10</t>
         </is>
       </c>
       <c r="C69" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/09-Testing_for_Session_Hijacking", "Testing for Session Hijacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/10-Testing_JSON_Web_Tokens", "Testing JSON Web Tokens")</f>
         <v/>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>- Identify vulnerable session cookies.
-- Hijack vulnerable cookies and assess the risk level.</t>
+          <t>- Determine whether the JWTs expose sensitive information.
+- Determine whether the JWTs can be tampered with or modified.</t>
         </is>
       </c>
       <c r="E69" s="18" t="inlineStr">
@@ -3003,17 +3004,16 @@
       <c r="A70" s="19" t="n"/>
       <c r="B70" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-10</t>
+          <t>WSTG-SESS-11</t>
         </is>
       </c>
       <c r="C70" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/10-Testing_JSON_Web_Tokens", "Testing JSON Web Tokens")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/11-Testing_for_Concurrent_Sessions", "Testing for Concurrent Sessions")</f>
         <v/>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the JWTs expose sensitive information.
-- Determine whether the JWTs can be tampered with or modified.</t>
+          <t>- Evaluate the application's session management by assessing the handling of multiple active sessions for a single user account.</t>
         </is>
       </c>
       <c r="E70" s="18" t="inlineStr">
@@ -3023,79 +3023,80 @@
       </c>
       <c r="F70" s="18" t="n"/>
     </row>
-    <row r="71" ht="49.5" customHeight="1" s="82">
-      <c r="A71" s="19" t="n"/>
-      <c r="B71" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-11</t>
-        </is>
-      </c>
-      <c r="C71" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/11-Testing_for_Concurrent_Sessions", "Testing for Concurrent Sessions")</f>
-        <v/>
-      </c>
-      <c r="D71" s="16" t="inlineStr">
-        <is>
-          <t>- Evaluate the application's session management by assessing the handling of multiple active sessions for a single user account.</t>
-        </is>
-      </c>
-      <c r="E71" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F71" s="18" t="n"/>
-    </row>
-    <row r="72" ht="15" customHeight="1" s="82">
-      <c r="A72" s="97" t="n"/>
-      <c r="B72" s="98" t="n"/>
-      <c r="C72" s="99" t="n"/>
-      <c r="D72" s="99" t="n"/>
-      <c r="E72" s="99" t="n"/>
-      <c r="F72" s="99" t="n"/>
-    </row>
-    <row r="73" ht="47.25" customHeight="1" s="82">
-      <c r="A73" s="9" t="n"/>
-      <c r="B73" s="100" t="inlineStr">
+    <row r="71" ht="15" customHeight="1" s="82">
+      <c r="A71" s="97" t="n"/>
+      <c r="B71" s="98" t="n"/>
+      <c r="C71" s="99" t="n"/>
+      <c r="D71" s="99" t="n"/>
+      <c r="E71" s="99" t="n"/>
+      <c r="F71" s="99" t="n"/>
+    </row>
+    <row r="72" ht="47.25" customHeight="1" s="82">
+      <c r="A72" s="9" t="n"/>
+      <c r="B72" s="100" t="inlineStr">
         <is>
           <t>Input Validation Testing</t>
         </is>
       </c>
-      <c r="C73" s="101" t="inlineStr">
+      <c r="C72" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D73" s="101" t="inlineStr">
+      <c r="D72" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E73" s="101" t="inlineStr">
+      <c r="E72" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F73" s="101" t="inlineStr">
+      <c r="F72" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="49.5" customHeight="1" s="82">
+    <row r="73" ht="49.5" customHeight="1" s="82">
+      <c r="A73" s="19" t="n"/>
+      <c r="B73" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-01</t>
+        </is>
+      </c>
+      <c r="C73" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <v/>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>- Identify variables that are reflected in responses.
+- Assess the input they accept and the encoding that gets applied on return (if any).</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="n"/>
+    </row>
+    <row r="74" ht="66" customHeight="1" s="82">
       <c r="A74" s="19" t="n"/>
       <c r="B74" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-01</t>
+          <t>WSTG-INPV-02</t>
         </is>
       </c>
       <c r="C74" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>- Identify variables that are reflected in responses.
+          <t>- Identify stored input that is reflected on the client-side.
 - Assess the input they accept and the encoding that gets applied on return (if any).</t>
         </is>
       </c>
@@ -3106,21 +3107,20 @@
       </c>
       <c r="F74" s="18" t="n"/>
     </row>
-    <row r="75" ht="66" customHeight="1" s="82">
+    <row r="75" ht="16.5" customHeight="1" s="82">
       <c r="A75" s="19" t="n"/>
       <c r="B75" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-02</t>
+          <t>WSTG-INPV-03</t>
         </is>
       </c>
       <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>- Identify stored input that is reflected on the client-side.
-- Assess the input they accept and the encoding that gets applied on return (if any).</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E75" s="18" t="inlineStr">
@@ -3130,20 +3130,21 @@
       </c>
       <c r="F75" s="18" t="n"/>
     </row>
-    <row r="76" ht="16.5" customHeight="1" s="82">
+    <row r="76" ht="49.5" customHeight="1" s="82">
       <c r="A76" s="19" t="n"/>
       <c r="B76" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-03</t>
+          <t>WSTG-INPV-04</t>
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- Identify the backend and the parsing method used.
+- Assess injection points and try bypassing input filters using HPP.</t>
         </is>
       </c>
       <c r="E76" s="18" t="inlineStr">
@@ -3157,17 +3158,17 @@
       <c r="A77" s="19" t="n"/>
       <c r="B77" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-04</t>
+          <t>WSTG-INPV-05</t>
         </is>
       </c>
       <c r="C77" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
         <v/>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>- Identify the backend and the parsing method used.
-- Assess injection points and try bypassing input filters using HPP.</t>
+          <t>- Identify SQL injection points.
+- Assess the severity of the injection and the level of access that can be achieved through it.</t>
         </is>
       </c>
       <c r="E77" s="18" t="inlineStr">
@@ -3177,21 +3178,21 @@
       </c>
       <c r="F77" s="18" t="n"/>
     </row>
-    <row r="78" ht="49.5" customHeight="1" s="82">
+    <row r="78" ht="33" customHeight="1" s="82">
       <c r="A78" s="19" t="n"/>
       <c r="B78" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-05</t>
+          <t>WSTG-INPV-06</t>
         </is>
       </c>
       <c r="C78" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
         <v/>
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>- Identify SQL injection points.
-- Assess the severity of the injection and the level of access that can be achieved through it.</t>
+          <t>- Identify LDAP injection points.
+- Assess the severity of the injection.</t>
         </is>
       </c>
       <c r="E78" s="18" t="inlineStr">
@@ -3201,21 +3202,21 @@
       </c>
       <c r="F78" s="18" t="n"/>
     </row>
-    <row r="79" ht="33" customHeight="1" s="82">
+    <row r="79" ht="49.5" customHeight="1" s="82">
       <c r="A79" s="19" t="n"/>
       <c r="B79" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-06</t>
+          <t>WSTG-INPV-07</t>
         </is>
       </c>
       <c r="C79" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
         <v/>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>- Identify LDAP injection points.
-- Assess the severity of the injection.</t>
+          <t>- Identify XML injection points.
+- Assess the types of exploits that can be attained and their severities.</t>
         </is>
       </c>
       <c r="E79" s="18" t="inlineStr">
@@ -3225,21 +3226,21 @@
       </c>
       <c r="F79" s="18" t="n"/>
     </row>
-    <row r="80" ht="49.5" customHeight="1" s="82">
+    <row r="80" ht="33" customHeight="1" s="82">
       <c r="A80" s="19" t="n"/>
       <c r="B80" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-07</t>
+          <t>WSTG-INPV-08</t>
         </is>
       </c>
       <c r="C80" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
         <v/>
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>- Identify XML injection points.
-- Assess the types of exploits that can be attained and their severities.</t>
+          <t>- Identify SSI injection points.
+- Assess the severity of the injection.</t>
         </is>
       </c>
       <c r="E80" s="18" t="inlineStr">
@@ -3249,21 +3250,20 @@
       </c>
       <c r="F80" s="18" t="n"/>
     </row>
-    <row r="81" ht="33" customHeight="1" s="82">
+    <row r="81" ht="16.5" customHeight="1" s="82">
       <c r="A81" s="19" t="n"/>
       <c r="B81" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-08</t>
+          <t>WSTG-INPV-09</t>
         </is>
       </c>
       <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
         <v/>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>- Identify SSI injection points.
-- Assess the severity of the injection.</t>
+          <t>- Identify XPATH injection points.</t>
         </is>
       </c>
       <c r="E81" s="18" t="inlineStr">
@@ -3273,47 +3273,48 @@
       </c>
       <c r="F81" s="18" t="n"/>
     </row>
-    <row r="82" ht="16.5" customHeight="1" s="82">
+    <row r="82" ht="66" customHeight="1" s="82">
       <c r="A82" s="19" t="n"/>
       <c r="B82" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-09</t>
+          <t>WSTG-INPV-10</t>
         </is>
       </c>
       <c r="C82" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
         <v/>
       </c>
       <c r="D82" s="16" t="inlineStr">
-        <is>
-          <t>- Identify XPATH injection points.</t>
-        </is>
-      </c>
-      <c r="E82" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F82" s="18" t="n"/>
-    </row>
-    <row r="83" ht="66" customHeight="1" s="82">
-      <c r="A83" s="19" t="n"/>
-      <c r="B83" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-10</t>
-        </is>
-      </c>
-      <c r="C83" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
-        <v/>
-      </c>
-      <c r="D83" s="16" t="inlineStr">
         <is>
           <t>- Identify IMAP/SMTP injection points.
 - Understand the data flow and deployment structure of the system.
 - Assess the injection impacts.</t>
         </is>
       </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="n"/>
+    </row>
+    <row r="83" ht="49.5" customHeight="1" s="82">
+      <c r="A83" s="19" t="n"/>
+      <c r="B83" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-11</t>
+        </is>
+      </c>
+      <c r="C83" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <v/>
+      </c>
+      <c r="D83" s="16" t="inlineStr">
+        <is>
+          <t>- Identify injection points where you can inject code into the application.
+- Assess the injection severity.</t>
+        </is>
+      </c>
       <c r="E83" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3321,21 +3322,21 @@
       </c>
       <c r="F83" s="18" t="n"/>
     </row>
-    <row r="84" ht="49.5" customHeight="1" s="82">
+    <row r="84" ht="33" customHeight="1" s="82">
       <c r="A84" s="19" t="n"/>
       <c r="B84" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-11</t>
+          <t>WSTG-INPV-12</t>
         </is>
       </c>
       <c r="C84" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
         <v/>
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points where you can inject code into the application.
-- Assess the injection severity.</t>
+          <t>- Identify and assess command injection points.
+- Bypass special characters and OS commands filter.</t>
         </is>
       </c>
       <c r="E84" s="18" t="inlineStr">
@@ -3345,21 +3346,20 @@
       </c>
       <c r="F84" s="18" t="n"/>
     </row>
-    <row r="85" ht="33" customHeight="1" s="82">
+    <row r="85" ht="49.5" customHeight="1" s="82">
       <c r="A85" s="19" t="n"/>
       <c r="B85" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-12</t>
+          <t>WSTG-INPV-13</t>
         </is>
       </c>
       <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
         <v/>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>- Identify and assess command injection points.
-- Bypass special characters and OS commands filter.</t>
+          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
         </is>
       </c>
       <c r="E85" s="18" t="inlineStr">
@@ -3369,114 +3369,68 @@
       </c>
       <c r="F85" s="18" t="n"/>
     </row>
-    <row r="86" ht="16.5" customHeight="1" s="82">
+    <row r="86" ht="66" customHeight="1" s="82">
       <c r="A86" s="19" t="n"/>
       <c r="B86" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-13</t>
+          <t>WSTG-INPV-14</t>
         </is>
       </c>
       <c r="C86" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Buffer_Overflow", "Testing for Buffer Overflow")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
         <v/>
       </c>
       <c r="D86" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E86" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F86" s="18" t="n"/>
-    </row>
-    <row r="87" ht="49.5" customHeight="1" s="82">
-      <c r="A87" s="19" t="n"/>
-      <c r="B87" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-13</t>
-        </is>
-      </c>
-      <c r="C87" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
-        <v/>
-      </c>
-      <c r="D87" s="16" t="inlineStr">
-        <is>
-          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
-        </is>
-      </c>
-      <c r="E87" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F87" s="18" t="n"/>
-    </row>
-    <row r="88" ht="66" customHeight="1" s="82">
-      <c r="A88" s="19" t="n"/>
-      <c r="B88" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-14</t>
-        </is>
-      </c>
-      <c r="C88" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
-        <v/>
-      </c>
-      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>- Identify injections that are stored and require a recall step to the stored injection.
 - Understand how a recall step could occur.
 - Set listeners or activate the recall step if possible.</t>
         </is>
       </c>
-      <c r="E88" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F88" s="18" t="n"/>
-    </row>
-    <row r="89" ht="115.5" customHeight="1" s="82">
-      <c r="A89" s="19" t="n"/>
-      <c r="B89" s="34" t="inlineStr">
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="n"/>
+    </row>
+    <row r="87" ht="115.5" customHeight="1" s="82">
+      <c r="A87" s="19" t="n"/>
+      <c r="B87" s="34" t="inlineStr">
         <is>
           <t>WSTG-INPV-15</t>
         </is>
       </c>
-      <c r="C89" s="15">
+      <c r="C87" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
         <v/>
       </c>
-      <c r="D89" s="16" t="inlineStr">
+      <c r="D87" s="16" t="inlineStr">
         <is>
           <t>- Identify user-controlled input that is reflected into HTTP response headers.
 - Assess whether CR (`\r`) and LF (`\n`) characters can be injected into response headers.
 - Determine the potential impact of successful HTTP Response Splitting attacks, such as cache poisoning or client-side exploitation.</t>
         </is>
       </c>
-      <c r="E89" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F89" s="18" t="n"/>
-    </row>
-    <row r="90" ht="99" customHeight="1" s="82">
-      <c r="A90" s="19" t="n"/>
-      <c r="B90" s="34" t="inlineStr">
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="n"/>
+    </row>
+    <row r="88" ht="99" customHeight="1" s="82">
+      <c r="A88" s="19" t="n"/>
+      <c r="B88" s="34" t="inlineStr">
         <is>
           <t>WSTG-INPV-16</t>
         </is>
       </c>
-      <c r="C90" s="15">
+      <c r="C88" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
         <v/>
       </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>- Identify request boundary inconsistencies between frontend and backend components
 - Detect classic CL/TE desynchronization vulnerabilities
@@ -3485,6 +3439,55 @@
 - Confirm backend request queue poisoning</t>
         </is>
       </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="n"/>
+    </row>
+    <row r="89" ht="49.5" customHeight="1" s="82">
+      <c r="A89" s="19" t="n"/>
+      <c r="B89" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-17</t>
+        </is>
+      </c>
+      <c r="C89" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <v/>
+      </c>
+      <c r="D89" s="16" t="inlineStr">
+        <is>
+          <t>- Assess if the Host header is being parsed dynamically in the application.
+- Bypass security controls that rely on the header.</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="n"/>
+    </row>
+    <row r="90" ht="49.5" customHeight="1" s="82">
+      <c r="A90" s="19" t="n"/>
+      <c r="B90" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-18</t>
+        </is>
+      </c>
+      <c r="C90" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <v/>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>- Detect template injection vulnerability points.
+- Identify the templating engine.
+- Build the exploit.</t>
+        </is>
+      </c>
       <c r="E90" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3496,17 +3499,18 @@
       <c r="A91" s="19" t="n"/>
       <c r="B91" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-17</t>
+          <t>WSTG-INPV-19</t>
         </is>
       </c>
       <c r="C91" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
         <v/>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>- Assess if the Host header is being parsed dynamically in the application.
-- Bypass security controls that rely on the header.</t>
+          <t>- Identify SSRF injection points.
+- Test if the injection points are exploitable.
+- Asses the severity of the vulnerability.</t>
         </is>
       </c>
       <c r="E91" s="18" t="inlineStr">
@@ -3520,18 +3524,17 @@
       <c r="A92" s="19" t="n"/>
       <c r="B92" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-18</t>
+          <t>WSTG-INPV-20</t>
         </is>
       </c>
       <c r="C92" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
         <v/>
       </c>
       <c r="D92" s="16" t="inlineStr">
         <is>
-          <t>- Detect template injection vulnerability points.
-- Identify the templating engine.
-- Build the exploit.</t>
+          <t>- Identify requests that modify objects
+- Assess if it is possible to modify fields never intended to be modified from outside</t>
         </is>
       </c>
       <c r="E92" s="18" t="inlineStr">
@@ -3541,67 +3544,18 @@
       </c>
       <c r="F92" s="18" t="n"/>
     </row>
-    <row r="93" ht="49.5" customHeight="1" s="82">
+    <row r="93" ht="181.5" customHeight="1" s="82">
       <c r="A93" s="19" t="n"/>
       <c r="B93" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-19</t>
+          <t>WSTG-INPV-21</t>
         </is>
       </c>
       <c r="C93" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
         <v/>
       </c>
       <c r="D93" s="16" t="inlineStr">
-        <is>
-          <t>- Identify SSRF injection points.
-- Test if the injection points are exploitable.
-- Asses the severity of the vulnerability.</t>
-        </is>
-      </c>
-      <c r="E93" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F93" s="18" t="n"/>
-    </row>
-    <row r="94" ht="49.5" customHeight="1" s="82">
-      <c r="A94" s="19" t="n"/>
-      <c r="B94" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-20</t>
-        </is>
-      </c>
-      <c r="C94" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
-        <v/>
-      </c>
-      <c r="D94" s="16" t="inlineStr">
-        <is>
-          <t>- Identify requests that modify objects
-- Assess if it is possible to modify fields never intended to be modified from outside</t>
-        </is>
-      </c>
-      <c r="E94" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F94" s="18" t="n"/>
-    </row>
-    <row r="95" ht="181.5" customHeight="1" s="82">
-      <c r="A95" s="19" t="n"/>
-      <c r="B95" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-21</t>
-        </is>
-      </c>
-      <c r="C95" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
-        <v/>
-      </c>
-      <c r="D95" s="16" t="inlineStr">
         <is>
           <t>- Identify CSV/spreadsheet export features that include untrusted input.
 - Verify whether attacker-controlled values are interpreted as formulas when the export is opened in common spreadsheet applications.
@@ -3610,150 +3564,198 @@
 - Assess practical impact based on who opens the export and how it is used.</t>
         </is>
       </c>
-      <c r="E95" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F95" s="18" t="n"/>
-    </row>
-    <row r="96" ht="15" customHeight="1" s="82">
-      <c r="A96" s="97" t="n"/>
-      <c r="B96" s="98" t="n"/>
-      <c r="C96" s="99" t="n"/>
-      <c r="D96" s="99" t="n"/>
-      <c r="E96" s="99" t="n"/>
-      <c r="F96" s="99" t="n"/>
-    </row>
-    <row r="97" ht="47.25" customHeight="1" s="82">
-      <c r="A97" s="9" t="n"/>
-      <c r="B97" s="100" t="inlineStr">
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="n"/>
+    </row>
+    <row r="94" ht="15" customHeight="1" s="82">
+      <c r="A94" s="97" t="n"/>
+      <c r="B94" s="98" t="n"/>
+      <c r="C94" s="99" t="n"/>
+      <c r="D94" s="99" t="n"/>
+      <c r="E94" s="99" t="n"/>
+      <c r="F94" s="99" t="n"/>
+    </row>
+    <row r="95" ht="47.25" customHeight="1" s="82">
+      <c r="A95" s="9" t="n"/>
+      <c r="B95" s="100" t="inlineStr">
         <is>
           <t>Testing for Error Handling</t>
         </is>
       </c>
-      <c r="C97" s="101" t="inlineStr">
+      <c r="C95" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D97" s="101" t="inlineStr">
+      <c r="D95" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E97" s="101" t="inlineStr">
+      <c r="E95" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F97" s="101" t="inlineStr">
+      <c r="F95" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="33" customHeight="1" s="82">
-      <c r="A98" s="19" t="n"/>
-      <c r="B98" s="34" t="inlineStr">
+    <row r="96" ht="33" customHeight="1" s="82">
+      <c r="A96" s="19" t="n"/>
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C98" s="15">
+      <c r="C96" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D96" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="n"/>
-    </row>
-    <row r="99" ht="16.5" customHeight="1" s="82">
-      <c r="A99" s="19" t="n"/>
-      <c r="B99" s="34" t="inlineStr">
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="n"/>
+    </row>
+    <row r="97" ht="16.5" customHeight="1" s="82">
+      <c r="A97" s="19" t="n"/>
+      <c r="B97" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C99" s="15">
+      <c r="C97" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
         <v/>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D97" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E99" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F99" s="18" t="n"/>
-    </row>
-    <row r="100" ht="15" customHeight="1" s="82">
-      <c r="A100" s="97" t="n"/>
-      <c r="B100" s="98" t="n"/>
-      <c r="C100" s="99" t="n"/>
-      <c r="D100" s="99" t="n"/>
-      <c r="E100" s="99" t="n"/>
-      <c r="F100" s="99" t="n"/>
-    </row>
-    <row r="101" ht="47.25" customHeight="1" s="82">
-      <c r="A101" s="9" t="n"/>
-      <c r="B101" s="100" t="inlineStr">
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="n"/>
+    </row>
+    <row r="98" ht="15" customHeight="1" s="82">
+      <c r="A98" s="97" t="n"/>
+      <c r="B98" s="98" t="n"/>
+      <c r="C98" s="99" t="n"/>
+      <c r="D98" s="99" t="n"/>
+      <c r="E98" s="99" t="n"/>
+      <c r="F98" s="99" t="n"/>
+    </row>
+    <row r="99" ht="47.25" customHeight="1" s="82">
+      <c r="A99" s="9" t="n"/>
+      <c r="B99" s="100" t="inlineStr">
         <is>
           <t>Testing for Weak Cryptography</t>
         </is>
       </c>
-      <c r="C101" s="101" t="inlineStr">
+      <c r="C99" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D101" s="101" t="inlineStr">
+      <c r="D99" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E101" s="101" t="inlineStr">
+      <c r="E99" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F101" s="101" t="inlineStr">
+      <c r="F99" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="82.5" customHeight="1" s="82">
-      <c r="A102" s="19" t="n"/>
-      <c r="B102" s="34" t="inlineStr">
+    <row r="100" ht="82.5" customHeight="1" s="82">
+      <c r="A100" s="19" t="n"/>
+      <c r="B100" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C102" s="15">
+      <c r="C100" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D100" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="n"/>
+    </row>
+    <row r="101" ht="49.5" customHeight="1" s="82">
+      <c r="A101" s="19" t="n"/>
+      <c r="B101" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C101" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F101" s="18" t="n"/>
+    </row>
+    <row r="102" ht="49.5" customHeight="1" s="82">
+      <c r="A102" s="19" t="n"/>
+      <c r="B102" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CRYP-03</t>
+        </is>
+      </c>
+      <c r="C102" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
+        <v/>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sensitive information transmitted through the various channels.
+- Assess the privacy and security of the channels used.</t>
+        </is>
+      </c>
       <c r="E102" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3761,21 +3763,20 @@
       </c>
       <c r="F102" s="18" t="n"/>
     </row>
-    <row r="103" ht="49.5" customHeight="1" s="82">
+    <row r="103" ht="33" customHeight="1" s="82">
       <c r="A103" s="19" t="n"/>
       <c r="B103" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CRYP-02</t>
+          <t>WSTG-CRYP-04</t>
         </is>
       </c>
       <c r="C103" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+          <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
       <c r="E103" s="18" t="inlineStr">
@@ -3785,150 +3786,103 @@
       </c>
       <c r="F103" s="18" t="n"/>
     </row>
-    <row r="104" ht="49.5" customHeight="1" s="82">
-      <c r="A104" s="19" t="n"/>
-      <c r="B104" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-03</t>
-        </is>
-      </c>
-      <c r="C104" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
-        <v/>
-      </c>
-      <c r="D104" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sensitive information transmitted through the various channels.
-- Assess the privacy and security of the channels used.</t>
-        </is>
-      </c>
-      <c r="E104" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F104" s="18" t="n"/>
-    </row>
-    <row r="105" ht="33" customHeight="1" s="82">
-      <c r="A105" s="19" t="n"/>
-      <c r="B105" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-04</t>
-        </is>
-      </c>
-      <c r="C105" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
-        <v/>
-      </c>
-      <c r="D105" s="16" t="inlineStr">
-        <is>
-          <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
-        </is>
-      </c>
-      <c r="E105" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F105" s="18" t="n"/>
-    </row>
-    <row r="106" ht="15" customHeight="1" s="82">
-      <c r="A106" s="97" t="n"/>
-      <c r="B106" s="98" t="n"/>
-      <c r="C106" s="99" t="n"/>
-      <c r="D106" s="99" t="n"/>
-      <c r="E106" s="99" t="n"/>
-      <c r="F106" s="99" t="n"/>
-    </row>
-    <row r="107" ht="47.25" customHeight="1" s="82">
-      <c r="A107" s="9" t="n"/>
-      <c r="B107" s="100" t="inlineStr">
+    <row r="104" ht="15" customHeight="1" s="82">
+      <c r="A104" s="97" t="n"/>
+      <c r="B104" s="98" t="n"/>
+      <c r="C104" s="99" t="n"/>
+      <c r="D104" s="99" t="n"/>
+      <c r="E104" s="99" t="n"/>
+      <c r="F104" s="99" t="n"/>
+    </row>
+    <row r="105" ht="47.25" customHeight="1" s="82">
+      <c r="A105" s="9" t="n"/>
+      <c r="B105" s="100" t="inlineStr">
         <is>
           <t>Business Logic Testing</t>
         </is>
       </c>
-      <c r="C107" s="101" t="inlineStr">
+      <c r="C105" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D107" s="101" t="inlineStr">
+      <c r="D105" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E107" s="101" t="inlineStr">
+      <c r="E105" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F107" s="101" t="inlineStr">
+      <c r="F105" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="82.5" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+    <row r="106" ht="82.5" customHeight="1" s="82">
+      <c r="A106" s="19" t="n"/>
+      <c r="B106" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C106" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D106" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="66" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="n"/>
+    </row>
+    <row r="107" ht="66" customHeight="1" s="82">
+      <c r="A107" s="19" t="n"/>
+      <c r="B107" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C107" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D107" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="148.5" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="n"/>
+    </row>
+    <row r="108" ht="148.5" customHeight="1" s="82">
+      <c r="A108" s="19" t="n"/>
+      <c r="B108" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C108" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3936,6 +3890,54 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="n"/>
+    </row>
+    <row r="109" ht="49.5" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-BUSL-04</t>
+        </is>
+      </c>
+      <c r="C109" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
+        <v/>
+      </c>
+      <c r="D109" s="16" t="inlineStr">
+        <is>
+          <t>- Review the project documentation for system functionality that may be impacted by time.
+- Develop and execute misuse cases.</t>
+        </is>
+      </c>
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="66" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-BUSL-05</t>
+        </is>
+      </c>
+      <c r="C110" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
+        <v/>
+      </c>
+      <c r="D110" s="16" t="inlineStr">
+        <is>
+          <t>- Identify functions that must set limits to the times they can be called.
+- Assess if there is a logical limit set on the functions and if it is properly validated.</t>
+        </is>
+      </c>
       <c r="E110" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3943,21 +3945,21 @@
       </c>
       <c r="F110" s="18" t="n"/>
     </row>
-    <row r="111" ht="49.5" customHeight="1" s="82">
+    <row r="111" ht="82.5" customHeight="1" s="82">
       <c r="A111" s="19" t="n"/>
       <c r="B111" s="34" t="inlineStr">
         <is>
-          <t>WSTG-BUSL-04</t>
+          <t>WSTG-BUSL-06</t>
         </is>
       </c>
       <c r="C111" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
         <v/>
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>- Review the project documentation for system functionality that may be impacted by time.
-- Develop and execute misuse cases.</t>
+          <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
+- Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
       <c r="E111" s="18" t="inlineStr">
@@ -3967,116 +3969,68 @@
       </c>
       <c r="F111" s="18" t="n"/>
     </row>
-    <row r="112" ht="66" customHeight="1" s="82">
+    <row r="112" ht="99" customHeight="1" s="82">
       <c r="A112" s="19" t="n"/>
       <c r="B112" s="34" t="inlineStr">
         <is>
-          <t>WSTG-BUSL-05</t>
+          <t>WSTG-BUSL-07</t>
         </is>
       </c>
       <c r="C112" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
         <v/>
       </c>
       <c r="D112" s="16" t="inlineStr">
-        <is>
-          <t>- Identify functions that must set limits to the times they can be called.
-- Assess if there is a logical limit set on the functions and if it is properly validated.</t>
-        </is>
-      </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="82.5" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-BUSL-06</t>
-        </is>
-      </c>
-      <c r="C113" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
-        <v/>
-      </c>
-      <c r="D113" s="16" t="inlineStr">
-        <is>
-          <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
-- Develop a misuse case and try to circumvent every logic flow identified.</t>
-        </is>
-      </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="99" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-BUSL-07</t>
-        </is>
-      </c>
-      <c r="C114" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
-        <v/>
-      </c>
-      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="99" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="99" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="165" customHeight="1" s="82">
-      <c r="A116" s="19" t="n"/>
-      <c r="B116" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="165" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C116" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D116" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4086,89 +4040,135 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F116" s="18" t="n"/>
-    </row>
-    <row r="117" ht="66" customHeight="1" s="82">
-      <c r="A117" s="19" t="n"/>
-      <c r="B117" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="66" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C117" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D117" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E117" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F117" s="18" t="n"/>
-    </row>
-    <row r="118" ht="15" customHeight="1" s="82">
-      <c r="A118" s="97" t="n"/>
-      <c r="B118" s="98" t="n"/>
-      <c r="C118" s="99" t="n"/>
-      <c r="D118" s="99" t="n"/>
-      <c r="E118" s="99" t="n"/>
-      <c r="F118" s="99" t="n"/>
-    </row>
-    <row r="119" ht="47.25" customHeight="1" s="82">
-      <c r="A119" s="9" t="n"/>
-      <c r="B119" s="100" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="15" customHeight="1" s="82">
+      <c r="A116" s="97" t="n"/>
+      <c r="B116" s="98" t="n"/>
+      <c r="C116" s="99" t="n"/>
+      <c r="D116" s="99" t="n"/>
+      <c r="E116" s="99" t="n"/>
+      <c r="F116" s="99" t="n"/>
+    </row>
+    <row r="117" ht="47.25" customHeight="1" s="82">
+      <c r="A117" s="9" t="n"/>
+      <c r="B117" s="100" t="inlineStr">
         <is>
           <t>Client-side Testing</t>
         </is>
       </c>
-      <c r="C119" s="101" t="inlineStr">
+      <c r="C117" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D119" s="101" t="inlineStr">
+      <c r="D117" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E119" s="101" t="inlineStr">
+      <c r="E117" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F119" s="101" t="inlineStr">
+      <c r="F117" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="118" ht="33" customHeight="1" s="82">
+      <c r="A118" s="19" t="n"/>
+      <c r="B118" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CLNT-01</t>
+        </is>
+      </c>
+      <c r="C118" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
+        <v/>
+      </c>
+      <c r="D118" s="16" t="inlineStr">
+        <is>
+          <t>- Identify DOM sinks.
+- Build payloads that pertain to every sink type.</t>
+        </is>
+      </c>
+      <c r="E118" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="n"/>
+    </row>
+    <row r="119" ht="16.5" customHeight="1" s="82">
+      <c r="A119" s="19" t="n"/>
+      <c r="B119" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CLNT-02</t>
+        </is>
+      </c>
+      <c r="C119" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
+        <v/>
+      </c>
+      <c r="D119" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
+        </is>
+      </c>
+      <c r="E119" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F119" s="18" t="n"/>
     </row>
     <row r="120" ht="33" customHeight="1" s="82">
       <c r="A120" s="19" t="n"/>
       <c r="B120" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-01</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
         <v/>
       </c>
       <c r="D120" s="16" t="inlineStr">
         <is>
-          <t>- Identify DOM sinks.
-- Build payloads that pertain to every sink type.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E120" s="18" t="inlineStr">
@@ -4178,20 +4178,21 @@
       </c>
       <c r="F120" s="18" t="n"/>
     </row>
-    <row r="121" ht="16.5" customHeight="1" s="82">
+    <row r="121" ht="33" customHeight="1" s="82">
       <c r="A121" s="19" t="n"/>
       <c r="B121" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-02</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr">
@@ -4205,16 +4206,17 @@
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4228,17 +4230,17 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-06</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4252,17 +4254,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-07</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify endpoints that implement CORS.
+- Ensure that the CORS configuration is secure or harmless.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4276,17 +4278,17 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-08</t>
         </is>
       </c>
       <c r="C125" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
         <v/>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Decompile and analyze the application's code.
+- Assess sinks inputs and unsafe method usages.</t>
         </is>
       </c>
       <c r="E125" s="18" t="inlineStr">
@@ -4296,21 +4298,20 @@
       </c>
       <c r="F125" s="18" t="n"/>
     </row>
-    <row r="126" ht="33" customHeight="1" s="82">
+    <row r="126" ht="16.5" customHeight="1" s="82">
       <c r="A126" s="19" t="n"/>
       <c r="B126" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-07</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D126" s="16" t="inlineStr">
         <is>
-          <t>- Identify endpoints that implement CORS.
-- Ensure that the CORS configuration is secure or harmless.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E126" s="18" t="inlineStr">
@@ -4320,21 +4321,21 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="33" customHeight="1" s="82">
+    <row r="127" ht="49.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-08</t>
+          <t>WSTG-CLNT-10</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Decompile and analyze the application's code.
-- Assess sinks inputs and unsafe method usages.</t>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4344,20 +4345,21 @@
       </c>
       <c r="F127" s="18" t="n"/>
     </row>
-    <row r="128" ht="16.5" customHeight="1" s="82">
+    <row r="128" ht="49.5" customHeight="1" s="82">
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-09</t>
+          <t>WSTG-CLNT-11</t>
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
         <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
+          <t>- Assess the security of the message's origin.
+- Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
       <c r="E128" s="18" t="inlineStr">
@@ -4367,21 +4369,21 @@
       </c>
       <c r="F128" s="18" t="n"/>
     </row>
-    <row r="129" ht="49.5" customHeight="1" s="82">
+    <row r="129" ht="82.5" customHeight="1" s="82">
       <c r="A129" s="19" t="n"/>
       <c r="B129" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-12</t>
         </is>
       </c>
       <c r="C129" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Determine whether the site is storing sensitive data in client-side storage.
+- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
       <c r="E129" s="18" t="inlineStr">
@@ -4395,17 +4397,17 @@
       <c r="A130" s="19" t="n"/>
       <c r="B130" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-11</t>
+          <t>WSTG-CLNT-13</t>
         </is>
       </c>
       <c r="C130" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
       <c r="D130" s="16" t="inlineStr">
         <is>
-          <t>- Assess the security of the message's origin.
-- Validate that it's using safe methods and validating its input.</t>
+          <t>- Locate sensitive data across the system.
+- Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
       <c r="E130" s="18" t="inlineStr">
@@ -4415,21 +4417,20 @@
       </c>
       <c r="F130" s="18" t="n"/>
     </row>
-    <row r="131" ht="82.5" customHeight="1" s="82">
+    <row r="131" ht="16.5" customHeight="1" s="82">
       <c r="A131" s="19" t="n"/>
       <c r="B131" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-12</t>
+          <t>WSTG-CLNT-14</t>
         </is>
       </c>
       <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
         <v/>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the site is storing sensitive data in client-side storage.
-- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E131" s="18" t="inlineStr">
@@ -4439,242 +4440,195 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="49.5" customHeight="1" s="82">
+    <row r="132" ht="99" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-13</t>
+          <t>WSTG-CLNT-15</t>
         </is>
       </c>
       <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
       <c r="D132" s="16" t="inlineStr">
-        <is>
-          <t>- Locate sensitive data across the system.
-- Assess the leakage of sensitive data through various techniques.</t>
-        </is>
-      </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="16.5" customHeight="1" s="82">
-      <c r="A133" s="19" t="n"/>
-      <c r="B133" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C133" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D133" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F133" s="18" t="n"/>
-    </row>
-    <row r="134" ht="99" customHeight="1" s="82">
-      <c r="A134" s="19" t="n"/>
-      <c r="B134" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-15</t>
-        </is>
-      </c>
-      <c r="C134" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
-        <v/>
-      </c>
-      <c r="D134" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E134" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F134" s="18" t="n"/>
-    </row>
-    <row r="135" ht="15" customHeight="1" s="82">
-      <c r="A135" s="97" t="n"/>
-      <c r="B135" s="98" t="n"/>
-      <c r="C135" s="99" t="n"/>
-      <c r="D135" s="99" t="n"/>
-      <c r="E135" s="99" t="n"/>
-      <c r="F135" s="99" t="n"/>
-    </row>
-    <row r="136" ht="47.25" customHeight="1" s="82">
-      <c r="A136" s="9" t="n"/>
-      <c r="B136" s="100" t="inlineStr">
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="15" customHeight="1" s="82">
+      <c r="A133" s="97" t="n"/>
+      <c r="B133" s="98" t="n"/>
+      <c r="C133" s="99" t="n"/>
+      <c r="D133" s="99" t="n"/>
+      <c r="E133" s="99" t="n"/>
+      <c r="F133" s="99" t="n"/>
+    </row>
+    <row r="134" ht="47.25" customHeight="1" s="82">
+      <c r="A134" s="9" t="n"/>
+      <c r="B134" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C136" s="101" t="inlineStr">
+      <c r="C134" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D136" s="101" t="inlineStr">
+      <c r="D134" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E136" s="101" t="inlineStr">
+      <c r="E134" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F136" s="101" t="inlineStr">
+      <c r="F134" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="99" customHeight="1" s="82">
-      <c r="A137" s="19" t="n"/>
-      <c r="B137" s="34" t="inlineStr">
+    <row r="135" ht="99" customHeight="1" s="82">
+      <c r="A135" s="19" t="n"/>
+      <c r="B135" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C137" s="15">
+      <c r="C135" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D135" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="66" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
+      <c r="E135" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F135" s="18" t="n"/>
+    </row>
+    <row r="136" ht="66" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-02</t>
         </is>
       </c>
-      <c r="C138" s="15">
+      <c r="C136" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
         <v/>
       </c>
-      <c r="D138" s="16" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
         </is>
       </c>
-      <c r="E138" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F138" s="18" t="n"/>
-    </row>
-    <row r="139" ht="132" customHeight="1" s="82">
-      <c r="A139" s="19" t="n"/>
-      <c r="B139" s="34" t="inlineStr">
+      <c r="E136" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F136" s="18" t="n"/>
+    </row>
+    <row r="137" ht="132" customHeight="1" s="82">
+      <c r="A137" s="19" t="n"/>
+      <c r="B137" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C137" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D137" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="82.5" customHeight="1" s="82">
-      <c r="A140" s="19" t="n"/>
-      <c r="B140" s="34" t="inlineStr">
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="82.5" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C140" s="15">
+      <c r="C138" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
         <v/>
       </c>
-      <c r="D140" s="16" t="inlineStr">
+      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="66" customHeight="1" s="82">
-      <c r="A141" s="19" t="n"/>
-      <c r="B141" s="34" t="inlineStr">
+      <c r="E138" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F138" s="18" t="n"/>
+    </row>
+    <row r="139" ht="66" customHeight="1" s="82">
+      <c r="A139" s="19" t="n"/>
+      <c r="B139" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C141" s="15">
+      <c r="C139" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D141" s="16" t="inlineStr">
+      <c r="D139" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E141" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F141" s="18" t="n"/>
-    </row>
-    <row r="142" ht="15" customHeight="1" s="82">
-      <c r="A142" s="97" t="n"/>
-      <c r="B142" s="98" t="n"/>
-      <c r="C142" s="99" t="n"/>
-      <c r="D142" s="99" t="n"/>
-      <c r="E142" s="99" t="n"/>
-      <c r="F142" s="99" t="n"/>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="15" customHeight="1" s="82">
+      <c r="A140" s="97" t="n"/>
+      <c r="B140" s="98" t="n"/>
+      <c r="C140" s="99" t="n"/>
+      <c r="D140" s="99" t="n"/>
+      <c r="E140" s="99" t="n"/>
+      <c r="F140" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4691,7 +4645,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F142">
+  <conditionalFormatting sqref="B4:F140">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4703,7 +4657,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E96 E97 E100 E101 E102 E103 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-04-22 (#1406)
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -1983,16 +1983,16 @@
       <c r="A25" s="19" t="n"/>
       <c r="B25" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-08</t>
+          <t>WSTG-CONF-09</t>
         </is>
       </c>
       <c r="C25" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/08-Test_RIA_Cross_Domain_Policy", "Test RIA Cross Domain Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/09-Test_File_Permission", "Test File Permission")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- Review and identify any rogue file permissions.</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
@@ -2002,20 +2002,21 @@
       </c>
       <c r="F25" s="18" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="82">
+    <row r="26" ht="33" customHeight="1" s="82">
       <c r="A26" s="19" t="n"/>
       <c r="B26" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-09</t>
+          <t>WSTG-CONF-10</t>
         </is>
       </c>
       <c r="C26" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/09-Test_File_Permission", "Test File Permission")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/10-Test_for_Subdomain_Takeover", "Test for Subdomain Takeover")</f>
         <v/>
       </c>
       <c r="D26" s="16" t="inlineStr">
         <is>
-          <t>- Review and identify any rogue file permissions.</t>
+          <t>- Enumerate all possible domains (previous and current).
+- Identify any forgotten or misconfigured domains.</t>
         </is>
       </c>
       <c r="E26" s="18" t="inlineStr">
@@ -2029,17 +2030,16 @@
       <c r="A27" s="19" t="n"/>
       <c r="B27" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-10</t>
+          <t>WSTG-CONF-11</t>
         </is>
       </c>
       <c r="C27" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/10-Test_for_Subdomain_Takeover", "Test for Subdomain Takeover")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/11-Test_Cloud_Storage", "Test Cloud Storage")</f>
         <v/>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>- Enumerate all possible domains (previous and current).
-- Identify any forgotten or misconfigured domains.</t>
+          <t>- Assess that the access control configuration for the storage services is properly in place.</t>
         </is>
       </c>
       <c r="E27" s="18" t="inlineStr">
@@ -2053,16 +2053,16 @@
       <c r="A28" s="19" t="n"/>
       <c r="B28" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-11</t>
+          <t>WSTG-CONF-12</t>
         </is>
       </c>
       <c r="C28" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/11-Test_Cloud_Storage", "Test Cloud Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Testing for Content Security Policy")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="inlineStr">
         <is>
-          <t>- Assess that the access control configuration for the storage services is properly in place.</t>
+          <t>- Review the Content-Security-Policy header or meta element to identify misconfigurations.</t>
         </is>
       </c>
       <c r="E28" s="18" t="inlineStr">
@@ -2072,20 +2072,20 @@
       </c>
       <c r="F28" s="18" t="n"/>
     </row>
-    <row r="29" ht="33" customHeight="1" s="82">
+    <row r="29" ht="16.5" customHeight="1" s="82">
       <c r="A29" s="19" t="n"/>
       <c r="B29" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-12</t>
+          <t>WSTG-CONF-13</t>
         </is>
       </c>
       <c r="C29" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Testing for Content Security Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/13-Test_for_Path_Confusion", "Test Path Confusion")</f>
         <v/>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>- Review the Content-Security-Policy header or meta element to identify misconfigurations.</t>
+          <t>- Make sure application paths are configured correctly.</t>
         </is>
       </c>
       <c r="E29" s="18" t="inlineStr">
@@ -2095,108 +2095,109 @@
       </c>
       <c r="F29" s="18" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="82">
+    <row r="30" ht="66" customHeight="1" s="82">
       <c r="A30" s="19" t="n"/>
       <c r="B30" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CONF-13</t>
+          <t>WSTG-CONF-14</t>
         </is>
       </c>
       <c r="C30" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/13-Test_for_Path_Confusion", "Test Path Confusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/14-Test_Other_HTTP_Security_Header_Misconfigurations", "Test Other HTTP Security Header Misconfigurations")</f>
         <v/>
       </c>
       <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t>- Make sure application paths are configured correctly.</t>
-        </is>
-      </c>
-      <c r="E30" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="n"/>
-    </row>
-    <row r="31" ht="66" customHeight="1" s="82">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CONF-14</t>
-        </is>
-      </c>
-      <c r="C31" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/14-Test_Other_HTTP_Security_Header_Misconfigurations", "Test Other HTTP Security Header Misconfigurations")</f>
-        <v/>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>- Identify improperly configured security headers.
 - Assess the impact of misconfigured security headers.
 - Validate the correct implementation of required security headers.</t>
         </is>
       </c>
-      <c r="E31" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F31" s="18" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="82">
-      <c r="A32" s="97" t="n"/>
-      <c r="B32" s="98" t="n"/>
-      <c r="C32" s="99" t="n"/>
-      <c r="D32" s="99" t="n"/>
-      <c r="E32" s="99" t="n"/>
-      <c r="F32" s="99" t="n"/>
-    </row>
-    <row r="33" ht="47.25" customHeight="1" s="82">
-      <c r="A33" s="9" t="n"/>
-      <c r="B33" s="100" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="82">
+      <c r="A31" s="97" t="n"/>
+      <c r="B31" s="98" t="n"/>
+      <c r="C31" s="99" t="n"/>
+      <c r="D31" s="99" t="n"/>
+      <c r="E31" s="99" t="n"/>
+      <c r="F31" s="99" t="n"/>
+    </row>
+    <row r="32" ht="47.25" customHeight="1" s="82">
+      <c r="A32" s="9" t="n"/>
+      <c r="B32" s="100" t="inlineStr">
         <is>
           <t>Identity Management Testing</t>
         </is>
       </c>
-      <c r="C33" s="101" t="inlineStr">
+      <c r="C32" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D33" s="101" t="inlineStr">
+      <c r="D32" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E33" s="101" t="inlineStr">
+      <c r="E32" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F33" s="101" t="inlineStr">
+      <c r="F32" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="66" customHeight="1" s="82">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="34" t="inlineStr">
+    <row r="33" ht="66" customHeight="1" s="82">
+      <c r="A33" s="19" t="n"/>
+      <c r="B33" s="34" t="inlineStr">
         <is>
           <t>WSTG-IDNT-01</t>
         </is>
       </c>
-      <c r="C34" s="15">
+      <c r="C33" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/01-Test_Role_Definitions", "Test Role Definitions")</f>
         <v/>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>- Identify and document roles used by the application.
 - Attempt to switch, change, or access another role.
 - Review the granularity of the roles and the needs behind the permissions given.</t>
         </is>
       </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F33" s="18" t="n"/>
+    </row>
+    <row r="34" ht="49.5" customHeight="1" s="82">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-IDNT-02</t>
+        </is>
+      </c>
+      <c r="C34" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/02-Test_User_Registration_Process", "Test User Registration Process")</f>
+        <v/>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>- Verify that the identity requirements for user registration are aligned with business and security requirements.
+- Validate the registration process.</t>
+        </is>
+      </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2204,21 +2205,20 @@
       </c>
       <c r="F34" s="18" t="n"/>
     </row>
-    <row r="35" ht="49.5" customHeight="1" s="82">
+    <row r="35" ht="33" customHeight="1" s="82">
       <c r="A35" s="19" t="n"/>
       <c r="B35" s="34" t="inlineStr">
         <is>
-          <t>WSTG-IDNT-02</t>
+          <t>WSTG-IDNT-03</t>
         </is>
       </c>
       <c r="C35" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/02-Test_User_Registration_Process", "Test User Registration Process")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/03-Test_Account_Provisioning_Process", "Test Account Provisioning Process")</f>
         <v/>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>- Verify that the identity requirements for user registration are aligned with business and security requirements.
-- Validate the registration process.</t>
+          <t>- Verify which accounts may provision other accounts and of what type.</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
@@ -2228,20 +2228,21 @@
       </c>
       <c r="F35" s="18" t="n"/>
     </row>
-    <row r="36" ht="33" customHeight="1" s="82">
+    <row r="36" ht="49.5" customHeight="1" s="82">
       <c r="A36" s="19" t="n"/>
       <c r="B36" s="34" t="inlineStr">
         <is>
-          <t>WSTG-IDNT-03</t>
+          <t>WSTG-IDNT-04</t>
         </is>
       </c>
       <c r="C36" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/03-Test_Account_Provisioning_Process", "Test Account Provisioning Process")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/04-Testing_for_Account_Enumeration_and_Guessable_User_Account", "Testing for Account Enumeration and Guessable User Account")</f>
         <v/>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>- Verify which accounts may provision other accounts and of what type.</t>
+          <t>- Review processes that pertain to user identification (*e.g.* registration, login, etc.).
+- Enumerate users where possible through response analysis.</t>
         </is>
       </c>
       <c r="E36" s="18" t="inlineStr">
@@ -2251,21 +2252,20 @@
       </c>
       <c r="F36" s="18" t="n"/>
     </row>
-    <row r="37" ht="49.5" customHeight="1" s="82">
+    <row r="37" ht="33" customHeight="1" s="82">
       <c r="A37" s="19" t="n"/>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>WSTG-IDNT-04</t>
+          <t>WSTG-IDNT-05</t>
         </is>
       </c>
       <c r="C37" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/04-Testing_for_Account_Enumeration_and_Guessable_User_Account", "Testing for Account Enumeration and Guessable User Account")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/05-Testing_for_Weak_or_Unenforced_Username_Policy", "Testing for Weak or Unenforced Username Policy")</f>
         <v/>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>- Review processes that pertain to user identification (*e.g.* registration, login, etc.).
-- Enumerate users where possible through response analysis.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E37" s="18" t="inlineStr">
@@ -2275,79 +2275,80 @@
       </c>
       <c r="F37" s="18" t="n"/>
     </row>
-    <row r="38" ht="33" customHeight="1" s="82">
-      <c r="A38" s="19" t="n"/>
-      <c r="B38" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-IDNT-05</t>
-        </is>
-      </c>
-      <c r="C38" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/05-Testing_for_Weak_or_Unenforced_Username_Policy", "Testing for Weak or Unenforced Username Policy")</f>
-        <v/>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+    <row r="38" ht="15" customHeight="1" s="82">
+      <c r="A38" s="97" t="n"/>
+      <c r="B38" s="98" t="n"/>
+      <c r="C38" s="99" t="n"/>
+      <c r="D38" s="99" t="n"/>
+      <c r="E38" s="99" t="n"/>
+      <c r="F38" s="99" t="n"/>
+    </row>
+    <row r="39" ht="47.25" customHeight="1" s="82">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="100" t="inlineStr">
+        <is>
+          <t>Authentication Testing</t>
+        </is>
+      </c>
+      <c r="C39" s="101" t="inlineStr">
+        <is>
+          <t>Test Name</t>
+        </is>
+      </c>
+      <c r="D39" s="101" t="inlineStr">
+        <is>
+          <t>Objectives</t>
+        </is>
+      </c>
+      <c r="E39" s="101" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F39" s="101" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="33" customHeight="1" s="82">
+      <c r="A40" s="19" t="n"/>
+      <c r="B40" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-ATHN-01</t>
+        </is>
+      </c>
+      <c r="C40" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/01-Testing_for_Credentials_Transported_over_an_Encrypted_Channel", "Testing for Credentials Transported over an Encrypted Channel")</f>
+        <v/>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F38" s="18" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="82">
-      <c r="A39" s="97" t="n"/>
-      <c r="B39" s="98" t="n"/>
-      <c r="C39" s="99" t="n"/>
-      <c r="D39" s="99" t="n"/>
-      <c r="E39" s="99" t="n"/>
-      <c r="F39" s="99" t="n"/>
-    </row>
-    <row r="40" ht="47.25" customHeight="1" s="82">
-      <c r="A40" s="9" t="n"/>
-      <c r="B40" s="100" t="inlineStr">
-        <is>
-          <t>Authentication Testing</t>
-        </is>
-      </c>
-      <c r="C40" s="101" t="inlineStr">
-        <is>
-          <t>Test Name</t>
-        </is>
-      </c>
-      <c r="D40" s="101" t="inlineStr">
-        <is>
-          <t>Objectives</t>
-        </is>
-      </c>
-      <c r="E40" s="101" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F40" s="101" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="33" customHeight="1" s="82">
+      <c r="E40" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F40" s="18" t="n"/>
+    </row>
+    <row r="41" ht="66" customHeight="1" s="82">
       <c r="A41" s="19" t="n"/>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-01</t>
+          <t>WSTG-ATHN-02</t>
         </is>
       </c>
       <c r="C41" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/01-Testing_for_Credentials_Transported_over_an_Encrypted_Channel", "Testing for Credentials Transported over an Encrypted Channel")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/02-Testing_for_Default_Credentials", "Testing for Default Credentials")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- Determine whether the application has any user accounts with default passwords.
+- Review whether new user accounts are created with weak or predictable passwords.</t>
         </is>
       </c>
       <c r="E41" s="18" t="inlineStr">
@@ -2361,17 +2362,17 @@
       <c r="A42" s="19" t="n"/>
       <c r="B42" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-02</t>
+          <t>WSTG-ATHN-03</t>
         </is>
       </c>
       <c r="C42" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/02-Testing_for_Default_Credentials", "Testing for Default Credentials")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/03-Testing_for_Weak_Lock_Out_Mechanism", "Testing for Weak Lock Out Mechanism")</f>
         <v/>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the application has any user accounts with default passwords.
-- Review whether new user accounts are created with weak or predictable passwords.</t>
+          <t>- Evaluate the account lockout mechanism's ability to mitigate brute force password guessing.
+- Evaluate the unlock mechanism's resistance to unauthorized account unlocking.</t>
         </is>
       </c>
       <c r="E42" s="18" t="inlineStr">
@@ -2381,21 +2382,20 @@
       </c>
       <c r="F42" s="18" t="n"/>
     </row>
-    <row r="43" ht="66" customHeight="1" s="82">
+    <row r="43" ht="33" customHeight="1" s="82">
       <c r="A43" s="19" t="n"/>
       <c r="B43" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-03</t>
+          <t>WSTG-ATHN-04</t>
         </is>
       </c>
       <c r="C43" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/03-Testing_for_Weak_Lock_Out_Mechanism", "Testing for Weak Lock Out Mechanism")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/04-Testing_for_Bypassing_Authentication_Schema", "Testing for Bypassing Authentication Schema")</f>
         <v/>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>- Evaluate the account lockout mechanism's ability to mitigate brute force password guessing.
-- Evaluate the unlock mechanism's resistance to unauthorized account unlocking.</t>
+          <t>- Ensure that authentication is applied across all services that require it.</t>
         </is>
       </c>
       <c r="E43" s="18" t="inlineStr">
@@ -2409,16 +2409,16 @@
       <c r="A44" s="19" t="n"/>
       <c r="B44" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-04</t>
+          <t>WSTG-ATHN-05</t>
         </is>
       </c>
       <c r="C44" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/04-Testing_for_Bypassing_Authentication_Schema", "Testing for Bypassing Authentication Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/05-Testing_for_Vulnerable_Remember_Password", "Testing for Vulnerable Remember Password")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>- Ensure that authentication is applied across all services that require it.</t>
+          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
         </is>
       </c>
       <c r="E44" s="18" t="inlineStr">
@@ -2428,20 +2428,21 @@
       </c>
       <c r="F44" s="18" t="n"/>
     </row>
-    <row r="45" ht="33" customHeight="1" s="82">
+    <row r="45" ht="49.5" customHeight="1" s="82">
       <c r="A45" s="19" t="n"/>
       <c r="B45" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-05</t>
+          <t>WSTG-ATHN-06</t>
         </is>
       </c>
       <c r="C45" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/05-Testing_for_Vulnerable_Remember_Password", "Testing for Vulnerable Remember Password")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/06-Testing_for_Browser_Cache_Weaknesses", "Testing for Browser Cache Weaknesses")</f>
         <v/>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>- Validate that the generated session is managed securely and do not put the user's credentials in danger.</t>
+          <t>- Review if the application stores sensitive information on the client-side.
+- Review if access can occur without authorization.</t>
         </is>
       </c>
       <c r="E45" s="18" t="inlineStr">
@@ -2451,21 +2452,20 @@
       </c>
       <c r="F45" s="18" t="n"/>
     </row>
-    <row r="46" ht="49.5" customHeight="1" s="82">
+    <row r="46" ht="66" customHeight="1" s="82">
       <c r="A46" s="19" t="n"/>
       <c r="B46" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-06</t>
+          <t>WSTG-ATHN-07</t>
         </is>
       </c>
       <c r="C46" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/06-Testing_for_Browser_Cache_Weaknesses", "Testing for Browser Cache Weaknesses")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/07-Testing_for_Weak_Authentication_Methods", "Testing for Weak Authentication Methods")</f>
         <v/>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>- Review if the application stores sensitive information on the client-side.
-- Review if access can occur without authorization.</t>
+          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
         </is>
       </c>
       <c r="E46" s="18" t="inlineStr">
@@ -2475,20 +2475,21 @@
       </c>
       <c r="F46" s="18" t="n"/>
     </row>
-    <row r="47" ht="66" customHeight="1" s="82">
+    <row r="47" ht="49.5" customHeight="1" s="82">
       <c r="A47" s="19" t="n"/>
       <c r="B47" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-07</t>
+          <t>WSTG-ATHN-08</t>
         </is>
       </c>
       <c r="C47" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/07-Testing_for_Weak_Authentication_Methods", "Testing for Weak Authentication Methods")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/08-Testing_for_Weak_Security_Question_Answer", "Testing for Weak Security Question Answer")</f>
         <v/>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>- Determine the resistance of the application against brute force password guessing using available password dictionaries by evaluating the length, complexity, reuse, and aging requirements of passwords.</t>
+          <t>- Determine the complexity and how straight-forward the questions are.
+- Assess possible user answers and brute force capabilities.</t>
         </is>
       </c>
       <c r="E47" s="18" t="inlineStr">
@@ -2498,21 +2499,20 @@
       </c>
       <c r="F47" s="18" t="n"/>
     </row>
-    <row r="48" ht="49.5" customHeight="1" s="82">
+    <row r="48" ht="33" customHeight="1" s="82">
       <c r="A48" s="19" t="n"/>
       <c r="B48" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-08</t>
+          <t>WSTG-ATHN-09</t>
         </is>
       </c>
       <c r="C48" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/08-Testing_for_Weak_Security_Question_Answer", "Testing for Weak Security Question Answer")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/09-Testing_for_Weak_Password_Change_or_Reset_Functionalities", "Testing for Weak Password Change or Reset Functionalities")</f>
         <v/>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>- Determine the complexity and how straight-forward the questions are.
-- Assess possible user answers and brute force capabilities.</t>
+          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
         </is>
       </c>
       <c r="E48" s="18" t="inlineStr">
@@ -2522,20 +2522,21 @@
       </c>
       <c r="F48" s="18" t="n"/>
     </row>
-    <row r="49" ht="33" customHeight="1" s="82">
+    <row r="49" ht="49.5" customHeight="1" s="82">
       <c r="A49" s="19" t="n"/>
       <c r="B49" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-09</t>
+          <t>WSTG-ATHN-10</t>
         </is>
       </c>
       <c r="C49" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/09-Testing_for_Weak_Password_Change_or_Reset_Functionalities", "Testing for Weak Password Change or Reset Functionalities")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/10-Testing_for_Weaker_Authentication_in_Alternative_Channel", "Testing for Weaker Authentication in Alternative Channel")</f>
         <v/>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the password change and reset functionality allows accounts to be compromised.</t>
+          <t>- Identify alternative authentication channels.
+- Assess the security measures used and if any bypasses exists on the alternative channels.</t>
         </is>
       </c>
       <c r="E49" s="18" t="inlineStr">
@@ -2545,106 +2546,105 @@
       </c>
       <c r="F49" s="18" t="n"/>
     </row>
-    <row r="50" ht="49.5" customHeight="1" s="82">
+    <row r="50" ht="66" customHeight="1" s="82">
       <c r="A50" s="19" t="n"/>
       <c r="B50" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHN-10</t>
+          <t>WSTG-ATHN-11</t>
         </is>
       </c>
       <c r="C50" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/10-Testing_for_Weaker_Authentication_in_Alternative_Channel", "Testing for Weaker Authentication in Alternative Channel")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/11-Testing_Multi-Factor_Authentication", "Testing Multi-Factor Authentication (MFA)")</f>
         <v/>
       </c>
       <c r="D50" s="16" t="inlineStr">
-        <is>
-          <t>- Identify alternative authentication channels.
-- Assess the security measures used and if any bypasses exists on the alternative channels.</t>
-        </is>
-      </c>
-      <c r="E50" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F50" s="18" t="n"/>
-    </row>
-    <row r="51" ht="66" customHeight="1" s="82">
-      <c r="A51" s="19" t="n"/>
-      <c r="B51" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHN-11</t>
-        </is>
-      </c>
-      <c r="C51" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/11-Testing_Multi-Factor_Authentication", "Testing Multi-Factor Authentication (MFA)")</f>
-        <v/>
-      </c>
-      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>- Identify the type of MFA used by the application.
 - Determine whether the MFA implementation is robust and secure.
 - Attempt to bypass the MFA.</t>
         </is>
       </c>
-      <c r="E51" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="82">
-      <c r="A52" s="97" t="n"/>
-      <c r="B52" s="98" t="n"/>
-      <c r="C52" s="99" t="n"/>
-      <c r="D52" s="99" t="n"/>
-      <c r="E52" s="99" t="n"/>
-      <c r="F52" s="99" t="n"/>
-    </row>
-    <row r="53" ht="47.25" customHeight="1" s="82">
-      <c r="A53" s="9" t="n"/>
-      <c r="B53" s="100" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F50" s="18" t="n"/>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="82">
+      <c r="A51" s="97" t="n"/>
+      <c r="B51" s="98" t="n"/>
+      <c r="C51" s="99" t="n"/>
+      <c r="D51" s="99" t="n"/>
+      <c r="E51" s="99" t="n"/>
+      <c r="F51" s="99" t="n"/>
+    </row>
+    <row r="52" ht="47.25" customHeight="1" s="82">
+      <c r="A52" s="9" t="n"/>
+      <c r="B52" s="100" t="inlineStr">
         <is>
           <t>Authorization Testing</t>
         </is>
       </c>
-      <c r="C53" s="101" t="inlineStr">
+      <c r="C52" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D53" s="101" t="inlineStr">
+      <c r="D52" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E53" s="101" t="inlineStr">
+      <c r="E52" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F53" s="101" t="inlineStr">
+      <c r="F52" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="49.5" customHeight="1" s="82">
+    <row r="53" ht="49.5" customHeight="1" s="82">
+      <c r="A53" s="19" t="n"/>
+      <c r="B53" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-ATHZ-01</t>
+        </is>
+      </c>
+      <c r="C53" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/01-Testing_Directory_Traversal_File_Include", "Testing Directory Traversal File Include")</f>
+        <v/>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>- Identify injection points that pertain to path traversal.
+- Assess bypassing techniques and identify the extent of path traversal.</t>
+        </is>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="n"/>
+    </row>
+    <row r="54" ht="33" customHeight="1" s="82">
       <c r="A54" s="19" t="n"/>
       <c r="B54" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-01</t>
+          <t>WSTG-ATHZ-02</t>
         </is>
       </c>
       <c r="C54" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/01-Testing_Directory_Traversal_File_Include", "Testing Directory Traversal File Include")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/02-Testing_for_Bypassing_Authorization_Schema", "Testing for Bypassing Authorization Schema")</f>
         <v/>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that pertain to path traversal.
-- Assess bypassing techniques and identify the extent of path traversal.</t>
+          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
         </is>
       </c>
       <c r="E54" s="18" t="inlineStr">
@@ -2654,20 +2654,21 @@
       </c>
       <c r="F54" s="18" t="n"/>
     </row>
-    <row r="55" ht="33" customHeight="1" s="82">
+    <row r="55" ht="49.5" customHeight="1" s="82">
       <c r="A55" s="19" t="n"/>
       <c r="B55" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-02</t>
+          <t>WSTG-ATHZ-03</t>
         </is>
       </c>
       <c r="C55" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/02-Testing_for_Bypassing_Authorization_Schema", "Testing for Bypassing Authorization Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/03-Testing_for_Privilege_Escalation", "Testing for Privilege Escalation")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>- Assess if unauthenticated, horizontal, or vertical access is possible.</t>
+          <t>- Identify injection points related to privilege manipulation.
+- Fuzz or otherwise attempt to bypass security measures.</t>
         </is>
       </c>
       <c r="E55" s="18" t="inlineStr">
@@ -2681,17 +2682,17 @@
       <c r="A56" s="19" t="n"/>
       <c r="B56" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-03</t>
+          <t>WSTG-ATHZ-04</t>
         </is>
       </c>
       <c r="C56" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/03-Testing_for_Privilege_Escalation", "Testing for Privilege Escalation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/04-Testing_for_Insecure_Direct_Object_References", "Testing for Insecure Direct Object References")</f>
         <v/>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points related to privilege manipulation.
-- Fuzz or otherwise attempt to bypass security measures.</t>
+          <t>- Identify points where object references may occur.
+- Assess the access control measures and if they're vulnerable to IDOR.</t>
         </is>
       </c>
       <c r="E56" s="18" t="inlineStr">
@@ -2701,21 +2702,20 @@
       </c>
       <c r="F56" s="18" t="n"/>
     </row>
-    <row r="57" ht="49.5" customHeight="1" s="82">
+    <row r="57" ht="33" customHeight="1" s="82">
       <c r="A57" s="19" t="n"/>
       <c r="B57" s="34" t="inlineStr">
         <is>
-          <t>WSTG-ATHZ-04</t>
+          <t>WSTG-ATHZ-05</t>
         </is>
       </c>
       <c r="C57" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/04-Testing_for_Insecure_Direct_Object_References", "Testing for Insecure Direct Object References")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/05-Testing_for_OAuth_Weaknesses", "Testing for OAuth Weaknesses")</f>
         <v/>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>- Identify points where object references may occur.
-- Assess the access control measures and if they're vulnerable to IDOR.</t>
+          <t>- Determine if OAuth2 implementation is vulnerable or using a deprecated or custom implementation.</t>
         </is>
       </c>
       <c r="E57" s="18" t="inlineStr">
@@ -2725,83 +2725,83 @@
       </c>
       <c r="F57" s="18" t="n"/>
     </row>
-    <row r="58" ht="33" customHeight="1" s="82">
-      <c r="A58" s="19" t="n"/>
-      <c r="B58" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-ATHZ-05</t>
-        </is>
-      </c>
-      <c r="C58" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/05-Testing_for_OAuth_Weaknesses", "Testing for OAuth Weaknesses")</f>
-        <v/>
-      </c>
-      <c r="D58" s="16" t="inlineStr">
-        <is>
-          <t>- Determine if OAuth2 implementation is vulnerable or using a deprecated or custom implementation.</t>
-        </is>
-      </c>
-      <c r="E58" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F58" s="18" t="n"/>
-    </row>
-    <row r="59" ht="15" customHeight="1" s="82">
-      <c r="A59" s="97" t="n"/>
-      <c r="B59" s="98" t="n"/>
-      <c r="C59" s="99" t="n"/>
-      <c r="D59" s="99" t="n"/>
-      <c r="E59" s="99" t="n"/>
-      <c r="F59" s="99" t="n"/>
-    </row>
-    <row r="60" ht="47.25" customHeight="1" s="82">
-      <c r="A60" s="9" t="n"/>
-      <c r="B60" s="100" t="inlineStr">
+    <row r="58" ht="15" customHeight="1" s="82">
+      <c r="A58" s="97" t="n"/>
+      <c r="B58" s="98" t="n"/>
+      <c r="C58" s="99" t="n"/>
+      <c r="D58" s="99" t="n"/>
+      <c r="E58" s="99" t="n"/>
+      <c r="F58" s="99" t="n"/>
+    </row>
+    <row r="59" ht="47.25" customHeight="1" s="82">
+      <c r="A59" s="9" t="n"/>
+      <c r="B59" s="100" t="inlineStr">
         <is>
           <t>Session Management Testing</t>
         </is>
       </c>
-      <c r="C60" s="101" t="inlineStr">
+      <c r="C59" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D60" s="101" t="inlineStr">
+      <c r="D59" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E60" s="101" t="inlineStr">
+      <c r="E59" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F60" s="101" t="inlineStr">
+      <c r="F59" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="99" customHeight="1" s="82">
-      <c r="A61" s="19" t="n"/>
-      <c r="B61" s="34" t="inlineStr">
+    <row r="60" ht="99" customHeight="1" s="82">
+      <c r="A60" s="19" t="n"/>
+      <c r="B60" s="34" t="inlineStr">
         <is>
           <t>WSTG-SESS-01</t>
         </is>
       </c>
-      <c r="C61" s="15">
+      <c r="C60" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/01-Testing_for_Session_Management_Schema", "Testing for Session Management Schema")</f>
         <v/>
       </c>
-      <c r="D61" s="16" t="inlineStr">
+      <c r="D60" s="16" t="inlineStr">
         <is>
           <t>- Gather session tokens, for the same user and for different users where possible.
 - Analyze and ensure that enough randomness exists to stop session forging attacks.
 - Modify cookies that are not signed and contain information that can be manipulated.</t>
         </is>
       </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F60" s="18" t="n"/>
+    </row>
+    <row r="61" ht="33" customHeight="1" s="82">
+      <c r="A61" s="19" t="n"/>
+      <c r="B61" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-SESS-02</t>
+        </is>
+      </c>
+      <c r="C61" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/02-Testing_for_Cookies_Attributes", "Testing for Cookies Attributes")</f>
+        <v/>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>- Ensure that the proper security configuration is set for cookies.</t>
+        </is>
+      </c>
       <c r="E61" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2813,16 +2813,17 @@
       <c r="A62" s="19" t="n"/>
       <c r="B62" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-02</t>
+          <t>WSTG-SESS-03</t>
         </is>
       </c>
       <c r="C62" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/02-Testing_for_Cookies_Attributes", "Testing for Cookies Attributes")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/03-Testing_for_Session_Fixation", "Testing for Session Fixation")</f>
         <v/>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>- Ensure that the proper security configuration is set for cookies.</t>
+          <t>- Analyze the authentication mechanism and its flow.
+- Force cookies and assess the impact.</t>
         </is>
       </c>
       <c r="E62" s="18" t="inlineStr">
@@ -2832,48 +2833,47 @@
       </c>
       <c r="F62" s="18" t="n"/>
     </row>
-    <row r="63" ht="33" customHeight="1" s="82">
+    <row r="63" ht="49.5" customHeight="1" s="82">
       <c r="A63" s="19" t="n"/>
       <c r="B63" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-03</t>
+          <t>WSTG-SESS-04</t>
         </is>
       </c>
       <c r="C63" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/03-Testing_for_Session_Fixation", "Testing for Session Fixation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/04-Testing_for_Exposed_Session_Variables", "Testing for Exposed Session Variables")</f>
         <v/>
       </c>
       <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>- Analyze the authentication mechanism and its flow.
-- Force cookies and assess the impact.</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F63" s="18" t="n"/>
-    </row>
-    <row r="64" ht="49.5" customHeight="1" s="82">
-      <c r="A64" s="19" t="n"/>
-      <c r="B64" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-04</t>
-        </is>
-      </c>
-      <c r="C64" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/04-Testing_for_Exposed_Session_Variables", "Testing for Exposed Session Variables")</f>
-        <v/>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>- Ensure that proper encryption is implemented.
 - Review the caching configuration.
 - Assess the channel and methods' security.</t>
         </is>
       </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="n"/>
+    </row>
+    <row r="64" ht="33" customHeight="1" s="82">
+      <c r="A64" s="19" t="n"/>
+      <c r="B64" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-SESS-05</t>
+        </is>
+      </c>
+      <c r="C64" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/05-Testing_for_Cross_Site_Request_Forgery", "Testing for Cross Site Request Forgery")</f>
+        <v/>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
+        </is>
+      </c>
       <c r="E64" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -2881,20 +2881,21 @@
       </c>
       <c r="F64" s="18" t="n"/>
     </row>
-    <row r="65" ht="33" customHeight="1" s="82">
+    <row r="65" ht="49.5" customHeight="1" s="82">
       <c r="A65" s="19" t="n"/>
       <c r="B65" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-05</t>
+          <t>WSTG-SESS-06</t>
         </is>
       </c>
       <c r="C65" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/05-Testing_for_Cross_Site_Request_Forgery", "Testing for Cross Site Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/06-Testing_for_Logout_Functionality", "Testing for Logout Functionality")</f>
         <v/>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether it is possible to initiate requests on a user's behalf that are not initiated by the user.</t>
+          <t>- Assess the logout UI.
+- Analyze the session timeout and if the session is properly killed after logout.</t>
         </is>
       </c>
       <c r="E65" s="18" t="inlineStr">
@@ -2904,21 +2905,20 @@
       </c>
       <c r="F65" s="18" t="n"/>
     </row>
-    <row r="66" ht="49.5" customHeight="1" s="82">
+    <row r="66" ht="16.5" customHeight="1" s="82">
       <c r="A66" s="19" t="n"/>
       <c r="B66" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-06</t>
+          <t>WSTG-SESS-07</t>
         </is>
       </c>
       <c r="C66" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/06-Testing_for_Logout_Functionality", "Testing for Logout Functionality")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/07-Testing_Session_Timeout", "Testing Session Timeout")</f>
         <v/>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>- Assess the logout UI.
-- Analyze the session timeout and if the session is properly killed after logout.</t>
+          <t>- Validate that a hard session timeout exists.</t>
         </is>
       </c>
       <c r="E66" s="18" t="inlineStr">
@@ -2928,20 +2928,21 @@
       </c>
       <c r="F66" s="18" t="n"/>
     </row>
-    <row r="67" ht="16.5" customHeight="1" s="82">
+    <row r="67" ht="33" customHeight="1" s="82">
       <c r="A67" s="19" t="n"/>
       <c r="B67" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-07</t>
+          <t>WSTG-SESS-08</t>
         </is>
       </c>
       <c r="C67" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/07-Testing_Session_Timeout", "Testing Session Timeout")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/08-Testing_for_Session_Puzzling", "Testing for Session Puzzling")</f>
         <v/>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>- Validate that a hard session timeout exists.</t>
+          <t>- Identify all session variables.
+- Break the logical flow of session generation.</t>
         </is>
       </c>
       <c r="E67" s="18" t="inlineStr">
@@ -2955,17 +2956,17 @@
       <c r="A68" s="19" t="n"/>
       <c r="B68" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-08</t>
+          <t>WSTG-SESS-09</t>
         </is>
       </c>
       <c r="C68" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/08-Testing_for_Session_Puzzling", "Testing for Session Puzzling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/09-Testing_for_Session_Hijacking", "Testing for Session Hijacking")</f>
         <v/>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>- Identify all session variables.
-- Break the logical flow of session generation.</t>
+          <t>- Identify vulnerable session cookies.
+- Hijack vulnerable cookies and assess the risk level.</t>
         </is>
       </c>
       <c r="E68" s="18" t="inlineStr">
@@ -2975,21 +2976,21 @@
       </c>
       <c r="F68" s="18" t="n"/>
     </row>
-    <row r="69" ht="33" customHeight="1" s="82">
+    <row r="69" ht="49.5" customHeight="1" s="82">
       <c r="A69" s="19" t="n"/>
       <c r="B69" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-09</t>
+          <t>WSTG-SESS-10</t>
         </is>
       </c>
       <c r="C69" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/09-Testing_for_Session_Hijacking", "Testing for Session Hijacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/10-Testing_JSON_Web_Tokens", "Testing JSON Web Tokens")</f>
         <v/>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>- Identify vulnerable session cookies.
-- Hijack vulnerable cookies and assess the risk level.</t>
+          <t>- Determine whether the JWTs expose sensitive information.
+- Determine whether the JWTs can be tampered with or modified.</t>
         </is>
       </c>
       <c r="E69" s="18" t="inlineStr">
@@ -3003,17 +3004,16 @@
       <c r="A70" s="19" t="n"/>
       <c r="B70" s="34" t="inlineStr">
         <is>
-          <t>WSTG-SESS-10</t>
+          <t>WSTG-SESS-11</t>
         </is>
       </c>
       <c r="C70" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/10-Testing_JSON_Web_Tokens", "Testing JSON Web Tokens")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/11-Testing_for_Concurrent_Sessions", "Testing for Concurrent Sessions")</f>
         <v/>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the JWTs expose sensitive information.
-- Determine whether the JWTs can be tampered with or modified.</t>
+          <t>- Evaluate the application's session management by assessing the handling of multiple active sessions for a single user account.</t>
         </is>
       </c>
       <c r="E70" s="18" t="inlineStr">
@@ -3023,79 +3023,80 @@
       </c>
       <c r="F70" s="18" t="n"/>
     </row>
-    <row r="71" ht="49.5" customHeight="1" s="82">
-      <c r="A71" s="19" t="n"/>
-      <c r="B71" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-SESS-11</t>
-        </is>
-      </c>
-      <c r="C71" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/11-Testing_for_Concurrent_Sessions", "Testing for Concurrent Sessions")</f>
-        <v/>
-      </c>
-      <c r="D71" s="16" t="inlineStr">
-        <is>
-          <t>- Evaluate the application's session management by assessing the handling of multiple active sessions for a single user account.</t>
-        </is>
-      </c>
-      <c r="E71" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F71" s="18" t="n"/>
-    </row>
-    <row r="72" ht="15" customHeight="1" s="82">
-      <c r="A72" s="97" t="n"/>
-      <c r="B72" s="98" t="n"/>
-      <c r="C72" s="99" t="n"/>
-      <c r="D72" s="99" t="n"/>
-      <c r="E72" s="99" t="n"/>
-      <c r="F72" s="99" t="n"/>
-    </row>
-    <row r="73" ht="47.25" customHeight="1" s="82">
-      <c r="A73" s="9" t="n"/>
-      <c r="B73" s="100" t="inlineStr">
+    <row r="71" ht="15" customHeight="1" s="82">
+      <c r="A71" s="97" t="n"/>
+      <c r="B71" s="98" t="n"/>
+      <c r="C71" s="99" t="n"/>
+      <c r="D71" s="99" t="n"/>
+      <c r="E71" s="99" t="n"/>
+      <c r="F71" s="99" t="n"/>
+    </row>
+    <row r="72" ht="47.25" customHeight="1" s="82">
+      <c r="A72" s="9" t="n"/>
+      <c r="B72" s="100" t="inlineStr">
         <is>
           <t>Input Validation Testing</t>
         </is>
       </c>
-      <c r="C73" s="101" t="inlineStr">
+      <c r="C72" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D73" s="101" t="inlineStr">
+      <c r="D72" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E73" s="101" t="inlineStr">
+      <c r="E72" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F73" s="101" t="inlineStr">
+      <c r="F72" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="49.5" customHeight="1" s="82">
+    <row r="73" ht="49.5" customHeight="1" s="82">
+      <c r="A73" s="19" t="n"/>
+      <c r="B73" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-01</t>
+        </is>
+      </c>
+      <c r="C73" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <v/>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>- Identify variables that are reflected in responses.
+- Assess the input they accept and the encoding that gets applied on return (if any).</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="n"/>
+    </row>
+    <row r="74" ht="66" customHeight="1" s="82">
       <c r="A74" s="19" t="n"/>
       <c r="B74" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-01</t>
+          <t>WSTG-INPV-02</t>
         </is>
       </c>
       <c r="C74" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>- Identify variables that are reflected in responses.
+          <t>- Identify stored input that is reflected on the client-side.
 - Assess the input they accept and the encoding that gets applied on return (if any).</t>
         </is>
       </c>
@@ -3106,21 +3107,20 @@
       </c>
       <c r="F74" s="18" t="n"/>
     </row>
-    <row r="75" ht="66" customHeight="1" s="82">
+    <row r="75" ht="16.5" customHeight="1" s="82">
       <c r="A75" s="19" t="n"/>
       <c r="B75" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-02</t>
+          <t>WSTG-INPV-03</t>
         </is>
       </c>
       <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>- Identify stored input that is reflected on the client-side.
-- Assess the input they accept and the encoding that gets applied on return (if any).</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E75" s="18" t="inlineStr">
@@ -3130,20 +3130,21 @@
       </c>
       <c r="F75" s="18" t="n"/>
     </row>
-    <row r="76" ht="16.5" customHeight="1" s="82">
+    <row r="76" ht="49.5" customHeight="1" s="82">
       <c r="A76" s="19" t="n"/>
       <c r="B76" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-03</t>
+          <t>WSTG-INPV-04</t>
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>- Identify the backend and the parsing method used.
+- Assess injection points and try bypassing input filters using HPP.</t>
         </is>
       </c>
       <c r="E76" s="18" t="inlineStr">
@@ -3157,17 +3158,17 @@
       <c r="A77" s="19" t="n"/>
       <c r="B77" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-04</t>
+          <t>WSTG-INPV-05</t>
         </is>
       </c>
       <c r="C77" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
         <v/>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>- Identify the backend and the parsing method used.
-- Assess injection points and try bypassing input filters using HPP.</t>
+          <t>- Identify SQL injection points.
+- Assess the severity of the injection and the level of access that can be achieved through it.</t>
         </is>
       </c>
       <c r="E77" s="18" t="inlineStr">
@@ -3177,21 +3178,21 @@
       </c>
       <c r="F77" s="18" t="n"/>
     </row>
-    <row r="78" ht="49.5" customHeight="1" s="82">
+    <row r="78" ht="33" customHeight="1" s="82">
       <c r="A78" s="19" t="n"/>
       <c r="B78" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-05</t>
+          <t>WSTG-INPV-06</t>
         </is>
       </c>
       <c r="C78" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
         <v/>
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>- Identify SQL injection points.
-- Assess the severity of the injection and the level of access that can be achieved through it.</t>
+          <t>- Identify LDAP injection points.
+- Assess the severity of the injection.</t>
         </is>
       </c>
       <c r="E78" s="18" t="inlineStr">
@@ -3201,21 +3202,21 @@
       </c>
       <c r="F78" s="18" t="n"/>
     </row>
-    <row r="79" ht="33" customHeight="1" s="82">
+    <row r="79" ht="49.5" customHeight="1" s="82">
       <c r="A79" s="19" t="n"/>
       <c r="B79" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-06</t>
+          <t>WSTG-INPV-07</t>
         </is>
       </c>
       <c r="C79" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
         <v/>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>- Identify LDAP injection points.
-- Assess the severity of the injection.</t>
+          <t>- Identify XML injection points.
+- Assess the types of exploits that can be attained and their severities.</t>
         </is>
       </c>
       <c r="E79" s="18" t="inlineStr">
@@ -3225,21 +3226,21 @@
       </c>
       <c r="F79" s="18" t="n"/>
     </row>
-    <row r="80" ht="49.5" customHeight="1" s="82">
+    <row r="80" ht="33" customHeight="1" s="82">
       <c r="A80" s="19" t="n"/>
       <c r="B80" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-07</t>
+          <t>WSTG-INPV-08</t>
         </is>
       </c>
       <c r="C80" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
         <v/>
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>- Identify XML injection points.
-- Assess the types of exploits that can be attained and their severities.</t>
+          <t>- Identify SSI injection points.
+- Assess the severity of the injection.</t>
         </is>
       </c>
       <c r="E80" s="18" t="inlineStr">
@@ -3249,21 +3250,20 @@
       </c>
       <c r="F80" s="18" t="n"/>
     </row>
-    <row r="81" ht="33" customHeight="1" s="82">
+    <row r="81" ht="16.5" customHeight="1" s="82">
       <c r="A81" s="19" t="n"/>
       <c r="B81" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-08</t>
+          <t>WSTG-INPV-09</t>
         </is>
       </c>
       <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
         <v/>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>- Identify SSI injection points.
-- Assess the severity of the injection.</t>
+          <t>- Identify XPATH injection points.</t>
         </is>
       </c>
       <c r="E81" s="18" t="inlineStr">
@@ -3273,47 +3273,48 @@
       </c>
       <c r="F81" s="18" t="n"/>
     </row>
-    <row r="82" ht="16.5" customHeight="1" s="82">
+    <row r="82" ht="66" customHeight="1" s="82">
       <c r="A82" s="19" t="n"/>
       <c r="B82" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-09</t>
+          <t>WSTG-INPV-10</t>
         </is>
       </c>
       <c r="C82" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
         <v/>
       </c>
       <c r="D82" s="16" t="inlineStr">
-        <is>
-          <t>- Identify XPATH injection points.</t>
-        </is>
-      </c>
-      <c r="E82" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F82" s="18" t="n"/>
-    </row>
-    <row r="83" ht="66" customHeight="1" s="82">
-      <c r="A83" s="19" t="n"/>
-      <c r="B83" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-10</t>
-        </is>
-      </c>
-      <c r="C83" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
-        <v/>
-      </c>
-      <c r="D83" s="16" t="inlineStr">
         <is>
           <t>- Identify IMAP/SMTP injection points.
 - Understand the data flow and deployment structure of the system.
 - Assess the injection impacts.</t>
         </is>
       </c>
+      <c r="E82" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F82" s="18" t="n"/>
+    </row>
+    <row r="83" ht="49.5" customHeight="1" s="82">
+      <c r="A83" s="19" t="n"/>
+      <c r="B83" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-11</t>
+        </is>
+      </c>
+      <c r="C83" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <v/>
+      </c>
+      <c r="D83" s="16" t="inlineStr">
+        <is>
+          <t>- Identify injection points where you can inject code into the application.
+- Assess the injection severity.</t>
+        </is>
+      </c>
       <c r="E83" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3321,21 +3322,21 @@
       </c>
       <c r="F83" s="18" t="n"/>
     </row>
-    <row r="84" ht="49.5" customHeight="1" s="82">
+    <row r="84" ht="33" customHeight="1" s="82">
       <c r="A84" s="19" t="n"/>
       <c r="B84" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-11</t>
+          <t>WSTG-INPV-12</t>
         </is>
       </c>
       <c r="C84" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
         <v/>
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points where you can inject code into the application.
-- Assess the injection severity.</t>
+          <t>- Identify and assess command injection points.
+- Bypass special characters and OS commands filter.</t>
         </is>
       </c>
       <c r="E84" s="18" t="inlineStr">
@@ -3345,21 +3346,20 @@
       </c>
       <c r="F84" s="18" t="n"/>
     </row>
-    <row r="85" ht="33" customHeight="1" s="82">
+    <row r="85" ht="49.5" customHeight="1" s="82">
       <c r="A85" s="19" t="n"/>
       <c r="B85" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-12</t>
+          <t>WSTG-INPV-13</t>
         </is>
       </c>
       <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
         <v/>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>- Identify and assess command injection points.
-- Bypass special characters and OS commands filter.</t>
+          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
         </is>
       </c>
       <c r="E85" s="18" t="inlineStr">
@@ -3369,114 +3369,68 @@
       </c>
       <c r="F85" s="18" t="n"/>
     </row>
-    <row r="86" ht="16.5" customHeight="1" s="82">
+    <row r="86" ht="66" customHeight="1" s="82">
       <c r="A86" s="19" t="n"/>
       <c r="B86" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-13</t>
+          <t>WSTG-INPV-14</t>
         </is>
       </c>
       <c r="C86" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Buffer_Overflow", "Testing for Buffer Overflow")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
         <v/>
       </c>
       <c r="D86" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E86" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F86" s="18" t="n"/>
-    </row>
-    <row r="87" ht="49.5" customHeight="1" s="82">
-      <c r="A87" s="19" t="n"/>
-      <c r="B87" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-13</t>
-        </is>
-      </c>
-      <c r="C87" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
-        <v/>
-      </c>
-      <c r="D87" s="16" t="inlineStr">
-        <is>
-          <t>- Assess whether injecting format string conversion specifiers into user-controlled fields causes undesired behavior from the application.</t>
-        </is>
-      </c>
-      <c r="E87" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F87" s="18" t="n"/>
-    </row>
-    <row r="88" ht="66" customHeight="1" s="82">
-      <c r="A88" s="19" t="n"/>
-      <c r="B88" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-14</t>
-        </is>
-      </c>
-      <c r="C88" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
-        <v/>
-      </c>
-      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>- Identify injections that are stored and require a recall step to the stored injection.
 - Understand how a recall step could occur.
 - Set listeners or activate the recall step if possible.</t>
         </is>
       </c>
-      <c r="E88" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F88" s="18" t="n"/>
-    </row>
-    <row r="89" ht="115.5" customHeight="1" s="82">
-      <c r="A89" s="19" t="n"/>
-      <c r="B89" s="34" t="inlineStr">
+      <c r="E86" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F86" s="18" t="n"/>
+    </row>
+    <row r="87" ht="115.5" customHeight="1" s="82">
+      <c r="A87" s="19" t="n"/>
+      <c r="B87" s="34" t="inlineStr">
         <is>
           <t>WSTG-INPV-15</t>
         </is>
       </c>
-      <c r="C89" s="15">
+      <c r="C87" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
         <v/>
       </c>
-      <c r="D89" s="16" t="inlineStr">
+      <c r="D87" s="16" t="inlineStr">
         <is>
           <t>- Identify user-controlled input that is reflected into HTTP response headers.
 - Assess whether CR (`\r`) and LF (`\n`) characters can be injected into response headers.
 - Determine the potential impact of successful HTTP Response Splitting attacks, such as cache poisoning or client-side exploitation.</t>
         </is>
       </c>
-      <c r="E89" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F89" s="18" t="n"/>
-    </row>
-    <row r="90" ht="99" customHeight="1" s="82">
-      <c r="A90" s="19" t="n"/>
-      <c r="B90" s="34" t="inlineStr">
+      <c r="E87" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F87" s="18" t="n"/>
+    </row>
+    <row r="88" ht="99" customHeight="1" s="82">
+      <c r="A88" s="19" t="n"/>
+      <c r="B88" s="34" t="inlineStr">
         <is>
           <t>WSTG-INPV-16</t>
         </is>
       </c>
-      <c r="C90" s="15">
+      <c r="C88" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
         <v/>
       </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="D88" s="16" t="inlineStr">
         <is>
           <t>- Identify request boundary inconsistencies between frontend and backend components
 - Detect classic CL/TE desynchronization vulnerabilities
@@ -3485,6 +3439,55 @@
 - Confirm backend request queue poisoning</t>
         </is>
       </c>
+      <c r="E88" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F88" s="18" t="n"/>
+    </row>
+    <row r="89" ht="49.5" customHeight="1" s="82">
+      <c r="A89" s="19" t="n"/>
+      <c r="B89" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-17</t>
+        </is>
+      </c>
+      <c r="C89" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <v/>
+      </c>
+      <c r="D89" s="16" t="inlineStr">
+        <is>
+          <t>- Assess if the Host header is being parsed dynamically in the application.
+- Bypass security controls that rely on the header.</t>
+        </is>
+      </c>
+      <c r="E89" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F89" s="18" t="n"/>
+    </row>
+    <row r="90" ht="49.5" customHeight="1" s="82">
+      <c r="A90" s="19" t="n"/>
+      <c r="B90" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-18</t>
+        </is>
+      </c>
+      <c r="C90" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <v/>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>- Detect template injection vulnerability points.
+- Identify the templating engine.
+- Build the exploit.</t>
+        </is>
+      </c>
       <c r="E90" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3496,17 +3499,18 @@
       <c r="A91" s="19" t="n"/>
       <c r="B91" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-17</t>
+          <t>WSTG-INPV-19</t>
         </is>
       </c>
       <c r="C91" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
         <v/>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>- Assess if the Host header is being parsed dynamically in the application.
-- Bypass security controls that rely on the header.</t>
+          <t>- Identify SSRF injection points.
+- Test if the injection points are exploitable.
+- Asses the severity of the vulnerability.</t>
         </is>
       </c>
       <c r="E91" s="18" t="inlineStr">
@@ -3520,18 +3524,17 @@
       <c r="A92" s="19" t="n"/>
       <c r="B92" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-18</t>
+          <t>WSTG-INPV-20</t>
         </is>
       </c>
       <c r="C92" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
         <v/>
       </c>
       <c r="D92" s="16" t="inlineStr">
         <is>
-          <t>- Detect template injection vulnerability points.
-- Identify the templating engine.
-- Build the exploit.</t>
+          <t>- Identify requests that modify objects
+- Assess if it is possible to modify fields never intended to be modified from outside</t>
         </is>
       </c>
       <c r="E92" s="18" t="inlineStr">
@@ -3541,67 +3544,18 @@
       </c>
       <c r="F92" s="18" t="n"/>
     </row>
-    <row r="93" ht="49.5" customHeight="1" s="82">
+    <row r="93" ht="181.5" customHeight="1" s="82">
       <c r="A93" s="19" t="n"/>
       <c r="B93" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-19</t>
+          <t>WSTG-INPV-21</t>
         </is>
       </c>
       <c r="C93" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
         <v/>
       </c>
       <c r="D93" s="16" t="inlineStr">
-        <is>
-          <t>- Identify SSRF injection points.
-- Test if the injection points are exploitable.
-- Asses the severity of the vulnerability.</t>
-        </is>
-      </c>
-      <c r="E93" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F93" s="18" t="n"/>
-    </row>
-    <row r="94" ht="49.5" customHeight="1" s="82">
-      <c r="A94" s="19" t="n"/>
-      <c r="B94" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-20</t>
-        </is>
-      </c>
-      <c r="C94" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
-        <v/>
-      </c>
-      <c r="D94" s="16" t="inlineStr">
-        <is>
-          <t>- Identify requests that modify objects
-- Assess if it is possible to modify fields never intended to be modified from outside</t>
-        </is>
-      </c>
-      <c r="E94" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F94" s="18" t="n"/>
-    </row>
-    <row r="95" ht="181.5" customHeight="1" s="82">
-      <c r="A95" s="19" t="n"/>
-      <c r="B95" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-INPV-21</t>
-        </is>
-      </c>
-      <c r="C95" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
-        <v/>
-      </c>
-      <c r="D95" s="16" t="inlineStr">
         <is>
           <t>- Identify CSV/spreadsheet export features that include untrusted input.
 - Verify whether attacker-controlled values are interpreted as formulas when the export is opened in common spreadsheet applications.
@@ -3610,150 +3564,198 @@
 - Assess practical impact based on who opens the export and how it is used.</t>
         </is>
       </c>
-      <c r="E95" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F95" s="18" t="n"/>
-    </row>
-    <row r="96" ht="15" customHeight="1" s="82">
-      <c r="A96" s="97" t="n"/>
-      <c r="B96" s="98" t="n"/>
-      <c r="C96" s="99" t="n"/>
-      <c r="D96" s="99" t="n"/>
-      <c r="E96" s="99" t="n"/>
-      <c r="F96" s="99" t="n"/>
-    </row>
-    <row r="97" ht="47.25" customHeight="1" s="82">
-      <c r="A97" s="9" t="n"/>
-      <c r="B97" s="100" t="inlineStr">
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F93" s="18" t="n"/>
+    </row>
+    <row r="94" ht="15" customHeight="1" s="82">
+      <c r="A94" s="97" t="n"/>
+      <c r="B94" s="98" t="n"/>
+      <c r="C94" s="99" t="n"/>
+      <c r="D94" s="99" t="n"/>
+      <c r="E94" s="99" t="n"/>
+      <c r="F94" s="99" t="n"/>
+    </row>
+    <row r="95" ht="47.25" customHeight="1" s="82">
+      <c r="A95" s="9" t="n"/>
+      <c r="B95" s="100" t="inlineStr">
         <is>
           <t>Testing for Error Handling</t>
         </is>
       </c>
-      <c r="C97" s="101" t="inlineStr">
+      <c r="C95" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D97" s="101" t="inlineStr">
+      <c r="D95" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E97" s="101" t="inlineStr">
+      <c r="E95" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F97" s="101" t="inlineStr">
+      <c r="F95" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="33" customHeight="1" s="82">
-      <c r="A98" s="19" t="n"/>
-      <c r="B98" s="34" t="inlineStr">
+    <row r="96" ht="33" customHeight="1" s="82">
+      <c r="A96" s="19" t="n"/>
+      <c r="B96" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C98" s="15">
+      <c r="C96" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D96" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="n"/>
-    </row>
-    <row r="99" ht="16.5" customHeight="1" s="82">
-      <c r="A99" s="19" t="n"/>
-      <c r="B99" s="34" t="inlineStr">
+      <c r="E96" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F96" s="18" t="n"/>
+    </row>
+    <row r="97" ht="16.5" customHeight="1" s="82">
+      <c r="A97" s="19" t="n"/>
+      <c r="B97" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C99" s="15">
+      <c r="C97" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
         <v/>
       </c>
-      <c r="D99" s="16" t="inlineStr">
+      <c r="D97" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E99" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F99" s="18" t="n"/>
-    </row>
-    <row r="100" ht="15" customHeight="1" s="82">
-      <c r="A100" s="97" t="n"/>
-      <c r="B100" s="98" t="n"/>
-      <c r="C100" s="99" t="n"/>
-      <c r="D100" s="99" t="n"/>
-      <c r="E100" s="99" t="n"/>
-      <c r="F100" s="99" t="n"/>
-    </row>
-    <row r="101" ht="47.25" customHeight="1" s="82">
-      <c r="A101" s="9" t="n"/>
-      <c r="B101" s="100" t="inlineStr">
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="n"/>
+    </row>
+    <row r="98" ht="15" customHeight="1" s="82">
+      <c r="A98" s="97" t="n"/>
+      <c r="B98" s="98" t="n"/>
+      <c r="C98" s="99" t="n"/>
+      <c r="D98" s="99" t="n"/>
+      <c r="E98" s="99" t="n"/>
+      <c r="F98" s="99" t="n"/>
+    </row>
+    <row r="99" ht="47.25" customHeight="1" s="82">
+      <c r="A99" s="9" t="n"/>
+      <c r="B99" s="100" t="inlineStr">
         <is>
           <t>Testing for Weak Cryptography</t>
         </is>
       </c>
-      <c r="C101" s="101" t="inlineStr">
+      <c r="C99" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D101" s="101" t="inlineStr">
+      <c r="D99" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E101" s="101" t="inlineStr">
+      <c r="E99" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F101" s="101" t="inlineStr">
+      <c r="F99" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="82.5" customHeight="1" s="82">
-      <c r="A102" s="19" t="n"/>
-      <c r="B102" s="34" t="inlineStr">
+    <row r="100" ht="82.5" customHeight="1" s="82">
+      <c r="A100" s="19" t="n"/>
+      <c r="B100" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C102" s="15">
+      <c r="C100" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D100" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
+      <c r="E100" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F100" s="18" t="n"/>
+    </row>
+    <row r="101" ht="49.5" customHeight="1" s="82">
+      <c r="A101" s="19" t="n"/>
+      <c r="B101" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C101" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F101" s="18" t="n"/>
+    </row>
+    <row r="102" ht="49.5" customHeight="1" s="82">
+      <c r="A102" s="19" t="n"/>
+      <c r="B102" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CRYP-03</t>
+        </is>
+      </c>
+      <c r="C102" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
+        <v/>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sensitive information transmitted through the various channels.
+- Assess the privacy and security of the channels used.</t>
+        </is>
+      </c>
       <c r="E102" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3761,21 +3763,20 @@
       </c>
       <c r="F102" s="18" t="n"/>
     </row>
-    <row r="103" ht="49.5" customHeight="1" s="82">
+    <row r="103" ht="33" customHeight="1" s="82">
       <c r="A103" s="19" t="n"/>
       <c r="B103" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CRYP-02</t>
+          <t>WSTG-CRYP-04</t>
         </is>
       </c>
       <c r="C103" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+          <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
       <c r="E103" s="18" t="inlineStr">
@@ -3785,150 +3786,103 @@
       </c>
       <c r="F103" s="18" t="n"/>
     </row>
-    <row r="104" ht="49.5" customHeight="1" s="82">
-      <c r="A104" s="19" t="n"/>
-      <c r="B104" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-03</t>
-        </is>
-      </c>
-      <c r="C104" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
-        <v/>
-      </c>
-      <c r="D104" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sensitive information transmitted through the various channels.
-- Assess the privacy and security of the channels used.</t>
-        </is>
-      </c>
-      <c r="E104" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F104" s="18" t="n"/>
-    </row>
-    <row r="105" ht="33" customHeight="1" s="82">
-      <c r="A105" s="19" t="n"/>
-      <c r="B105" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-04</t>
-        </is>
-      </c>
-      <c r="C105" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
-        <v/>
-      </c>
-      <c r="D105" s="16" t="inlineStr">
-        <is>
-          <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
-        </is>
-      </c>
-      <c r="E105" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F105" s="18" t="n"/>
-    </row>
-    <row r="106" ht="15" customHeight="1" s="82">
-      <c r="A106" s="97" t="n"/>
-      <c r="B106" s="98" t="n"/>
-      <c r="C106" s="99" t="n"/>
-      <c r="D106" s="99" t="n"/>
-      <c r="E106" s="99" t="n"/>
-      <c r="F106" s="99" t="n"/>
-    </row>
-    <row r="107" ht="47.25" customHeight="1" s="82">
-      <c r="A107" s="9" t="n"/>
-      <c r="B107" s="100" t="inlineStr">
+    <row r="104" ht="15" customHeight="1" s="82">
+      <c r="A104" s="97" t="n"/>
+      <c r="B104" s="98" t="n"/>
+      <c r="C104" s="99" t="n"/>
+      <c r="D104" s="99" t="n"/>
+      <c r="E104" s="99" t="n"/>
+      <c r="F104" s="99" t="n"/>
+    </row>
+    <row r="105" ht="47.25" customHeight="1" s="82">
+      <c r="A105" s="9" t="n"/>
+      <c r="B105" s="100" t="inlineStr">
         <is>
           <t>Business Logic Testing</t>
         </is>
       </c>
-      <c r="C107" s="101" t="inlineStr">
+      <c r="C105" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D107" s="101" t="inlineStr">
+      <c r="D105" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E107" s="101" t="inlineStr">
+      <c r="E105" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F107" s="101" t="inlineStr">
+      <c r="F105" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="108" ht="82.5" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+    <row r="106" ht="82.5" customHeight="1" s="82">
+      <c r="A106" s="19" t="n"/>
+      <c r="B106" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C106" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D106" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="66" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E106" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F106" s="18" t="n"/>
+    </row>
+    <row r="107" ht="66" customHeight="1" s="82">
+      <c r="A107" s="19" t="n"/>
+      <c r="B107" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C107" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D107" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="148.5" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="n"/>
+    </row>
+    <row r="108" ht="148.5" customHeight="1" s="82">
+      <c r="A108" s="19" t="n"/>
+      <c r="B108" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C108" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3936,6 +3890,54 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="n"/>
+    </row>
+    <row r="109" ht="49.5" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-BUSL-04</t>
+        </is>
+      </c>
+      <c r="C109" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
+        <v/>
+      </c>
+      <c r="D109" s="16" t="inlineStr">
+        <is>
+          <t>- Review the project documentation for system functionality that may be impacted by time.
+- Develop and execute misuse cases.</t>
+        </is>
+      </c>
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="66" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-BUSL-05</t>
+        </is>
+      </c>
+      <c r="C110" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
+        <v/>
+      </c>
+      <c r="D110" s="16" t="inlineStr">
+        <is>
+          <t>- Identify functions that must set limits to the times they can be called.
+- Assess if there is a logical limit set on the functions and if it is properly validated.</t>
+        </is>
+      </c>
       <c r="E110" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3943,21 +3945,21 @@
       </c>
       <c r="F110" s="18" t="n"/>
     </row>
-    <row r="111" ht="49.5" customHeight="1" s="82">
+    <row r="111" ht="82.5" customHeight="1" s="82">
       <c r="A111" s="19" t="n"/>
       <c r="B111" s="34" t="inlineStr">
         <is>
-          <t>WSTG-BUSL-04</t>
+          <t>WSTG-BUSL-06</t>
         </is>
       </c>
       <c r="C111" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
         <v/>
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>- Review the project documentation for system functionality that may be impacted by time.
-- Develop and execute misuse cases.</t>
+          <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
+- Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
       <c r="E111" s="18" t="inlineStr">
@@ -3967,116 +3969,68 @@
       </c>
       <c r="F111" s="18" t="n"/>
     </row>
-    <row r="112" ht="66" customHeight="1" s="82">
+    <row r="112" ht="99" customHeight="1" s="82">
       <c r="A112" s="19" t="n"/>
       <c r="B112" s="34" t="inlineStr">
         <is>
-          <t>WSTG-BUSL-05</t>
+          <t>WSTG-BUSL-07</t>
         </is>
       </c>
       <c r="C112" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
         <v/>
       </c>
       <c r="D112" s="16" t="inlineStr">
-        <is>
-          <t>- Identify functions that must set limits to the times they can be called.
-- Assess if there is a logical limit set on the functions and if it is properly validated.</t>
-        </is>
-      </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="82.5" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-BUSL-06</t>
-        </is>
-      </c>
-      <c r="C113" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
-        <v/>
-      </c>
-      <c r="D113" s="16" t="inlineStr">
-        <is>
-          <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
-- Develop a misuse case and try to circumvent every logic flow identified.</t>
-        </is>
-      </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="99" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-BUSL-07</t>
-        </is>
-      </c>
-      <c r="C114" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
-        <v/>
-      </c>
-      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="99" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="99" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="165" customHeight="1" s="82">
-      <c r="A116" s="19" t="n"/>
-      <c r="B116" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="165" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C116" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D116" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4086,89 +4040,135 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F116" s="18" t="n"/>
-    </row>
-    <row r="117" ht="66" customHeight="1" s="82">
-      <c r="A117" s="19" t="n"/>
-      <c r="B117" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="66" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C117" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D117" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E117" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F117" s="18" t="n"/>
-    </row>
-    <row r="118" ht="15" customHeight="1" s="82">
-      <c r="A118" s="97" t="n"/>
-      <c r="B118" s="98" t="n"/>
-      <c r="C118" s="99" t="n"/>
-      <c r="D118" s="99" t="n"/>
-      <c r="E118" s="99" t="n"/>
-      <c r="F118" s="99" t="n"/>
-    </row>
-    <row r="119" ht="47.25" customHeight="1" s="82">
-      <c r="A119" s="9" t="n"/>
-      <c r="B119" s="100" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="15" customHeight="1" s="82">
+      <c r="A116" s="97" t="n"/>
+      <c r="B116" s="98" t="n"/>
+      <c r="C116" s="99" t="n"/>
+      <c r="D116" s="99" t="n"/>
+      <c r="E116" s="99" t="n"/>
+      <c r="F116" s="99" t="n"/>
+    </row>
+    <row r="117" ht="47.25" customHeight="1" s="82">
+      <c r="A117" s="9" t="n"/>
+      <c r="B117" s="100" t="inlineStr">
         <is>
           <t>Client-side Testing</t>
         </is>
       </c>
-      <c r="C119" s="101" t="inlineStr">
+      <c r="C117" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D119" s="101" t="inlineStr">
+      <c r="D117" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E119" s="101" t="inlineStr">
+      <c r="E117" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F119" s="101" t="inlineStr">
+      <c r="F117" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
+    </row>
+    <row r="118" ht="33" customHeight="1" s="82">
+      <c r="A118" s="19" t="n"/>
+      <c r="B118" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CLNT-01</t>
+        </is>
+      </c>
+      <c r="C118" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
+        <v/>
+      </c>
+      <c r="D118" s="16" t="inlineStr">
+        <is>
+          <t>- Identify DOM sinks.
+- Build payloads that pertain to every sink type.</t>
+        </is>
+      </c>
+      <c r="E118" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F118" s="18" t="n"/>
+    </row>
+    <row r="119" ht="16.5" customHeight="1" s="82">
+      <c r="A119" s="19" t="n"/>
+      <c r="B119" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-CLNT-02</t>
+        </is>
+      </c>
+      <c r="C119" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
+        <v/>
+      </c>
+      <c r="D119" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
+        </is>
+      </c>
+      <c r="E119" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F119" s="18" t="n"/>
     </row>
     <row r="120" ht="33" customHeight="1" s="82">
       <c r="A120" s="19" t="n"/>
       <c r="B120" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-01</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
         <v/>
       </c>
       <c r="D120" s="16" t="inlineStr">
         <is>
-          <t>- Identify DOM sinks.
-- Build payloads that pertain to every sink type.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E120" s="18" t="inlineStr">
@@ -4178,20 +4178,21 @@
       </c>
       <c r="F120" s="18" t="n"/>
     </row>
-    <row r="121" ht="16.5" customHeight="1" s="82">
+    <row r="121" ht="33" customHeight="1" s="82">
       <c r="A121" s="19" t="n"/>
       <c r="B121" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-02</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr">
@@ -4205,16 +4206,17 @@
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4228,17 +4230,17 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-06</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4252,17 +4254,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-07</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify endpoints that implement CORS.
+- Ensure that the CORS configuration is secure or harmless.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4276,17 +4278,17 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-08</t>
         </is>
       </c>
       <c r="C125" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
         <v/>
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Decompile and analyze the application's code.
+- Assess sinks inputs and unsafe method usages.</t>
         </is>
       </c>
       <c r="E125" s="18" t="inlineStr">
@@ -4296,21 +4298,20 @@
       </c>
       <c r="F125" s="18" t="n"/>
     </row>
-    <row r="126" ht="33" customHeight="1" s="82">
+    <row r="126" ht="16.5" customHeight="1" s="82">
       <c r="A126" s="19" t="n"/>
       <c r="B126" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-07</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D126" s="16" t="inlineStr">
         <is>
-          <t>- Identify endpoints that implement CORS.
-- Ensure that the CORS configuration is secure or harmless.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E126" s="18" t="inlineStr">
@@ -4320,21 +4321,21 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="33" customHeight="1" s="82">
+    <row r="127" ht="49.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-08</t>
+          <t>WSTG-CLNT-10</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Decompile and analyze the application's code.
-- Assess sinks inputs and unsafe method usages.</t>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4344,20 +4345,21 @@
       </c>
       <c r="F127" s="18" t="n"/>
     </row>
-    <row r="128" ht="16.5" customHeight="1" s="82">
+    <row r="128" ht="49.5" customHeight="1" s="82">
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-09</t>
+          <t>WSTG-CLNT-11</t>
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
         <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
+          <t>- Assess the security of the message's origin.
+- Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
       <c r="E128" s="18" t="inlineStr">
@@ -4367,21 +4369,21 @@
       </c>
       <c r="F128" s="18" t="n"/>
     </row>
-    <row r="129" ht="49.5" customHeight="1" s="82">
+    <row r="129" ht="82.5" customHeight="1" s="82">
       <c r="A129" s="19" t="n"/>
       <c r="B129" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-12</t>
         </is>
       </c>
       <c r="C129" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Determine whether the site is storing sensitive data in client-side storage.
+- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
       <c r="E129" s="18" t="inlineStr">
@@ -4395,17 +4397,17 @@
       <c r="A130" s="19" t="n"/>
       <c r="B130" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-11</t>
+          <t>WSTG-CLNT-13</t>
         </is>
       </c>
       <c r="C130" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
       <c r="D130" s="16" t="inlineStr">
         <is>
-          <t>- Assess the security of the message's origin.
-- Validate that it's using safe methods and validating its input.</t>
+          <t>- Locate sensitive data across the system.
+- Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
       <c r="E130" s="18" t="inlineStr">
@@ -4415,21 +4417,20 @@
       </c>
       <c r="F130" s="18" t="n"/>
     </row>
-    <row r="131" ht="82.5" customHeight="1" s="82">
+    <row r="131" ht="16.5" customHeight="1" s="82">
       <c r="A131" s="19" t="n"/>
       <c r="B131" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-12</t>
+          <t>WSTG-CLNT-14</t>
         </is>
       </c>
       <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
         <v/>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the site is storing sensitive data in client-side storage.
-- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E131" s="18" t="inlineStr">
@@ -4439,242 +4440,195 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="49.5" customHeight="1" s="82">
+    <row r="132" ht="99" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-13</t>
+          <t>WSTG-CLNT-15</t>
         </is>
       </c>
       <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
       <c r="D132" s="16" t="inlineStr">
-        <is>
-          <t>- Locate sensitive data across the system.
-- Assess the leakage of sensitive data through various techniques.</t>
-        </is>
-      </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="16.5" customHeight="1" s="82">
-      <c r="A133" s="19" t="n"/>
-      <c r="B133" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C133" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D133" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F133" s="18" t="n"/>
-    </row>
-    <row r="134" ht="99" customHeight="1" s="82">
-      <c r="A134" s="19" t="n"/>
-      <c r="B134" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-15</t>
-        </is>
-      </c>
-      <c r="C134" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
-        <v/>
-      </c>
-      <c r="D134" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E134" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F134" s="18" t="n"/>
-    </row>
-    <row r="135" ht="15" customHeight="1" s="82">
-      <c r="A135" s="97" t="n"/>
-      <c r="B135" s="98" t="n"/>
-      <c r="C135" s="99" t="n"/>
-      <c r="D135" s="99" t="n"/>
-      <c r="E135" s="99" t="n"/>
-      <c r="F135" s="99" t="n"/>
-    </row>
-    <row r="136" ht="47.25" customHeight="1" s="82">
-      <c r="A136" s="9" t="n"/>
-      <c r="B136" s="100" t="inlineStr">
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="15" customHeight="1" s="82">
+      <c r="A133" s="97" t="n"/>
+      <c r="B133" s="98" t="n"/>
+      <c r="C133" s="99" t="n"/>
+      <c r="D133" s="99" t="n"/>
+      <c r="E133" s="99" t="n"/>
+      <c r="F133" s="99" t="n"/>
+    </row>
+    <row r="134" ht="47.25" customHeight="1" s="82">
+      <c r="A134" s="9" t="n"/>
+      <c r="B134" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C136" s="101" t="inlineStr">
+      <c r="C134" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D136" s="101" t="inlineStr">
+      <c r="D134" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E136" s="101" t="inlineStr">
+      <c r="E134" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F136" s="101" t="inlineStr">
+      <c r="F134" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="99" customHeight="1" s="82">
-      <c r="A137" s="19" t="n"/>
-      <c r="B137" s="34" t="inlineStr">
+    <row r="135" ht="99" customHeight="1" s="82">
+      <c r="A135" s="19" t="n"/>
+      <c r="B135" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C137" s="15">
+      <c r="C135" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D135" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="66" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
+      <c r="E135" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F135" s="18" t="n"/>
+    </row>
+    <row r="136" ht="66" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-02</t>
         </is>
       </c>
-      <c r="C138" s="15">
+      <c r="C136" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
         <v/>
       </c>
-      <c r="D138" s="16" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
         </is>
       </c>
-      <c r="E138" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F138" s="18" t="n"/>
-    </row>
-    <row r="139" ht="132" customHeight="1" s="82">
-      <c r="A139" s="19" t="n"/>
-      <c r="B139" s="34" t="inlineStr">
+      <c r="E136" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F136" s="18" t="n"/>
+    </row>
+    <row r="137" ht="132" customHeight="1" s="82">
+      <c r="A137" s="19" t="n"/>
+      <c r="B137" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C137" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D137" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="82.5" customHeight="1" s="82">
-      <c r="A140" s="19" t="n"/>
-      <c r="B140" s="34" t="inlineStr">
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="82.5" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C140" s="15">
+      <c r="C138" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
         <v/>
       </c>
-      <c r="D140" s="16" t="inlineStr">
+      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="66" customHeight="1" s="82">
-      <c r="A141" s="19" t="n"/>
-      <c r="B141" s="34" t="inlineStr">
+      <c r="E138" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F138" s="18" t="n"/>
+    </row>
+    <row r="139" ht="66" customHeight="1" s="82">
+      <c r="A139" s="19" t="n"/>
+      <c r="B139" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C141" s="15">
+      <c r="C139" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D141" s="16" t="inlineStr">
+      <c r="D139" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E141" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F141" s="18" t="n"/>
-    </row>
-    <row r="142" ht="15" customHeight="1" s="82">
-      <c r="A142" s="97" t="n"/>
-      <c r="B142" s="98" t="n"/>
-      <c r="C142" s="99" t="n"/>
-      <c r="D142" s="99" t="n"/>
-      <c r="E142" s="99" t="n"/>
-      <c r="F142" s="99" t="n"/>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="15" customHeight="1" s="82">
+      <c r="A140" s="97" t="n"/>
+      <c r="B140" s="98" t="n"/>
+      <c r="C140" s="99" t="n"/>
+      <c r="D140" s="99" t="n"/>
+      <c r="E140" s="99" t="n"/>
+      <c r="F140" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4691,7 +4645,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F142">
+  <conditionalFormatting sqref="B4:F140">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4703,7 +4657,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E31 E34 E35 E36 E37 E38 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E51 E54 E55 E56 E57 E58 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E71 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E134 E137 E138 E139 E140 E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E96 E97 E100 E101 E102 E103 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-06-30
Updates based on OWASP/wstg@b87d2b2
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3571,167 +3571,168 @@
       </c>
       <c r="F93" s="18" t="n"/>
     </row>
-    <row r="94" ht="15" customHeight="1" s="82">
-      <c r="A94" s="97" t="n"/>
-      <c r="B94" s="98" t="n"/>
-      <c r="C94" s="99" t="n"/>
-      <c r="D94" s="99" t="n"/>
-      <c r="E94" s="99" t="n"/>
-      <c r="F94" s="99" t="n"/>
-    </row>
-    <row r="95" ht="47.25" customHeight="1" s="82">
-      <c r="A95" s="9" t="n"/>
-      <c r="B95" s="100" t="inlineStr">
+    <row r="94" ht="99" customHeight="1" s="82">
+      <c r="A94" s="19" t="n"/>
+      <c r="B94" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-22</t>
+        </is>
+      </c>
+      <c r="C94" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
+        <v/>
+      </c>
+      <c r="D94" s="16" t="inlineStr">
+        <is>
+          <t>- Identify functions and libraries that recursively merge, clone, or assign user-controlled properties.
+- Determine whether user input can reach and modify `Object.prototype`.
+- Identify gadgets that turn prototype pollution into a concrete impact.</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="n"/>
+    </row>
+    <row r="95" ht="15" customHeight="1" s="82">
+      <c r="A95" s="97" t="n"/>
+      <c r="B95" s="98" t="n"/>
+      <c r="C95" s="99" t="n"/>
+      <c r="D95" s="99" t="n"/>
+      <c r="E95" s="99" t="n"/>
+      <c r="F95" s="99" t="n"/>
+    </row>
+    <row r="96" ht="47.25" customHeight="1" s="82">
+      <c r="A96" s="9" t="n"/>
+      <c r="B96" s="100" t="inlineStr">
         <is>
           <t>Testing for Error Handling</t>
         </is>
       </c>
-      <c r="C95" s="101" t="inlineStr">
+      <c r="C96" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D95" s="101" t="inlineStr">
+      <c r="D96" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E95" s="101" t="inlineStr">
+      <c r="E96" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F95" s="101" t="inlineStr">
+      <c r="F96" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="33" customHeight="1" s="82">
-      <c r="A96" s="19" t="n"/>
-      <c r="B96" s="34" t="inlineStr">
+    <row r="97" ht="33" customHeight="1" s="82">
+      <c r="A97" s="19" t="n"/>
+      <c r="B97" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C96" s="15">
+      <c r="C97" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D96" s="16" t="inlineStr">
+      <c r="D97" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E96" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F96" s="18" t="n"/>
-    </row>
-    <row r="97" ht="16.5" customHeight="1" s="82">
-      <c r="A97" s="19" t="n"/>
-      <c r="B97" s="34" t="inlineStr">
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="n"/>
+    </row>
+    <row r="98" ht="16.5" customHeight="1" s="82">
+      <c r="A98" s="19" t="n"/>
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C97" s="15">
+      <c r="C98" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
         <v/>
       </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="D98" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E97" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F97" s="18" t="n"/>
-    </row>
-    <row r="98" ht="15" customHeight="1" s="82">
-      <c r="A98" s="97" t="n"/>
-      <c r="B98" s="98" t="n"/>
-      <c r="C98" s="99" t="n"/>
-      <c r="D98" s="99" t="n"/>
-      <c r="E98" s="99" t="n"/>
-      <c r="F98" s="99" t="n"/>
-    </row>
-    <row r="99" ht="47.25" customHeight="1" s="82">
-      <c r="A99" s="9" t="n"/>
-      <c r="B99" s="100" t="inlineStr">
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="n"/>
+    </row>
+    <row r="99" ht="15" customHeight="1" s="82">
+      <c r="A99" s="97" t="n"/>
+      <c r="B99" s="98" t="n"/>
+      <c r="C99" s="99" t="n"/>
+      <c r="D99" s="99" t="n"/>
+      <c r="E99" s="99" t="n"/>
+      <c r="F99" s="99" t="n"/>
+    </row>
+    <row r="100" ht="47.25" customHeight="1" s="82">
+      <c r="A100" s="9" t="n"/>
+      <c r="B100" s="100" t="inlineStr">
         <is>
           <t>Testing for Weak Cryptography</t>
         </is>
       </c>
-      <c r="C99" s="101" t="inlineStr">
+      <c r="C100" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D99" s="101" t="inlineStr">
+      <c r="D100" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E99" s="101" t="inlineStr">
+      <c r="E100" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F99" s="101" t="inlineStr">
+      <c r="F100" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="82.5" customHeight="1" s="82">
-      <c r="A100" s="19" t="n"/>
-      <c r="B100" s="34" t="inlineStr">
+    <row r="101" ht="82.5" customHeight="1" s="82">
+      <c r="A101" s="19" t="n"/>
+      <c r="B101" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C100" s="15">
+      <c r="C101" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D100" s="16" t="inlineStr">
+      <c r="D101" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
-      <c r="E100" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F100" s="18" t="n"/>
-    </row>
-    <row r="101" ht="49.5" customHeight="1" s="82">
-      <c r="A101" s="19" t="n"/>
-      <c r="B101" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-02</t>
-        </is>
-      </c>
-      <c r="C101" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
-        <v/>
-      </c>
-      <c r="D101" s="16" t="inlineStr">
-        <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
-        </is>
-      </c>
       <c r="E101" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3743,146 +3744,170 @@
       <c r="A102" s="19" t="n"/>
       <c r="B102" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C102" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="n"/>
+    </row>
+    <row r="103" ht="49.5" customHeight="1" s="82">
+      <c r="A103" s="19" t="n"/>
+      <c r="B103" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CRYP-03</t>
         </is>
       </c>
-      <c r="C102" s="15">
+      <c r="C103" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D103" s="16" t="inlineStr">
         <is>
           <t>- Identify sensitive information transmitted through the various channels.
 - Assess the privacy and security of the channels used.</t>
         </is>
       </c>
-      <c r="E102" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F102" s="18" t="n"/>
-    </row>
-    <row r="103" ht="33" customHeight="1" s="82">
-      <c r="A103" s="19" t="n"/>
-      <c r="B103" s="34" t="inlineStr">
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="n"/>
+    </row>
+    <row r="104" ht="33" customHeight="1" s="82">
+      <c r="A104" s="19" t="n"/>
+      <c r="B104" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-04</t>
         </is>
       </c>
-      <c r="C103" s="15">
+      <c r="C104" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
-      <c r="D103" s="16" t="inlineStr">
+      <c r="D104" s="16" t="inlineStr">
         <is>
           <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
-      <c r="E103" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F103" s="18" t="n"/>
-    </row>
-    <row r="104" ht="15" customHeight="1" s="82">
-      <c r="A104" s="97" t="n"/>
-      <c r="B104" s="98" t="n"/>
-      <c r="C104" s="99" t="n"/>
-      <c r="D104" s="99" t="n"/>
-      <c r="E104" s="99" t="n"/>
-      <c r="F104" s="99" t="n"/>
-    </row>
-    <row r="105" ht="47.25" customHeight="1" s="82">
-      <c r="A105" s="9" t="n"/>
-      <c r="B105" s="100" t="inlineStr">
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="n"/>
+    </row>
+    <row r="105" ht="15" customHeight="1" s="82">
+      <c r="A105" s="97" t="n"/>
+      <c r="B105" s="98" t="n"/>
+      <c r="C105" s="99" t="n"/>
+      <c r="D105" s="99" t="n"/>
+      <c r="E105" s="99" t="n"/>
+      <c r="F105" s="99" t="n"/>
+    </row>
+    <row r="106" ht="47.25" customHeight="1" s="82">
+      <c r="A106" s="9" t="n"/>
+      <c r="B106" s="100" t="inlineStr">
         <is>
           <t>Business Logic Testing</t>
         </is>
       </c>
-      <c r="C105" s="101" t="inlineStr">
+      <c r="C106" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D105" s="101" t="inlineStr">
+      <c r="D106" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E105" s="101" t="inlineStr">
+      <c r="E106" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F105" s="101" t="inlineStr">
+      <c r="F106" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="82.5" customHeight="1" s="82">
-      <c r="A106" s="19" t="n"/>
-      <c r="B106" s="34" t="inlineStr">
+    <row r="107" ht="82.5" customHeight="1" s="82">
+      <c r="A107" s="19" t="n"/>
+      <c r="B107" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C106" s="15">
+      <c r="C107" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D106" s="16" t="inlineStr">
+      <c r="D107" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E106" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F106" s="18" t="n"/>
-    </row>
-    <row r="107" ht="66" customHeight="1" s="82">
-      <c r="A107" s="19" t="n"/>
-      <c r="B107" s="34" t="inlineStr">
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="n"/>
+    </row>
+    <row r="108" ht="66" customHeight="1" s="82">
+      <c r="A108" s="19" t="n"/>
+      <c r="B108" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C107" s="15">
+      <c r="C108" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D107" s="16" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E107" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F107" s="18" t="n"/>
-    </row>
-    <row r="108" ht="148.5" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="n"/>
+    </row>
+    <row r="109" ht="148.5" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C109" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3890,147 +3915,147 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="49.5" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="49.5" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-04</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C110" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for system functionality that may be impacted by time.
 - Develop and execute misuse cases.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="66" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="n"/>
+    </row>
+    <row r="111" ht="66" customHeight="1" s="82">
+      <c r="A111" s="19" t="n"/>
+      <c r="B111" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-05</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C111" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D111" s="16" t="inlineStr">
         <is>
           <t>- Identify functions that must set limits to the times they can be called.
 - Assess if there is a logical limit set on the functions and if it is properly validated.</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F110" s="18" t="n"/>
-    </row>
-    <row r="111" ht="82.5" customHeight="1" s="82">
-      <c r="A111" s="19" t="n"/>
-      <c r="B111" s="34" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="n"/>
+    </row>
+    <row r="112" ht="82.5" customHeight="1" s="82">
+      <c r="A112" s="19" t="n"/>
+      <c r="B112" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-06</t>
         </is>
       </c>
-      <c r="C111" s="15">
+      <c r="C112" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
         <v/>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D112" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
 - Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F111" s="18" t="n"/>
-    </row>
-    <row r="112" ht="99" customHeight="1" s="82">
-      <c r="A112" s="19" t="n"/>
-      <c r="B112" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="99" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-07</t>
         </is>
       </c>
-      <c r="C112" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
         <v/>
       </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="99" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="99" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C113" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="165" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="165" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C114" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D114" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4040,114 +4065,91 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="66" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="66" customHeight="1" s="82">
+      <c r="A116" s="19" t="n"/>
+      <c r="B116" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C116" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="15" customHeight="1" s="82">
-      <c r="A116" s="97" t="n"/>
-      <c r="B116" s="98" t="n"/>
-      <c r="C116" s="99" t="n"/>
-      <c r="D116" s="99" t="n"/>
-      <c r="E116" s="99" t="n"/>
-      <c r="F116" s="99" t="n"/>
-    </row>
-    <row r="117" ht="47.25" customHeight="1" s="82">
-      <c r="A117" s="9" t="n"/>
-      <c r="B117" s="100" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="n"/>
+    </row>
+    <row r="117" ht="15" customHeight="1" s="82">
+      <c r="A117" s="97" t="n"/>
+      <c r="B117" s="98" t="n"/>
+      <c r="C117" s="99" t="n"/>
+      <c r="D117" s="99" t="n"/>
+      <c r="E117" s="99" t="n"/>
+      <c r="F117" s="99" t="n"/>
+    </row>
+    <row r="118" ht="47.25" customHeight="1" s="82">
+      <c r="A118" s="9" t="n"/>
+      <c r="B118" s="100" t="inlineStr">
         <is>
           <t>Client-side Testing</t>
         </is>
       </c>
-      <c r="C117" s="101" t="inlineStr">
+      <c r="C118" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D117" s="101" t="inlineStr">
+      <c r="D118" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E117" s="101" t="inlineStr">
+      <c r="E118" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F117" s="101" t="inlineStr">
+      <c r="F118" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="33" customHeight="1" s="82">
-      <c r="A118" s="19" t="n"/>
-      <c r="B118" s="34" t="inlineStr">
+    <row r="119" ht="33" customHeight="1" s="82">
+      <c r="A119" s="19" t="n"/>
+      <c r="B119" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-01</t>
         </is>
       </c>
-      <c r="C118" s="15">
+      <c r="C119" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D118" s="16" t="inlineStr">
+      <c r="D119" s="16" t="inlineStr">
         <is>
           <t>- Identify DOM sinks.
 - Build payloads that pertain to every sink type.</t>
         </is>
       </c>
-      <c r="E118" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F118" s="18" t="n"/>
-    </row>
-    <row r="119" ht="16.5" customHeight="1" s="82">
-      <c r="A119" s="19" t="n"/>
-      <c r="B119" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-02</t>
-        </is>
-      </c>
-      <c r="C119" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
-        <v/>
-      </c>
-      <c r="D119" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
-        </is>
-      </c>
       <c r="E119" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4155,20 +4157,20 @@
       </c>
       <c r="F119" s="18" t="n"/>
     </row>
-    <row r="120" ht="33" customHeight="1" s="82">
+    <row r="120" ht="16.5" customHeight="1" s="82">
       <c r="A120" s="19" t="n"/>
       <c r="B120" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-02</t>
         </is>
       </c>
       <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D120" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
         </is>
       </c>
       <c r="E120" s="18" t="inlineStr">
@@ -4182,17 +4184,16 @@
       <c r="A121" s="19" t="n"/>
       <c r="B121" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr">
@@ -4206,17 +4207,17 @@
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4230,17 +4231,17 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4254,17 +4255,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-07</t>
+          <t>WSTG-CLNT-06</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify endpoints that implement CORS.
-- Ensure that the CORS configuration is secure or harmless.</t>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4278,42 +4279,43 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-07</t>
+        </is>
+      </c>
+      <c r="C125" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <v/>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>- Identify endpoints that implement CORS.
+- Ensure that the CORS configuration is secure or harmless.</t>
+        </is>
+      </c>
+      <c r="E125" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F125" s="18" t="n"/>
+    </row>
+    <row r="126" ht="33" customHeight="1" s="82">
+      <c r="A126" s="19" t="n"/>
+      <c r="B126" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-08</t>
         </is>
       </c>
-      <c r="C125" s="15">
+      <c r="C126" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
         <v/>
       </c>
-      <c r="D125" s="16" t="inlineStr">
+      <c r="D126" s="16" t="inlineStr">
         <is>
           <t>- Decompile and analyze the application's code.
 - Assess sinks inputs and unsafe method usages.</t>
         </is>
       </c>
-      <c r="E125" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F125" s="18" t="n"/>
-    </row>
-    <row r="126" ht="16.5" customHeight="1" s="82">
-      <c r="A126" s="19" t="n"/>
-      <c r="B126" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-09</t>
-        </is>
-      </c>
-      <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
-        <v/>
-      </c>
-      <c r="D126" s="16" t="inlineStr">
-        <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
-        </is>
-      </c>
       <c r="E126" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4321,21 +4323,20 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="49.5" customHeight="1" s="82">
+    <row r="127" ht="16.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4349,90 +4350,91 @@
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-10</t>
+        </is>
+      </c>
+      <c r="C128" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <v/>
+      </c>
+      <c r="D128" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="n"/>
+    </row>
+    <row r="129" ht="49.5" customHeight="1" s="82">
+      <c r="A129" s="19" t="n"/>
+      <c r="B129" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-11</t>
         </is>
       </c>
-      <c r="C128" s="15">
+      <c r="C129" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
-      <c r="D128" s="16" t="inlineStr">
+      <c r="D129" s="16" t="inlineStr">
         <is>
           <t>- Assess the security of the message's origin.
 - Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
-      <c r="E128" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F128" s="18" t="n"/>
-    </row>
-    <row r="129" ht="82.5" customHeight="1" s="82">
-      <c r="A129" s="19" t="n"/>
-      <c r="B129" s="34" t="inlineStr">
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="n"/>
+    </row>
+    <row r="130" ht="82.5" customHeight="1" s="82">
+      <c r="A130" s="19" t="n"/>
+      <c r="B130" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-12</t>
         </is>
       </c>
-      <c r="C129" s="15">
+      <c r="C130" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the site is storing sensitive data in client-side storage.
 - The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F129" s="18" t="n"/>
-    </row>
-    <row r="130" ht="49.5" customHeight="1" s="82">
-      <c r="A130" s="19" t="n"/>
-      <c r="B130" s="34" t="inlineStr">
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="n"/>
+    </row>
+    <row r="131" ht="49.5" customHeight="1" s="82">
+      <c r="A131" s="19" t="n"/>
+      <c r="B131" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-13</t>
         </is>
       </c>
-      <c r="C130" s="15">
+      <c r="C131" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
-      <c r="D130" s="16" t="inlineStr">
+      <c r="D131" s="16" t="inlineStr">
         <is>
           <t>- Locate sensitive data across the system.
 - Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F130" s="18" t="n"/>
-    </row>
-    <row r="131" ht="16.5" customHeight="1" s="82">
-      <c r="A131" s="19" t="n"/>
-      <c r="B131" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D131" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E131" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4440,108 +4442,108 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="99" customHeight="1" s="82">
+    <row r="132" ht="16.5" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-14</t>
+        </is>
+      </c>
+      <c r="C132" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <v/>
+      </c>
+      <c r="D132" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="99" customHeight="1" s="82">
+      <c r="A133" s="19" t="n"/>
+      <c r="B133" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-15</t>
         </is>
       </c>
-      <c r="C132" s="15">
+      <c r="C133" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D132" s="16" t="inlineStr">
+      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="15" customHeight="1" s="82">
-      <c r="A133" s="97" t="n"/>
-      <c r="B133" s="98" t="n"/>
-      <c r="C133" s="99" t="n"/>
-      <c r="D133" s="99" t="n"/>
-      <c r="E133" s="99" t="n"/>
-      <c r="F133" s="99" t="n"/>
-    </row>
-    <row r="134" ht="47.25" customHeight="1" s="82">
-      <c r="A134" s="9" t="n"/>
-      <c r="B134" s="100" t="inlineStr">
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="n"/>
+    </row>
+    <row r="134" ht="15" customHeight="1" s="82">
+      <c r="A134" s="97" t="n"/>
+      <c r="B134" s="98" t="n"/>
+      <c r="C134" s="99" t="n"/>
+      <c r="D134" s="99" t="n"/>
+      <c r="E134" s="99" t="n"/>
+      <c r="F134" s="99" t="n"/>
+    </row>
+    <row r="135" ht="47.25" customHeight="1" s="82">
+      <c r="A135" s="9" t="n"/>
+      <c r="B135" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C134" s="101" t="inlineStr">
+      <c r="C135" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D134" s="101" t="inlineStr">
+      <c r="D135" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E134" s="101" t="inlineStr">
+      <c r="E135" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F134" s="101" t="inlineStr">
+      <c r="F135" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="99" customHeight="1" s="82">
-      <c r="A135" s="19" t="n"/>
-      <c r="B135" s="34" t="inlineStr">
+    <row r="136" ht="99" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C135" s="15">
+      <c r="C136" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D135" s="16" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E135" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F135" s="18" t="n"/>
-    </row>
-    <row r="136" ht="66" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-02</t>
-        </is>
-      </c>
-      <c r="C136" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D136" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
       <c r="E136" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4549,47 +4551,47 @@
       </c>
       <c r="F136" s="18" t="n"/>
     </row>
-    <row r="137" ht="132" customHeight="1" s="82">
+    <row r="137" ht="66" customHeight="1" s="82">
       <c r="A137" s="19" t="n"/>
       <c r="B137" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C137" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="132" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C137" s="15">
+      <c r="C138" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="82.5" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-04</t>
-        </is>
-      </c>
-      <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D138" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
       <c r="E138" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4597,38 +4599,61 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="66" customHeight="1" s="82">
+    <row r="139" ht="82.5" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C139" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="66" customHeight="1" s="82">
+      <c r="A140" s="19" t="n"/>
+      <c r="B140" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C140" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="82">
-      <c r="A140" s="97" t="n"/>
-      <c r="B140" s="98" t="n"/>
-      <c r="C140" s="99" t="n"/>
-      <c r="D140" s="99" t="n"/>
-      <c r="E140" s="99" t="n"/>
-      <c r="F140" s="99" t="n"/>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="82">
+      <c r="A141" s="97" t="n"/>
+      <c r="B141" s="98" t="n"/>
+      <c r="C141" s="99" t="n"/>
+      <c r="D141" s="99" t="n"/>
+      <c r="E141" s="99" t="n"/>
+      <c r="F141" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4645,7 +4670,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F140">
+  <conditionalFormatting sqref="B4:F141">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4657,7 +4682,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E96 E97 E100 E101 E102 E103 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-06-30 (#1438)
Updates based on OWASP/wstg@b87d2b2
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3571,167 +3571,168 @@
       </c>
       <c r="F93" s="18" t="n"/>
     </row>
-    <row r="94" ht="15" customHeight="1" s="82">
-      <c r="A94" s="97" t="n"/>
-      <c r="B94" s="98" t="n"/>
-      <c r="C94" s="99" t="n"/>
-      <c r="D94" s="99" t="n"/>
-      <c r="E94" s="99" t="n"/>
-      <c r="F94" s="99" t="n"/>
-    </row>
-    <row r="95" ht="47.25" customHeight="1" s="82">
-      <c r="A95" s="9" t="n"/>
-      <c r="B95" s="100" t="inlineStr">
+    <row r="94" ht="99" customHeight="1" s="82">
+      <c r="A94" s="19" t="n"/>
+      <c r="B94" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-22</t>
+        </is>
+      </c>
+      <c r="C94" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
+        <v/>
+      </c>
+      <c r="D94" s="16" t="inlineStr">
+        <is>
+          <t>- Identify functions and libraries that recursively merge, clone, or assign user-controlled properties.
+- Determine whether user input can reach and modify `Object.prototype`.
+- Identify gadgets that turn prototype pollution into a concrete impact.</t>
+        </is>
+      </c>
+      <c r="E94" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F94" s="18" t="n"/>
+    </row>
+    <row r="95" ht="15" customHeight="1" s="82">
+      <c r="A95" s="97" t="n"/>
+      <c r="B95" s="98" t="n"/>
+      <c r="C95" s="99" t="n"/>
+      <c r="D95" s="99" t="n"/>
+      <c r="E95" s="99" t="n"/>
+      <c r="F95" s="99" t="n"/>
+    </row>
+    <row r="96" ht="47.25" customHeight="1" s="82">
+      <c r="A96" s="9" t="n"/>
+      <c r="B96" s="100" t="inlineStr">
         <is>
           <t>Testing for Error Handling</t>
         </is>
       </c>
-      <c r="C95" s="101" t="inlineStr">
+      <c r="C96" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D95" s="101" t="inlineStr">
+      <c r="D96" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E95" s="101" t="inlineStr">
+      <c r="E96" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F95" s="101" t="inlineStr">
+      <c r="F96" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="96" ht="33" customHeight="1" s="82">
-      <c r="A96" s="19" t="n"/>
-      <c r="B96" s="34" t="inlineStr">
+    <row r="97" ht="33" customHeight="1" s="82">
+      <c r="A97" s="19" t="n"/>
+      <c r="B97" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C96" s="15">
+      <c r="C97" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D96" s="16" t="inlineStr">
+      <c r="D97" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E96" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F96" s="18" t="n"/>
-    </row>
-    <row r="97" ht="16.5" customHeight="1" s="82">
-      <c r="A97" s="19" t="n"/>
-      <c r="B97" s="34" t="inlineStr">
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F97" s="18" t="n"/>
+    </row>
+    <row r="98" ht="16.5" customHeight="1" s="82">
+      <c r="A98" s="19" t="n"/>
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C97" s="15">
+      <c r="C98" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
         <v/>
       </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="D98" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E97" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F97" s="18" t="n"/>
-    </row>
-    <row r="98" ht="15" customHeight="1" s="82">
-      <c r="A98" s="97" t="n"/>
-      <c r="B98" s="98" t="n"/>
-      <c r="C98" s="99" t="n"/>
-      <c r="D98" s="99" t="n"/>
-      <c r="E98" s="99" t="n"/>
-      <c r="F98" s="99" t="n"/>
-    </row>
-    <row r="99" ht="47.25" customHeight="1" s="82">
-      <c r="A99" s="9" t="n"/>
-      <c r="B99" s="100" t="inlineStr">
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="n"/>
+    </row>
+    <row r="99" ht="15" customHeight="1" s="82">
+      <c r="A99" s="97" t="n"/>
+      <c r="B99" s="98" t="n"/>
+      <c r="C99" s="99" t="n"/>
+      <c r="D99" s="99" t="n"/>
+      <c r="E99" s="99" t="n"/>
+      <c r="F99" s="99" t="n"/>
+    </row>
+    <row r="100" ht="47.25" customHeight="1" s="82">
+      <c r="A100" s="9" t="n"/>
+      <c r="B100" s="100" t="inlineStr">
         <is>
           <t>Testing for Weak Cryptography</t>
         </is>
       </c>
-      <c r="C99" s="101" t="inlineStr">
+      <c r="C100" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D99" s="101" t="inlineStr">
+      <c r="D100" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E99" s="101" t="inlineStr">
+      <c r="E100" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F99" s="101" t="inlineStr">
+      <c r="F100" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="82.5" customHeight="1" s="82">
-      <c r="A100" s="19" t="n"/>
-      <c r="B100" s="34" t="inlineStr">
+    <row r="101" ht="82.5" customHeight="1" s="82">
+      <c r="A101" s="19" t="n"/>
+      <c r="B101" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C100" s="15">
+      <c r="C101" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D100" s="16" t="inlineStr">
+      <c r="D101" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
-      <c r="E100" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F100" s="18" t="n"/>
-    </row>
-    <row r="101" ht="49.5" customHeight="1" s="82">
-      <c r="A101" s="19" t="n"/>
-      <c r="B101" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-02</t>
-        </is>
-      </c>
-      <c r="C101" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
-        <v/>
-      </c>
-      <c r="D101" s="16" t="inlineStr">
-        <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
-        </is>
-      </c>
       <c r="E101" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3743,146 +3744,170 @@
       <c r="A102" s="19" t="n"/>
       <c r="B102" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C102" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D102" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E102" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F102" s="18" t="n"/>
+    </row>
+    <row r="103" ht="49.5" customHeight="1" s="82">
+      <c r="A103" s="19" t="n"/>
+      <c r="B103" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CRYP-03</t>
         </is>
       </c>
-      <c r="C102" s="15">
+      <c r="C103" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
-      <c r="D102" s="16" t="inlineStr">
+      <c r="D103" s="16" t="inlineStr">
         <is>
           <t>- Identify sensitive information transmitted through the various channels.
 - Assess the privacy and security of the channels used.</t>
         </is>
       </c>
-      <c r="E102" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F102" s="18" t="n"/>
-    </row>
-    <row r="103" ht="33" customHeight="1" s="82">
-      <c r="A103" s="19" t="n"/>
-      <c r="B103" s="34" t="inlineStr">
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="n"/>
+    </row>
+    <row r="104" ht="33" customHeight="1" s="82">
+      <c r="A104" s="19" t="n"/>
+      <c r="B104" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-04</t>
         </is>
       </c>
-      <c r="C103" s="15">
+      <c r="C104" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
-      <c r="D103" s="16" t="inlineStr">
+      <c r="D104" s="16" t="inlineStr">
         <is>
           <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
-      <c r="E103" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F103" s="18" t="n"/>
-    </row>
-    <row r="104" ht="15" customHeight="1" s="82">
-      <c r="A104" s="97" t="n"/>
-      <c r="B104" s="98" t="n"/>
-      <c r="C104" s="99" t="n"/>
-      <c r="D104" s="99" t="n"/>
-      <c r="E104" s="99" t="n"/>
-      <c r="F104" s="99" t="n"/>
-    </row>
-    <row r="105" ht="47.25" customHeight="1" s="82">
-      <c r="A105" s="9" t="n"/>
-      <c r="B105" s="100" t="inlineStr">
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="n"/>
+    </row>
+    <row r="105" ht="15" customHeight="1" s="82">
+      <c r="A105" s="97" t="n"/>
+      <c r="B105" s="98" t="n"/>
+      <c r="C105" s="99" t="n"/>
+      <c r="D105" s="99" t="n"/>
+      <c r="E105" s="99" t="n"/>
+      <c r="F105" s="99" t="n"/>
+    </row>
+    <row r="106" ht="47.25" customHeight="1" s="82">
+      <c r="A106" s="9" t="n"/>
+      <c r="B106" s="100" t="inlineStr">
         <is>
           <t>Business Logic Testing</t>
         </is>
       </c>
-      <c r="C105" s="101" t="inlineStr">
+      <c r="C106" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D105" s="101" t="inlineStr">
+      <c r="D106" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E105" s="101" t="inlineStr">
+      <c r="E106" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F105" s="101" t="inlineStr">
+      <c r="F106" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="106" ht="82.5" customHeight="1" s="82">
-      <c r="A106" s="19" t="n"/>
-      <c r="B106" s="34" t="inlineStr">
+    <row r="107" ht="82.5" customHeight="1" s="82">
+      <c r="A107" s="19" t="n"/>
+      <c r="B107" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C106" s="15">
+      <c r="C107" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D106" s="16" t="inlineStr">
+      <c r="D107" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E106" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F106" s="18" t="n"/>
-    </row>
-    <row r="107" ht="66" customHeight="1" s="82">
-      <c r="A107" s="19" t="n"/>
-      <c r="B107" s="34" t="inlineStr">
+      <c r="E107" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F107" s="18" t="n"/>
+    </row>
+    <row r="108" ht="66" customHeight="1" s="82">
+      <c r="A108" s="19" t="n"/>
+      <c r="B108" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C107" s="15">
+      <c r="C108" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D107" s="16" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E107" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F107" s="18" t="n"/>
-    </row>
-    <row r="108" ht="148.5" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="n"/>
+    </row>
+    <row r="109" ht="148.5" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C109" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3890,147 +3915,147 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="49.5" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="49.5" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-04</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C110" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for system functionality that may be impacted by time.
 - Develop and execute misuse cases.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="66" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="n"/>
+    </row>
+    <row r="111" ht="66" customHeight="1" s="82">
+      <c r="A111" s="19" t="n"/>
+      <c r="B111" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-05</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C111" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D111" s="16" t="inlineStr">
         <is>
           <t>- Identify functions that must set limits to the times they can be called.
 - Assess if there is a logical limit set on the functions and if it is properly validated.</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F110" s="18" t="n"/>
-    </row>
-    <row r="111" ht="82.5" customHeight="1" s="82">
-      <c r="A111" s="19" t="n"/>
-      <c r="B111" s="34" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="n"/>
+    </row>
+    <row r="112" ht="82.5" customHeight="1" s="82">
+      <c r="A112" s="19" t="n"/>
+      <c r="B112" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-06</t>
         </is>
       </c>
-      <c r="C111" s="15">
+      <c r="C112" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
         <v/>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D112" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
 - Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F111" s="18" t="n"/>
-    </row>
-    <row r="112" ht="99" customHeight="1" s="82">
-      <c r="A112" s="19" t="n"/>
-      <c r="B112" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="99" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-07</t>
         </is>
       </c>
-      <c r="C112" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
         <v/>
       </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="99" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="99" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C113" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="165" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="165" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C114" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D114" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4040,114 +4065,91 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="66" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="66" customHeight="1" s="82">
+      <c r="A116" s="19" t="n"/>
+      <c r="B116" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C116" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="15" customHeight="1" s="82">
-      <c r="A116" s="97" t="n"/>
-      <c r="B116" s="98" t="n"/>
-      <c r="C116" s="99" t="n"/>
-      <c r="D116" s="99" t="n"/>
-      <c r="E116" s="99" t="n"/>
-      <c r="F116" s="99" t="n"/>
-    </row>
-    <row r="117" ht="47.25" customHeight="1" s="82">
-      <c r="A117" s="9" t="n"/>
-      <c r="B117" s="100" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="n"/>
+    </row>
+    <row r="117" ht="15" customHeight="1" s="82">
+      <c r="A117" s="97" t="n"/>
+      <c r="B117" s="98" t="n"/>
+      <c r="C117" s="99" t="n"/>
+      <c r="D117" s="99" t="n"/>
+      <c r="E117" s="99" t="n"/>
+      <c r="F117" s="99" t="n"/>
+    </row>
+    <row r="118" ht="47.25" customHeight="1" s="82">
+      <c r="A118" s="9" t="n"/>
+      <c r="B118" s="100" t="inlineStr">
         <is>
           <t>Client-side Testing</t>
         </is>
       </c>
-      <c r="C117" s="101" t="inlineStr">
+      <c r="C118" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D117" s="101" t="inlineStr">
+      <c r="D118" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E117" s="101" t="inlineStr">
+      <c r="E118" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F117" s="101" t="inlineStr">
+      <c r="F118" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="33" customHeight="1" s="82">
-      <c r="A118" s="19" t="n"/>
-      <c r="B118" s="34" t="inlineStr">
+    <row r="119" ht="33" customHeight="1" s="82">
+      <c r="A119" s="19" t="n"/>
+      <c r="B119" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-01</t>
         </is>
       </c>
-      <c r="C118" s="15">
+      <c r="C119" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D118" s="16" t="inlineStr">
+      <c r="D119" s="16" t="inlineStr">
         <is>
           <t>- Identify DOM sinks.
 - Build payloads that pertain to every sink type.</t>
         </is>
       </c>
-      <c r="E118" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F118" s="18" t="n"/>
-    </row>
-    <row r="119" ht="16.5" customHeight="1" s="82">
-      <c r="A119" s="19" t="n"/>
-      <c r="B119" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-02</t>
-        </is>
-      </c>
-      <c r="C119" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
-        <v/>
-      </c>
-      <c r="D119" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
-        </is>
-      </c>
       <c r="E119" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4155,20 +4157,20 @@
       </c>
       <c r="F119" s="18" t="n"/>
     </row>
-    <row r="120" ht="33" customHeight="1" s="82">
+    <row r="120" ht="16.5" customHeight="1" s="82">
       <c r="A120" s="19" t="n"/>
       <c r="B120" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-02</t>
         </is>
       </c>
       <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D120" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
         </is>
       </c>
       <c r="E120" s="18" t="inlineStr">
@@ -4182,17 +4184,16 @@
       <c r="A121" s="19" t="n"/>
       <c r="B121" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr">
@@ -4206,17 +4207,17 @@
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4230,17 +4231,17 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4254,17 +4255,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-07</t>
+          <t>WSTG-CLNT-06</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify endpoints that implement CORS.
-- Ensure that the CORS configuration is secure or harmless.</t>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4278,42 +4279,43 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-07</t>
+        </is>
+      </c>
+      <c r="C125" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <v/>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>- Identify endpoints that implement CORS.
+- Ensure that the CORS configuration is secure or harmless.</t>
+        </is>
+      </c>
+      <c r="E125" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F125" s="18" t="n"/>
+    </row>
+    <row r="126" ht="33" customHeight="1" s="82">
+      <c r="A126" s="19" t="n"/>
+      <c r="B126" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-08</t>
         </is>
       </c>
-      <c r="C125" s="15">
+      <c r="C126" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
         <v/>
       </c>
-      <c r="D125" s="16" t="inlineStr">
+      <c r="D126" s="16" t="inlineStr">
         <is>
           <t>- Decompile and analyze the application's code.
 - Assess sinks inputs and unsafe method usages.</t>
         </is>
       </c>
-      <c r="E125" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F125" s="18" t="n"/>
-    </row>
-    <row r="126" ht="16.5" customHeight="1" s="82">
-      <c r="A126" s="19" t="n"/>
-      <c r="B126" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-09</t>
-        </is>
-      </c>
-      <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
-        <v/>
-      </c>
-      <c r="D126" s="16" t="inlineStr">
-        <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
-        </is>
-      </c>
       <c r="E126" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4321,21 +4323,20 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="49.5" customHeight="1" s="82">
+    <row r="127" ht="16.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4349,90 +4350,91 @@
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-10</t>
+        </is>
+      </c>
+      <c r="C128" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <v/>
+      </c>
+      <c r="D128" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="n"/>
+    </row>
+    <row r="129" ht="49.5" customHeight="1" s="82">
+      <c r="A129" s="19" t="n"/>
+      <c r="B129" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-11</t>
         </is>
       </c>
-      <c r="C128" s="15">
+      <c r="C129" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
-      <c r="D128" s="16" t="inlineStr">
+      <c r="D129" s="16" t="inlineStr">
         <is>
           <t>- Assess the security of the message's origin.
 - Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
-      <c r="E128" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F128" s="18" t="n"/>
-    </row>
-    <row r="129" ht="82.5" customHeight="1" s="82">
-      <c r="A129" s="19" t="n"/>
-      <c r="B129" s="34" t="inlineStr">
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="n"/>
+    </row>
+    <row r="130" ht="82.5" customHeight="1" s="82">
+      <c r="A130" s="19" t="n"/>
+      <c r="B130" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-12</t>
         </is>
       </c>
-      <c r="C129" s="15">
+      <c r="C130" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the site is storing sensitive data in client-side storage.
 - The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F129" s="18" t="n"/>
-    </row>
-    <row r="130" ht="49.5" customHeight="1" s="82">
-      <c r="A130" s="19" t="n"/>
-      <c r="B130" s="34" t="inlineStr">
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="n"/>
+    </row>
+    <row r="131" ht="49.5" customHeight="1" s="82">
+      <c r="A131" s="19" t="n"/>
+      <c r="B131" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-13</t>
         </is>
       </c>
-      <c r="C130" s="15">
+      <c r="C131" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
-      <c r="D130" s="16" t="inlineStr">
+      <c r="D131" s="16" t="inlineStr">
         <is>
           <t>- Locate sensitive data across the system.
 - Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F130" s="18" t="n"/>
-    </row>
-    <row r="131" ht="16.5" customHeight="1" s="82">
-      <c r="A131" s="19" t="n"/>
-      <c r="B131" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D131" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E131" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4440,108 +4442,108 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="99" customHeight="1" s="82">
+    <row r="132" ht="16.5" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-14</t>
+        </is>
+      </c>
+      <c r="C132" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <v/>
+      </c>
+      <c r="D132" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="99" customHeight="1" s="82">
+      <c r="A133" s="19" t="n"/>
+      <c r="B133" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-15</t>
         </is>
       </c>
-      <c r="C132" s="15">
+      <c r="C133" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D132" s="16" t="inlineStr">
+      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="15" customHeight="1" s="82">
-      <c r="A133" s="97" t="n"/>
-      <c r="B133" s="98" t="n"/>
-      <c r="C133" s="99" t="n"/>
-      <c r="D133" s="99" t="n"/>
-      <c r="E133" s="99" t="n"/>
-      <c r="F133" s="99" t="n"/>
-    </row>
-    <row r="134" ht="47.25" customHeight="1" s="82">
-      <c r="A134" s="9" t="n"/>
-      <c r="B134" s="100" t="inlineStr">
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="n"/>
+    </row>
+    <row r="134" ht="15" customHeight="1" s="82">
+      <c r="A134" s="97" t="n"/>
+      <c r="B134" s="98" t="n"/>
+      <c r="C134" s="99" t="n"/>
+      <c r="D134" s="99" t="n"/>
+      <c r="E134" s="99" t="n"/>
+      <c r="F134" s="99" t="n"/>
+    </row>
+    <row r="135" ht="47.25" customHeight="1" s="82">
+      <c r="A135" s="9" t="n"/>
+      <c r="B135" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C134" s="101" t="inlineStr">
+      <c r="C135" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D134" s="101" t="inlineStr">
+      <c r="D135" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E134" s="101" t="inlineStr">
+      <c r="E135" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F134" s="101" t="inlineStr">
+      <c r="F135" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="99" customHeight="1" s="82">
-      <c r="A135" s="19" t="n"/>
-      <c r="B135" s="34" t="inlineStr">
+    <row r="136" ht="99" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C135" s="15">
+      <c r="C136" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D135" s="16" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E135" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F135" s="18" t="n"/>
-    </row>
-    <row r="136" ht="66" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-02</t>
-        </is>
-      </c>
-      <c r="C136" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D136" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
       <c r="E136" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4549,47 +4551,47 @@
       </c>
       <c r="F136" s="18" t="n"/>
     </row>
-    <row r="137" ht="132" customHeight="1" s="82">
+    <row r="137" ht="66" customHeight="1" s="82">
       <c r="A137" s="19" t="n"/>
       <c r="B137" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C137" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="132" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C137" s="15">
+      <c r="C138" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="82.5" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-04</t>
-        </is>
-      </c>
-      <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D138" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
       <c r="E138" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4597,38 +4599,61 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="66" customHeight="1" s="82">
+    <row r="139" ht="82.5" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C139" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="66" customHeight="1" s="82">
+      <c r="A140" s="19" t="n"/>
+      <c r="B140" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C140" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="82">
-      <c r="A140" s="97" t="n"/>
-      <c r="B140" s="98" t="n"/>
-      <c r="C140" s="99" t="n"/>
-      <c r="D140" s="99" t="n"/>
-      <c r="E140" s="99" t="n"/>
-      <c r="F140" s="99" t="n"/>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="82">
+      <c r="A141" s="97" t="n"/>
+      <c r="B141" s="98" t="n"/>
+      <c r="C141" s="99" t="n"/>
+      <c r="D141" s="99" t="n"/>
+      <c r="E141" s="99" t="n"/>
+      <c r="F141" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4645,7 +4670,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F140">
+  <conditionalFormatting sqref="B4:F141">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4657,7 +4682,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E96 E97 E100 E101 E102 E103 E106 E107 E108 E109 E110 E111 E112 E113 E114 E115 E118 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-08-08
Updates based on OWASP/wstg@6b39572
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>- Identify the backend and the parsing method used.
+          <t>- Identify the back end and the parsing method used.
 - Assess injection points and try bypassing input filters using HPP.</t>
         </is>
       </c>
@@ -4299,21 +4299,20 @@
       </c>
       <c r="F125" s="18" t="n"/>
     </row>
-    <row r="126" ht="33" customHeight="1" s="82">
+    <row r="126" ht="16.5" customHeight="1" s="82">
       <c r="A126" s="19" t="n"/>
       <c r="B126" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-08</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D126" s="16" t="inlineStr">
         <is>
-          <t>- Decompile and analyze the application's code.
-- Assess sinks inputs and unsafe method usages.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E126" s="18" t="inlineStr">
@@ -4323,20 +4322,21 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="16.5" customHeight="1" s="82">
+    <row r="127" ht="49.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-09</t>
+          <t>WSTG-CLNT-10</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4350,17 +4350,17 @@
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-11</t>
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess the security of the message's origin.
+- Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
       <c r="E128" s="18" t="inlineStr">
@@ -4370,21 +4370,21 @@
       </c>
       <c r="F128" s="18" t="n"/>
     </row>
-    <row r="129" ht="49.5" customHeight="1" s="82">
+    <row r="129" ht="82.5" customHeight="1" s="82">
       <c r="A129" s="19" t="n"/>
       <c r="B129" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-11</t>
+          <t>WSTG-CLNT-12</t>
         </is>
       </c>
       <c r="C129" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>- Assess the security of the message's origin.
-- Validate that it's using safe methods and validating its input.</t>
+          <t>- Determine whether the site is storing sensitive data in client-side storage.
+- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
       <c r="E129" s="18" t="inlineStr">
@@ -4394,21 +4394,21 @@
       </c>
       <c r="F129" s="18" t="n"/>
     </row>
-    <row r="130" ht="82.5" customHeight="1" s="82">
+    <row r="130" ht="49.5" customHeight="1" s="82">
       <c r="A130" s="19" t="n"/>
       <c r="B130" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-12</t>
+          <t>WSTG-CLNT-13</t>
         </is>
       </c>
       <c r="C130" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
       <c r="D130" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the site is storing sensitive data in client-side storage.
-- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
+          <t>- Locate sensitive data across the system.
+- Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
       <c r="E130" s="18" t="inlineStr">
@@ -4418,21 +4418,20 @@
       </c>
       <c r="F130" s="18" t="n"/>
     </row>
-    <row r="131" ht="49.5" customHeight="1" s="82">
+    <row r="131" ht="16.5" customHeight="1" s="82">
       <c r="A131" s="19" t="n"/>
       <c r="B131" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-13</t>
+          <t>WSTG-CLNT-14</t>
         </is>
       </c>
       <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
         <v/>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>- Locate sensitive data across the system.
-- Assess the leakage of sensitive data through various techniques.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E131" s="18" t="inlineStr">
@@ -4442,108 +4441,108 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="16.5" customHeight="1" s="82">
+    <row r="132" ht="99" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-14</t>
+          <t>WSTG-CLNT-15</t>
         </is>
       </c>
       <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
       <c r="D132" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="99" customHeight="1" s="82">
-      <c r="A133" s="19" t="n"/>
-      <c r="B133" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-15</t>
-        </is>
-      </c>
-      <c r="C133" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
-        <v/>
-      </c>
-      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F133" s="18" t="n"/>
-    </row>
-    <row r="134" ht="15" customHeight="1" s="82">
-      <c r="A134" s="97" t="n"/>
-      <c r="B134" s="98" t="n"/>
-      <c r="C134" s="99" t="n"/>
-      <c r="D134" s="99" t="n"/>
-      <c r="E134" s="99" t="n"/>
-      <c r="F134" s="99" t="n"/>
-    </row>
-    <row r="135" ht="47.25" customHeight="1" s="82">
-      <c r="A135" s="9" t="n"/>
-      <c r="B135" s="100" t="inlineStr">
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="15" customHeight="1" s="82">
+      <c r="A133" s="97" t="n"/>
+      <c r="B133" s="98" t="n"/>
+      <c r="C133" s="99" t="n"/>
+      <c r="D133" s="99" t="n"/>
+      <c r="E133" s="99" t="n"/>
+      <c r="F133" s="99" t="n"/>
+    </row>
+    <row r="134" ht="47.25" customHeight="1" s="82">
+      <c r="A134" s="9" t="n"/>
+      <c r="B134" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C135" s="101" t="inlineStr">
+      <c r="C134" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D135" s="101" t="inlineStr">
+      <c r="D134" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E135" s="101" t="inlineStr">
+      <c r="E134" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F135" s="101" t="inlineStr">
+      <c r="F134" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="99" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
+    <row r="135" ht="99" customHeight="1" s="82">
+      <c r="A135" s="19" t="n"/>
+      <c r="B135" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C136" s="15">
+      <c r="C135" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D136" s="16" t="inlineStr">
+      <c r="D135" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
+      <c r="E135" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F135" s="18" t="n"/>
+    </row>
+    <row r="136" ht="66" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C136" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D136" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
       <c r="E136" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4551,47 +4550,47 @@
       </c>
       <c r="F136" s="18" t="n"/>
     </row>
-    <row r="137" ht="66" customHeight="1" s="82">
+    <row r="137" ht="132" customHeight="1" s="82">
       <c r="A137" s="19" t="n"/>
       <c r="B137" s="34" t="inlineStr">
         <is>
-          <t>WSTG-APIT-02</t>
+          <t>WSTG-APIT-03</t>
         </is>
       </c>
       <c r="C137" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
       <c r="D137" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="132" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-03</t>
-        </is>
-      </c>
-      <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
-        <v/>
-      </c>
-      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="82.5" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C138" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D138" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
       <c r="E138" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4599,61 +4598,38 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="82.5" customHeight="1" s="82">
+    <row r="139" ht="66" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
-          <t>WSTG-APIT-04</t>
+          <t>WSTG-APIT-99</t>
         </is>
       </c>
       <c r="C139" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
       <c r="D139" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="66" customHeight="1" s="82">
-      <c r="A140" s="19" t="n"/>
-      <c r="B140" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-99</t>
-        </is>
-      </c>
-      <c r="C140" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
-        <v/>
-      </c>
-      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="82">
-      <c r="A141" s="97" t="n"/>
-      <c r="B141" s="98" t="n"/>
-      <c r="C141" s="99" t="n"/>
-      <c r="D141" s="99" t="n"/>
-      <c r="E141" s="99" t="n"/>
-      <c r="F141" s="99" t="n"/>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="15" customHeight="1" s="82">
+      <c r="A140" s="97" t="n"/>
+      <c r="B140" s="98" t="n"/>
+      <c r="C140" s="99" t="n"/>
+      <c r="D140" s="99" t="n"/>
+      <c r="E140" s="99" t="n"/>
+      <c r="F140" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4670,7 +4646,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F141">
+  <conditionalFormatting sqref="B4:F140">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4682,7 +4658,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-08-08 (#1458)
Updates based on OWASP/wstg@6b39572
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>- Identify the backend and the parsing method used.
+          <t>- Identify the back end and the parsing method used.
 - Assess injection points and try bypassing input filters using HPP.</t>
         </is>
       </c>
@@ -4299,21 +4299,20 @@
       </c>
       <c r="F125" s="18" t="n"/>
     </row>
-    <row r="126" ht="33" customHeight="1" s="82">
+    <row r="126" ht="16.5" customHeight="1" s="82">
       <c r="A126" s="19" t="n"/>
       <c r="B126" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-08</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/08-Testing_for_Cross_Site_Flashing", "Testing for Cross Site Flashing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D126" s="16" t="inlineStr">
         <is>
-          <t>- Decompile and analyze the application's code.
-- Assess sinks inputs and unsafe method usages.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E126" s="18" t="inlineStr">
@@ -4323,20 +4322,21 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="16.5" customHeight="1" s="82">
+    <row r="127" ht="49.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-09</t>
+          <t>WSTG-CLNT-10</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4350,17 +4350,17 @@
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-11</t>
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess the security of the message's origin.
+- Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
       <c r="E128" s="18" t="inlineStr">
@@ -4370,21 +4370,21 @@
       </c>
       <c r="F128" s="18" t="n"/>
     </row>
-    <row r="129" ht="49.5" customHeight="1" s="82">
+    <row r="129" ht="82.5" customHeight="1" s="82">
       <c r="A129" s="19" t="n"/>
       <c r="B129" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-11</t>
+          <t>WSTG-CLNT-12</t>
         </is>
       </c>
       <c r="C129" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>- Assess the security of the message's origin.
-- Validate that it's using safe methods and validating its input.</t>
+          <t>- Determine whether the site is storing sensitive data in client-side storage.
+- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
       <c r="E129" s="18" t="inlineStr">
@@ -4394,21 +4394,21 @@
       </c>
       <c r="F129" s="18" t="n"/>
     </row>
-    <row r="130" ht="82.5" customHeight="1" s="82">
+    <row r="130" ht="49.5" customHeight="1" s="82">
       <c r="A130" s="19" t="n"/>
       <c r="B130" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-12</t>
+          <t>WSTG-CLNT-13</t>
         </is>
       </c>
       <c r="C130" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
       <c r="D130" s="16" t="inlineStr">
         <is>
-          <t>- Determine whether the site is storing sensitive data in client-side storage.
-- The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
+          <t>- Locate sensitive data across the system.
+- Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
       <c r="E130" s="18" t="inlineStr">
@@ -4418,21 +4418,20 @@
       </c>
       <c r="F130" s="18" t="n"/>
     </row>
-    <row r="131" ht="49.5" customHeight="1" s="82">
+    <row r="131" ht="16.5" customHeight="1" s="82">
       <c r="A131" s="19" t="n"/>
       <c r="B131" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-13</t>
+          <t>WSTG-CLNT-14</t>
         </is>
       </c>
       <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
         <v/>
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>- Locate sensitive data across the system.
-- Assess the leakage of sensitive data through various techniques.</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E131" s="18" t="inlineStr">
@@ -4442,108 +4441,108 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="16.5" customHeight="1" s="82">
+    <row r="132" ht="99" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-14</t>
+          <t>WSTG-CLNT-15</t>
         </is>
       </c>
       <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
       <c r="D132" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="99" customHeight="1" s="82">
-      <c r="A133" s="19" t="n"/>
-      <c r="B133" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-15</t>
-        </is>
-      </c>
-      <c r="C133" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
-        <v/>
-      </c>
-      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E133" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F133" s="18" t="n"/>
-    </row>
-    <row r="134" ht="15" customHeight="1" s="82">
-      <c r="A134" s="97" t="n"/>
-      <c r="B134" s="98" t="n"/>
-      <c r="C134" s="99" t="n"/>
-      <c r="D134" s="99" t="n"/>
-      <c r="E134" s="99" t="n"/>
-      <c r="F134" s="99" t="n"/>
-    </row>
-    <row r="135" ht="47.25" customHeight="1" s="82">
-      <c r="A135" s="9" t="n"/>
-      <c r="B135" s="100" t="inlineStr">
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="15" customHeight="1" s="82">
+      <c r="A133" s="97" t="n"/>
+      <c r="B133" s="98" t="n"/>
+      <c r="C133" s="99" t="n"/>
+      <c r="D133" s="99" t="n"/>
+      <c r="E133" s="99" t="n"/>
+      <c r="F133" s="99" t="n"/>
+    </row>
+    <row r="134" ht="47.25" customHeight="1" s="82">
+      <c r="A134" s="9" t="n"/>
+      <c r="B134" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C135" s="101" t="inlineStr">
+      <c r="C134" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D135" s="101" t="inlineStr">
+      <c r="D134" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E135" s="101" t="inlineStr">
+      <c r="E134" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F135" s="101" t="inlineStr">
+      <c r="F134" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="99" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
+    <row r="135" ht="99" customHeight="1" s="82">
+      <c r="A135" s="19" t="n"/>
+      <c r="B135" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C136" s="15">
+      <c r="C135" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D136" s="16" t="inlineStr">
+      <c r="D135" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
+      <c r="E135" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F135" s="18" t="n"/>
+    </row>
+    <row r="136" ht="66" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C136" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D136" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
       <c r="E136" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4551,47 +4550,47 @@
       </c>
       <c r="F136" s="18" t="n"/>
     </row>
-    <row r="137" ht="66" customHeight="1" s="82">
+    <row r="137" ht="132" customHeight="1" s="82">
       <c r="A137" s="19" t="n"/>
       <c r="B137" s="34" t="inlineStr">
         <is>
-          <t>WSTG-APIT-02</t>
+          <t>WSTG-APIT-03</t>
         </is>
       </c>
       <c r="C137" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
       <c r="D137" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="132" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-03</t>
-        </is>
-      </c>
-      <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
-        <v/>
-      </c>
-      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="82.5" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C138" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D138" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
       <c r="E138" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4599,61 +4598,38 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="82.5" customHeight="1" s="82">
+    <row r="139" ht="66" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
-          <t>WSTG-APIT-04</t>
+          <t>WSTG-APIT-99</t>
         </is>
       </c>
       <c r="C139" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
       <c r="D139" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="66" customHeight="1" s="82">
-      <c r="A140" s="19" t="n"/>
-      <c r="B140" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-99</t>
-        </is>
-      </c>
-      <c r="C140" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
-        <v/>
-      </c>
-      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E140" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F140" s="18" t="n"/>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="82">
-      <c r="A141" s="97" t="n"/>
-      <c r="B141" s="98" t="n"/>
-      <c r="C141" s="99" t="n"/>
-      <c r="D141" s="99" t="n"/>
-      <c r="E141" s="99" t="n"/>
-      <c r="F141" s="99" t="n"/>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="15" customHeight="1" s="82">
+      <c r="A140" s="97" t="n"/>
+      <c r="B140" s="98" t="n"/>
+      <c r="C140" s="99" t="n"/>
+      <c r="D140" s="99" t="n"/>
+      <c r="E140" s="99" t="n"/>
+      <c r="F140" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4670,7 +4646,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F141">
+  <conditionalFormatting sqref="B4:F140">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4682,7 +4658,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-08-10
Updates based on OWASP/wstg@3d5849b
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3596,167 +3596,171 @@
       </c>
       <c r="F94" s="18" t="n"/>
     </row>
-    <row r="95" ht="15" customHeight="1" s="82">
-      <c r="A95" s="97" t="n"/>
-      <c r="B95" s="98" t="n"/>
-      <c r="C95" s="99" t="n"/>
-      <c r="D95" s="99" t="n"/>
-      <c r="E95" s="99" t="n"/>
-      <c r="F95" s="99" t="n"/>
-    </row>
-    <row r="96" ht="47.25" customHeight="1" s="82">
-      <c r="A96" s="9" t="n"/>
-      <c r="B96" s="100" t="inlineStr">
+    <row r="95" ht="165" customHeight="1" s="82">
+      <c r="A95" s="19" t="n"/>
+      <c r="B95" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-23</t>
+        </is>
+      </c>
+      <c r="C95" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
+        <v/>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
+        <is>
+          <t>- Identify entry points where the application accepts serialized objects from untrusted
+- urces (for example, HTTP headers, parameters, or cookies).
+- Determine the serialization format used by the application.
+- Assess whether serialized input is validated or restricted prior to deserialization.
+- Evaluate whether manipulation of serialized data leads to unsafe behavior or security
+- pact.</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="n"/>
+    </row>
+    <row r="96" ht="15" customHeight="1" s="82">
+      <c r="A96" s="97" t="n"/>
+      <c r="B96" s="98" t="n"/>
+      <c r="C96" s="99" t="n"/>
+      <c r="D96" s="99" t="n"/>
+      <c r="E96" s="99" t="n"/>
+      <c r="F96" s="99" t="n"/>
+    </row>
+    <row r="97" ht="47.25" customHeight="1" s="82">
+      <c r="A97" s="9" t="n"/>
+      <c r="B97" s="100" t="inlineStr">
         <is>
           <t>Testing for Error Handling</t>
         </is>
       </c>
-      <c r="C96" s="101" t="inlineStr">
+      <c r="C97" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D96" s="101" t="inlineStr">
+      <c r="D97" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E96" s="101" t="inlineStr">
+      <c r="E97" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F96" s="101" t="inlineStr">
+      <c r="F97" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="33" customHeight="1" s="82">
-      <c r="A97" s="19" t="n"/>
-      <c r="B97" s="34" t="inlineStr">
+    <row r="98" ht="33" customHeight="1" s="82">
+      <c r="A98" s="19" t="n"/>
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C97" s="15">
+      <c r="C98" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="D98" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E97" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F97" s="18" t="n"/>
-    </row>
-    <row r="98" ht="16.5" customHeight="1" s="82">
-      <c r="A98" s="19" t="n"/>
-      <c r="B98" s="34" t="inlineStr">
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="n"/>
+    </row>
+    <row r="99" ht="16.5" customHeight="1" s="82">
+      <c r="A99" s="19" t="n"/>
+      <c r="B99" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C98" s="15">
+      <c r="C99" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
         <v/>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D99" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="n"/>
-    </row>
-    <row r="99" ht="15" customHeight="1" s="82">
-      <c r="A99" s="97" t="n"/>
-      <c r="B99" s="98" t="n"/>
-      <c r="C99" s="99" t="n"/>
-      <c r="D99" s="99" t="n"/>
-      <c r="E99" s="99" t="n"/>
-      <c r="F99" s="99" t="n"/>
-    </row>
-    <row r="100" ht="47.25" customHeight="1" s="82">
-      <c r="A100" s="9" t="n"/>
-      <c r="B100" s="100" t="inlineStr">
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="n"/>
+    </row>
+    <row r="100" ht="15" customHeight="1" s="82">
+      <c r="A100" s="97" t="n"/>
+      <c r="B100" s="98" t="n"/>
+      <c r="C100" s="99" t="n"/>
+      <c r="D100" s="99" t="n"/>
+      <c r="E100" s="99" t="n"/>
+      <c r="F100" s="99" t="n"/>
+    </row>
+    <row r="101" ht="47.25" customHeight="1" s="82">
+      <c r="A101" s="9" t="n"/>
+      <c r="B101" s="100" t="inlineStr">
         <is>
           <t>Testing for Weak Cryptography</t>
         </is>
       </c>
-      <c r="C100" s="101" t="inlineStr">
+      <c r="C101" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D100" s="101" t="inlineStr">
+      <c r="D101" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E100" s="101" t="inlineStr">
+      <c r="E101" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F100" s="101" t="inlineStr">
+      <c r="F101" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="82.5" customHeight="1" s="82">
-      <c r="A101" s="19" t="n"/>
-      <c r="B101" s="34" t="inlineStr">
+    <row r="102" ht="82.5" customHeight="1" s="82">
+      <c r="A102" s="19" t="n"/>
+      <c r="B102" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C101" s="15">
+      <c r="C102" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D101" s="16" t="inlineStr">
+      <c r="D102" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
-      <c r="E101" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F101" s="18" t="n"/>
-    </row>
-    <row r="102" ht="49.5" customHeight="1" s="82">
-      <c r="A102" s="19" t="n"/>
-      <c r="B102" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-02</t>
-        </is>
-      </c>
-      <c r="C102" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
-        <v/>
-      </c>
-      <c r="D102" s="16" t="inlineStr">
-        <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
-        </is>
-      </c>
       <c r="E102" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3768,146 +3772,170 @@
       <c r="A103" s="19" t="n"/>
       <c r="B103" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C103" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="n"/>
+    </row>
+    <row r="104" ht="49.5" customHeight="1" s="82">
+      <c r="A104" s="19" t="n"/>
+      <c r="B104" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CRYP-03</t>
         </is>
       </c>
-      <c r="C103" s="15">
+      <c r="C104" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
-      <c r="D103" s="16" t="inlineStr">
+      <c r="D104" s="16" t="inlineStr">
         <is>
           <t>- Identify sensitive information transmitted through the various channels.
 - Assess the privacy and security of the channels used.</t>
         </is>
       </c>
-      <c r="E103" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F103" s="18" t="n"/>
-    </row>
-    <row r="104" ht="33" customHeight="1" s="82">
-      <c r="A104" s="19" t="n"/>
-      <c r="B104" s="34" t="inlineStr">
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="n"/>
+    </row>
+    <row r="105" ht="33" customHeight="1" s="82">
+      <c r="A105" s="19" t="n"/>
+      <c r="B105" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-04</t>
         </is>
       </c>
-      <c r="C104" s="15">
+      <c r="C105" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="D105" s="16" t="inlineStr">
         <is>
           <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
-      <c r="E104" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F104" s="18" t="n"/>
-    </row>
-    <row r="105" ht="15" customHeight="1" s="82">
-      <c r="A105" s="97" t="n"/>
-      <c r="B105" s="98" t="n"/>
-      <c r="C105" s="99" t="n"/>
-      <c r="D105" s="99" t="n"/>
-      <c r="E105" s="99" t="n"/>
-      <c r="F105" s="99" t="n"/>
-    </row>
-    <row r="106" ht="47.25" customHeight="1" s="82">
-      <c r="A106" s="9" t="n"/>
-      <c r="B106" s="100" t="inlineStr">
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="n"/>
+    </row>
+    <row r="106" ht="15" customHeight="1" s="82">
+      <c r="A106" s="97" t="n"/>
+      <c r="B106" s="98" t="n"/>
+      <c r="C106" s="99" t="n"/>
+      <c r="D106" s="99" t="n"/>
+      <c r="E106" s="99" t="n"/>
+      <c r="F106" s="99" t="n"/>
+    </row>
+    <row r="107" ht="47.25" customHeight="1" s="82">
+      <c r="A107" s="9" t="n"/>
+      <c r="B107" s="100" t="inlineStr">
         <is>
           <t>Business Logic Testing</t>
         </is>
       </c>
-      <c r="C106" s="101" t="inlineStr">
+      <c r="C107" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D106" s="101" t="inlineStr">
+      <c r="D107" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E106" s="101" t="inlineStr">
+      <c r="E107" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F106" s="101" t="inlineStr">
+      <c r="F107" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="82.5" customHeight="1" s="82">
-      <c r="A107" s="19" t="n"/>
-      <c r="B107" s="34" t="inlineStr">
+    <row r="108" ht="82.5" customHeight="1" s="82">
+      <c r="A108" s="19" t="n"/>
+      <c r="B108" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C107" s="15">
+      <c r="C108" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D107" s="16" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E107" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F107" s="18" t="n"/>
-    </row>
-    <row r="108" ht="66" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="n"/>
+    </row>
+    <row r="109" ht="66" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C109" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="148.5" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="148.5" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C110" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3915,147 +3943,147 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="49.5" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="n"/>
+    </row>
+    <row r="111" ht="49.5" customHeight="1" s="82">
+      <c r="A111" s="19" t="n"/>
+      <c r="B111" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-04</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C111" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D111" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for system functionality that may be impacted by time.
 - Develop and execute misuse cases.</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F110" s="18" t="n"/>
-    </row>
-    <row r="111" ht="66" customHeight="1" s="82">
-      <c r="A111" s="19" t="n"/>
-      <c r="B111" s="34" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="n"/>
+    </row>
+    <row r="112" ht="66" customHeight="1" s="82">
+      <c r="A112" s="19" t="n"/>
+      <c r="B112" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-05</t>
         </is>
       </c>
-      <c r="C111" s="15">
+      <c r="C112" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D112" s="16" t="inlineStr">
         <is>
           <t>- Identify functions that must set limits to the times they can be called.
 - Assess if there is a logical limit set on the functions and if it is properly validated.</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F111" s="18" t="n"/>
-    </row>
-    <row r="112" ht="82.5" customHeight="1" s="82">
-      <c r="A112" s="19" t="n"/>
-      <c r="B112" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="82.5" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-06</t>
         </is>
       </c>
-      <c r="C112" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
         <v/>
       </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
 - Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="99" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="99" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-07</t>
         </is>
       </c>
-      <c r="C113" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
         <v/>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="99" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="99" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C114" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D114" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="165" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="165" customHeight="1" s="82">
+      <c r="A116" s="19" t="n"/>
+      <c r="B116" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C116" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4065,114 +4093,91 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="66" customHeight="1" s="82">
-      <c r="A116" s="19" t="n"/>
-      <c r="B116" s="34" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="n"/>
+    </row>
+    <row r="117" ht="66" customHeight="1" s="82">
+      <c r="A117" s="19" t="n"/>
+      <c r="B117" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C116" s="15">
+      <c r="C117" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D116" s="16" t="inlineStr">
+      <c r="D117" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F116" s="18" t="n"/>
-    </row>
-    <row r="117" ht="15" customHeight="1" s="82">
-      <c r="A117" s="97" t="n"/>
-      <c r="B117" s="98" t="n"/>
-      <c r="C117" s="99" t="n"/>
-      <c r="D117" s="99" t="n"/>
-      <c r="E117" s="99" t="n"/>
-      <c r="F117" s="99" t="n"/>
-    </row>
-    <row r="118" ht="47.25" customHeight="1" s="82">
-      <c r="A118" s="9" t="n"/>
-      <c r="B118" s="100" t="inlineStr">
+      <c r="E117" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F117" s="18" t="n"/>
+    </row>
+    <row r="118" ht="15" customHeight="1" s="82">
+      <c r="A118" s="97" t="n"/>
+      <c r="B118" s="98" t="n"/>
+      <c r="C118" s="99" t="n"/>
+      <c r="D118" s="99" t="n"/>
+      <c r="E118" s="99" t="n"/>
+      <c r="F118" s="99" t="n"/>
+    </row>
+    <row r="119" ht="47.25" customHeight="1" s="82">
+      <c r="A119" s="9" t="n"/>
+      <c r="B119" s="100" t="inlineStr">
         <is>
           <t>Client-side Testing</t>
         </is>
       </c>
-      <c r="C118" s="101" t="inlineStr">
+      <c r="C119" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D118" s="101" t="inlineStr">
+      <c r="D119" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E118" s="101" t="inlineStr">
+      <c r="E119" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F118" s="101" t="inlineStr">
+      <c r="F119" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="33" customHeight="1" s="82">
-      <c r="A119" s="19" t="n"/>
-      <c r="B119" s="34" t="inlineStr">
+    <row r="120" ht="33" customHeight="1" s="82">
+      <c r="A120" s="19" t="n"/>
+      <c r="B120" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-01</t>
         </is>
       </c>
-      <c r="C119" s="15">
+      <c r="C120" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D119" s="16" t="inlineStr">
+      <c r="D120" s="16" t="inlineStr">
         <is>
           <t>- Identify DOM sinks.
 - Build payloads that pertain to every sink type.</t>
         </is>
       </c>
-      <c r="E119" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F119" s="18" t="n"/>
-    </row>
-    <row r="120" ht="16.5" customHeight="1" s="82">
-      <c r="A120" s="19" t="n"/>
-      <c r="B120" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-02</t>
-        </is>
-      </c>
-      <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
-        <v/>
-      </c>
-      <c r="D120" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
-        </is>
-      </c>
       <c r="E120" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4180,20 +4185,20 @@
       </c>
       <c r="F120" s="18" t="n"/>
     </row>
-    <row r="121" ht="33" customHeight="1" s="82">
+    <row r="121" ht="16.5" customHeight="1" s="82">
       <c r="A121" s="19" t="n"/>
       <c r="B121" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-02</t>
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr">
@@ -4207,17 +4212,16 @@
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4231,17 +4235,17 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4255,17 +4259,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4279,42 +4283,43 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-06</t>
+        </is>
+      </c>
+      <c r="C125" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <v/>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
+        </is>
+      </c>
+      <c r="E125" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F125" s="18" t="n"/>
+    </row>
+    <row r="126" ht="33" customHeight="1" s="82">
+      <c r="A126" s="19" t="n"/>
+      <c r="B126" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-07</t>
         </is>
       </c>
-      <c r="C125" s="15">
+      <c r="C126" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
         <v/>
       </c>
-      <c r="D125" s="16" t="inlineStr">
+      <c r="D126" s="16" t="inlineStr">
         <is>
           <t>- Identify endpoints that implement CORS.
 - Ensure that the CORS configuration is secure or harmless.</t>
         </is>
       </c>
-      <c r="E125" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F125" s="18" t="n"/>
-    </row>
-    <row r="126" ht="16.5" customHeight="1" s="82">
-      <c r="A126" s="19" t="n"/>
-      <c r="B126" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-09</t>
-        </is>
-      </c>
-      <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
-        <v/>
-      </c>
-      <c r="D126" s="16" t="inlineStr">
-        <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
-        </is>
-      </c>
       <c r="E126" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4322,21 +4327,20 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="49.5" customHeight="1" s="82">
+    <row r="127" ht="16.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4350,90 +4354,91 @@
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-10</t>
+        </is>
+      </c>
+      <c r="C128" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <v/>
+      </c>
+      <c r="D128" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="n"/>
+    </row>
+    <row r="129" ht="49.5" customHeight="1" s="82">
+      <c r="A129" s="19" t="n"/>
+      <c r="B129" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-11</t>
         </is>
       </c>
-      <c r="C128" s="15">
+      <c r="C129" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
-      <c r="D128" s="16" t="inlineStr">
+      <c r="D129" s="16" t="inlineStr">
         <is>
           <t>- Assess the security of the message's origin.
 - Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
-      <c r="E128" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F128" s="18" t="n"/>
-    </row>
-    <row r="129" ht="82.5" customHeight="1" s="82">
-      <c r="A129" s="19" t="n"/>
-      <c r="B129" s="34" t="inlineStr">
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="n"/>
+    </row>
+    <row r="130" ht="82.5" customHeight="1" s="82">
+      <c r="A130" s="19" t="n"/>
+      <c r="B130" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-12</t>
         </is>
       </c>
-      <c r="C129" s="15">
+      <c r="C130" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the site is storing sensitive data in client-side storage.
 - The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F129" s="18" t="n"/>
-    </row>
-    <row r="130" ht="49.5" customHeight="1" s="82">
-      <c r="A130" s="19" t="n"/>
-      <c r="B130" s="34" t="inlineStr">
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="n"/>
+    </row>
+    <row r="131" ht="49.5" customHeight="1" s="82">
+      <c r="A131" s="19" t="n"/>
+      <c r="B131" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-13</t>
         </is>
       </c>
-      <c r="C130" s="15">
+      <c r="C131" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
-      <c r="D130" s="16" t="inlineStr">
+      <c r="D131" s="16" t="inlineStr">
         <is>
           <t>- Locate sensitive data across the system.
 - Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F130" s="18" t="n"/>
-    </row>
-    <row r="131" ht="16.5" customHeight="1" s="82">
-      <c r="A131" s="19" t="n"/>
-      <c r="B131" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D131" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E131" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4441,108 +4446,108 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="99" customHeight="1" s="82">
+    <row r="132" ht="16.5" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-14</t>
+        </is>
+      </c>
+      <c r="C132" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <v/>
+      </c>
+      <c r="D132" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="99" customHeight="1" s="82">
+      <c r="A133" s="19" t="n"/>
+      <c r="B133" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-15</t>
         </is>
       </c>
-      <c r="C132" s="15">
+      <c r="C133" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D132" s="16" t="inlineStr">
+      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="15" customHeight="1" s="82">
-      <c r="A133" s="97" t="n"/>
-      <c r="B133" s="98" t="n"/>
-      <c r="C133" s="99" t="n"/>
-      <c r="D133" s="99" t="n"/>
-      <c r="E133" s="99" t="n"/>
-      <c r="F133" s="99" t="n"/>
-    </row>
-    <row r="134" ht="47.25" customHeight="1" s="82">
-      <c r="A134" s="9" t="n"/>
-      <c r="B134" s="100" t="inlineStr">
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="n"/>
+    </row>
+    <row r="134" ht="15" customHeight="1" s="82">
+      <c r="A134" s="97" t="n"/>
+      <c r="B134" s="98" t="n"/>
+      <c r="C134" s="99" t="n"/>
+      <c r="D134" s="99" t="n"/>
+      <c r="E134" s="99" t="n"/>
+      <c r="F134" s="99" t="n"/>
+    </row>
+    <row r="135" ht="47.25" customHeight="1" s="82">
+      <c r="A135" s="9" t="n"/>
+      <c r="B135" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C134" s="101" t="inlineStr">
+      <c r="C135" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D134" s="101" t="inlineStr">
+      <c r="D135" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E134" s="101" t="inlineStr">
+      <c r="E135" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F134" s="101" t="inlineStr">
+      <c r="F135" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="99" customHeight="1" s="82">
-      <c r="A135" s="19" t="n"/>
-      <c r="B135" s="34" t="inlineStr">
+    <row r="136" ht="99" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C135" s="15">
+      <c r="C136" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D135" s="16" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E135" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F135" s="18" t="n"/>
-    </row>
-    <row r="136" ht="66" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-02</t>
-        </is>
-      </c>
-      <c r="C136" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D136" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
       <c r="E136" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4550,47 +4555,47 @@
       </c>
       <c r="F136" s="18" t="n"/>
     </row>
-    <row r="137" ht="132" customHeight="1" s="82">
+    <row r="137" ht="66" customHeight="1" s="82">
       <c r="A137" s="19" t="n"/>
       <c r="B137" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C137" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="132" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C137" s="15">
+      <c r="C138" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="82.5" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-04</t>
-        </is>
-      </c>
-      <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D138" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
       <c r="E138" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4598,38 +4603,61 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="66" customHeight="1" s="82">
+    <row r="139" ht="82.5" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C139" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="66" customHeight="1" s="82">
+      <c r="A140" s="19" t="n"/>
+      <c r="B140" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C140" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="82">
-      <c r="A140" s="97" t="n"/>
-      <c r="B140" s="98" t="n"/>
-      <c r="C140" s="99" t="n"/>
-      <c r="D140" s="99" t="n"/>
-      <c r="E140" s="99" t="n"/>
-      <c r="F140" s="99" t="n"/>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="82">
+      <c r="A141" s="97" t="n"/>
+      <c r="B141" s="98" t="n"/>
+      <c r="C141" s="99" t="n"/>
+      <c r="D141" s="99" t="n"/>
+      <c r="E141" s="99" t="n"/>
+      <c r="F141" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4646,7 +4674,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F140">
+  <conditionalFormatting sqref="B4:F141">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4658,7 +4686,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-08-10 (#1466)
Updates based on OWASP/wstg@de89650
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1461,7 +1461,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="82" min="1" max="1"/>
@@ -3596,167 +3596,171 @@
       </c>
       <c r="F94" s="18" t="n"/>
     </row>
-    <row r="95" ht="15" customHeight="1" s="82">
-      <c r="A95" s="97" t="n"/>
-      <c r="B95" s="98" t="n"/>
-      <c r="C95" s="99" t="n"/>
-      <c r="D95" s="99" t="n"/>
-      <c r="E95" s="99" t="n"/>
-      <c r="F95" s="99" t="n"/>
-    </row>
-    <row r="96" ht="47.25" customHeight="1" s="82">
-      <c r="A96" s="9" t="n"/>
-      <c r="B96" s="100" t="inlineStr">
+    <row r="95" ht="165" customHeight="1" s="82">
+      <c r="A95" s="19" t="n"/>
+      <c r="B95" s="34" t="inlineStr">
+        <is>
+          <t>WSTG-INPV-23</t>
+        </is>
+      </c>
+      <c r="C95" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
+        <v/>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
+        <is>
+          <t>- Identify entry points where the application accepts serialized objects from untrusted
+- urces (for example, HTTP headers, parameters, or cookies).
+- Determine the serialization format used by the application.
+- Assess whether serialized input is validated or restricted prior to deserialization.
+- Evaluate whether manipulation of serialized data leads to unsafe behavior or security
+- pact.</t>
+        </is>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F95" s="18" t="n"/>
+    </row>
+    <row r="96" ht="15" customHeight="1" s="82">
+      <c r="A96" s="97" t="n"/>
+      <c r="B96" s="98" t="n"/>
+      <c r="C96" s="99" t="n"/>
+      <c r="D96" s="99" t="n"/>
+      <c r="E96" s="99" t="n"/>
+      <c r="F96" s="99" t="n"/>
+    </row>
+    <row r="97" ht="47.25" customHeight="1" s="82">
+      <c r="A97" s="9" t="n"/>
+      <c r="B97" s="100" t="inlineStr">
         <is>
           <t>Testing for Error Handling</t>
         </is>
       </c>
-      <c r="C96" s="101" t="inlineStr">
+      <c r="C97" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D96" s="101" t="inlineStr">
+      <c r="D97" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E96" s="101" t="inlineStr">
+      <c r="E97" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F96" s="101" t="inlineStr">
+      <c r="F97" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="33" customHeight="1" s="82">
-      <c r="A97" s="19" t="n"/>
-      <c r="B97" s="34" t="inlineStr">
+    <row r="98" ht="33" customHeight="1" s="82">
+      <c r="A98" s="19" t="n"/>
+      <c r="B98" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-01</t>
         </is>
       </c>
-      <c r="C97" s="15">
+      <c r="C98" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
         <v/>
       </c>
-      <c r="D97" s="16" t="inlineStr">
+      <c r="D98" s="16" t="inlineStr">
         <is>
           <t>- Identify existing error output.
 - Analyze the different output returned.</t>
         </is>
       </c>
-      <c r="E97" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F97" s="18" t="n"/>
-    </row>
-    <row r="98" ht="16.5" customHeight="1" s="82">
-      <c r="A98" s="19" t="n"/>
-      <c r="B98" s="34" t="inlineStr">
+      <c r="E98" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F98" s="18" t="n"/>
+    </row>
+    <row r="99" ht="16.5" customHeight="1" s="82">
+      <c r="A99" s="19" t="n"/>
+      <c r="B99" s="34" t="inlineStr">
         <is>
           <t>WSTG-ERRH-02</t>
         </is>
       </c>
-      <c r="C98" s="15">
+      <c r="C99" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
         <v/>
       </c>
-      <c r="D98" s="16" t="inlineStr">
+      <c r="D99" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E98" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F98" s="18" t="n"/>
-    </row>
-    <row r="99" ht="15" customHeight="1" s="82">
-      <c r="A99" s="97" t="n"/>
-      <c r="B99" s="98" t="n"/>
-      <c r="C99" s="99" t="n"/>
-      <c r="D99" s="99" t="n"/>
-      <c r="E99" s="99" t="n"/>
-      <c r="F99" s="99" t="n"/>
-    </row>
-    <row r="100" ht="47.25" customHeight="1" s="82">
-      <c r="A100" s="9" t="n"/>
-      <c r="B100" s="100" t="inlineStr">
+      <c r="E99" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F99" s="18" t="n"/>
+    </row>
+    <row r="100" ht="15" customHeight="1" s="82">
+      <c r="A100" s="97" t="n"/>
+      <c r="B100" s="98" t="n"/>
+      <c r="C100" s="99" t="n"/>
+      <c r="D100" s="99" t="n"/>
+      <c r="E100" s="99" t="n"/>
+      <c r="F100" s="99" t="n"/>
+    </row>
+    <row r="101" ht="47.25" customHeight="1" s="82">
+      <c r="A101" s="9" t="n"/>
+      <c r="B101" s="100" t="inlineStr">
         <is>
           <t>Testing for Weak Cryptography</t>
         </is>
       </c>
-      <c r="C100" s="101" t="inlineStr">
+      <c r="C101" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D100" s="101" t="inlineStr">
+      <c r="D101" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E100" s="101" t="inlineStr">
+      <c r="E101" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F100" s="101" t="inlineStr">
+      <c r="F101" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="82.5" customHeight="1" s="82">
-      <c r="A101" s="19" t="n"/>
-      <c r="B101" s="34" t="inlineStr">
+    <row r="102" ht="82.5" customHeight="1" s="82">
+      <c r="A102" s="19" t="n"/>
+      <c r="B102" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-01</t>
         </is>
       </c>
-      <c r="C101" s="15">
+      <c r="C102" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
         <v/>
       </c>
-      <c r="D101" s="16" t="inlineStr">
+      <c r="D102" s="16" t="inlineStr">
         <is>
           <t>- Validate the service configuration.
 - Review the digital certificate's cryptographic strength and validity.
 - Ensure that the TLS security is not bypassable and is properly implemented across the application.</t>
         </is>
       </c>
-      <c r="E101" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F101" s="18" t="n"/>
-    </row>
-    <row r="102" ht="49.5" customHeight="1" s="82">
-      <c r="A102" s="19" t="n"/>
-      <c r="B102" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CRYP-02</t>
-        </is>
-      </c>
-      <c r="C102" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
-        <v/>
-      </c>
-      <c r="D102" s="16" t="inlineStr">
-        <is>
-          <t>- Identify encrypted messages that rely on padding.
-- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
-        </is>
-      </c>
       <c r="E102" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -3768,146 +3772,170 @@
       <c r="A103" s="19" t="n"/>
       <c r="B103" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CRYP-02</t>
+        </is>
+      </c>
+      <c r="C103" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <v/>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>- Identify encrypted messages that rely on padding.
+- Attempt to break the padding of the encrypted messages and analyze the returned error messages for further analysis.</t>
+        </is>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F103" s="18" t="n"/>
+    </row>
+    <row r="104" ht="49.5" customHeight="1" s="82">
+      <c r="A104" s="19" t="n"/>
+      <c r="B104" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CRYP-03</t>
         </is>
       </c>
-      <c r="C103" s="15">
+      <c r="C104" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
-      <c r="D103" s="16" t="inlineStr">
+      <c r="D104" s="16" t="inlineStr">
         <is>
           <t>- Identify sensitive information transmitted through the various channels.
 - Assess the privacy and security of the channels used.</t>
         </is>
       </c>
-      <c r="E103" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F103" s="18" t="n"/>
-    </row>
-    <row r="104" ht="33" customHeight="1" s="82">
-      <c r="A104" s="19" t="n"/>
-      <c r="B104" s="34" t="inlineStr">
+      <c r="E104" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F104" s="18" t="n"/>
+    </row>
+    <row r="105" ht="33" customHeight="1" s="82">
+      <c r="A105" s="19" t="n"/>
+      <c r="B105" s="34" t="inlineStr">
         <is>
           <t>WSTG-CRYP-04</t>
         </is>
       </c>
-      <c r="C104" s="15">
+      <c r="C105" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
         <v/>
       </c>
-      <c r="D104" s="16" t="inlineStr">
+      <c r="D105" s="16" t="inlineStr">
         <is>
           <t>- Provide a guideline for the identification weak encryption or hashing uses and implementations.</t>
         </is>
       </c>
-      <c r="E104" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F104" s="18" t="n"/>
-    </row>
-    <row r="105" ht="15" customHeight="1" s="82">
-      <c r="A105" s="97" t="n"/>
-      <c r="B105" s="98" t="n"/>
-      <c r="C105" s="99" t="n"/>
-      <c r="D105" s="99" t="n"/>
-      <c r="E105" s="99" t="n"/>
-      <c r="F105" s="99" t="n"/>
-    </row>
-    <row r="106" ht="47.25" customHeight="1" s="82">
-      <c r="A106" s="9" t="n"/>
-      <c r="B106" s="100" t="inlineStr">
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F105" s="18" t="n"/>
+    </row>
+    <row r="106" ht="15" customHeight="1" s="82">
+      <c r="A106" s="97" t="n"/>
+      <c r="B106" s="98" t="n"/>
+      <c r="C106" s="99" t="n"/>
+      <c r="D106" s="99" t="n"/>
+      <c r="E106" s="99" t="n"/>
+      <c r="F106" s="99" t="n"/>
+    </row>
+    <row r="107" ht="47.25" customHeight="1" s="82">
+      <c r="A107" s="9" t="n"/>
+      <c r="B107" s="100" t="inlineStr">
         <is>
           <t>Business Logic Testing</t>
         </is>
       </c>
-      <c r="C106" s="101" t="inlineStr">
+      <c r="C107" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D106" s="101" t="inlineStr">
+      <c r="D107" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E106" s="101" t="inlineStr">
+      <c r="E107" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F106" s="101" t="inlineStr">
+      <c r="F107" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="82.5" customHeight="1" s="82">
-      <c r="A107" s="19" t="n"/>
-      <c r="B107" s="34" t="inlineStr">
+    <row r="108" ht="82.5" customHeight="1" s="82">
+      <c r="A108" s="19" t="n"/>
+      <c r="B108" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-01</t>
         </is>
       </c>
-      <c r="C107" s="15">
+      <c r="C108" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
         <v/>
       </c>
-      <c r="D107" s="16" t="inlineStr">
+      <c r="D108" s="16" t="inlineStr">
         <is>
           <t>- Identify data injection points.
 - Validate that all checks are occurring on the backend and can't be bypassed.
 - Attempt to break the format of the expected data and analyze how the application is handling it.</t>
         </is>
       </c>
-      <c r="E107" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F107" s="18" t="n"/>
-    </row>
-    <row r="108" ht="66" customHeight="1" s="82">
-      <c r="A108" s="19" t="n"/>
-      <c r="B108" s="34" t="inlineStr">
+      <c r="E108" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F108" s="18" t="n"/>
+    </row>
+    <row r="109" ht="66" customHeight="1" s="82">
+      <c r="A109" s="19" t="n"/>
+      <c r="B109" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-02</t>
         </is>
       </c>
-      <c r="C108" s="15">
+      <c r="C109" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
         <v/>
       </c>
-      <c r="D108" s="16" t="inlineStr">
+      <c r="D109" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation looking for guessable, predictable, or hidden functionality of fields.
 - Insert logically valid data in order to bypass normal business logic workflow.</t>
         </is>
       </c>
-      <c r="E108" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F108" s="18" t="n"/>
-    </row>
-    <row r="109" ht="148.5" customHeight="1" s="82">
-      <c r="A109" s="19" t="n"/>
-      <c r="B109" s="34" t="inlineStr">
+      <c r="E109" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F109" s="18" t="n"/>
+    </row>
+    <row r="110" ht="148.5" customHeight="1" s="82">
+      <c r="A110" s="19" t="n"/>
+      <c r="B110" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-03</t>
         </is>
       </c>
-      <c r="C109" s="15">
+      <c r="C110" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
         <v/>
       </c>
-      <c r="D109" s="16" t="inlineStr">
+      <c r="D110" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for components of the system that move, store, or handle data.
 - Determine what type of data is logically acceptable by the component and what types the system should guard against.
@@ -3915,147 +3943,147 @@
 - Attempt to insert, update, or delete data values used by each component that should not be allowed per the business logic workflow.</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F109" s="18" t="n"/>
-    </row>
-    <row r="110" ht="49.5" customHeight="1" s="82">
-      <c r="A110" s="19" t="n"/>
-      <c r="B110" s="34" t="inlineStr">
+      <c r="E110" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="n"/>
+    </row>
+    <row r="111" ht="49.5" customHeight="1" s="82">
+      <c r="A111" s="19" t="n"/>
+      <c r="B111" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-04</t>
         </is>
       </c>
-      <c r="C110" s="15">
+      <c r="C111" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
         <v/>
       </c>
-      <c r="D110" s="16" t="inlineStr">
+      <c r="D111" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for system functionality that may be impacted by time.
 - Develop and execute misuse cases.</t>
         </is>
       </c>
-      <c r="E110" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F110" s="18" t="n"/>
-    </row>
-    <row r="111" ht="66" customHeight="1" s="82">
-      <c r="A111" s="19" t="n"/>
-      <c r="B111" s="34" t="inlineStr">
+      <c r="E111" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F111" s="18" t="n"/>
+    </row>
+    <row r="112" ht="66" customHeight="1" s="82">
+      <c r="A112" s="19" t="n"/>
+      <c r="B112" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-05</t>
         </is>
       </c>
-      <c r="C111" s="15">
+      <c r="C112" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
-      <c r="D111" s="16" t="inlineStr">
+      <c r="D112" s="16" t="inlineStr">
         <is>
           <t>- Identify functions that must set limits to the times they can be called.
 - Assess if there is a logical limit set on the functions and if it is properly validated.</t>
         </is>
       </c>
-      <c r="E111" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F111" s="18" t="n"/>
-    </row>
-    <row r="112" ht="82.5" customHeight="1" s="82">
-      <c r="A112" s="19" t="n"/>
-      <c r="B112" s="34" t="inlineStr">
+      <c r="E112" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F112" s="18" t="n"/>
+    </row>
+    <row r="113" ht="82.5" customHeight="1" s="82">
+      <c r="A113" s="19" t="n"/>
+      <c r="B113" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-06</t>
         </is>
       </c>
-      <c r="C112" s="15">
+      <c r="C113" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
         <v/>
       </c>
-      <c r="D112" s="16" t="inlineStr">
+      <c r="D113" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for methods to skip or go through steps in the application process in a different order from the intended business logic flow.
 - Develop a misuse case and try to circumvent every logic flow identified.</t>
         </is>
       </c>
-      <c r="E112" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="n"/>
-    </row>
-    <row r="113" ht="99" customHeight="1" s="82">
-      <c r="A113" s="19" t="n"/>
-      <c r="B113" s="34" t="inlineStr">
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F113" s="18" t="n"/>
+    </row>
+    <row r="114" ht="99" customHeight="1" s="82">
+      <c r="A114" s="19" t="n"/>
+      <c r="B114" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-07</t>
         </is>
       </c>
-      <c r="C113" s="15">
+      <c r="C114" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
         <v/>
       </c>
-      <c r="D113" s="16" t="inlineStr">
+      <c r="D114" s="16" t="inlineStr">
         <is>
           <t>- Generate notes from all tests conducted against the system.
 - Review which tests had a different functionality based on aggressive input.
 - Understand the defenses in place and verify if they are enough to protect the system against bypassing techniques.</t>
         </is>
       </c>
-      <c r="E113" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F113" s="18" t="n"/>
-    </row>
-    <row r="114" ht="99" customHeight="1" s="82">
-      <c r="A114" s="19" t="n"/>
-      <c r="B114" s="34" t="inlineStr">
+      <c r="E114" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F114" s="18" t="n"/>
+    </row>
+    <row r="115" ht="99" customHeight="1" s="82">
+      <c r="A115" s="19" t="n"/>
+      <c r="B115" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-08</t>
         </is>
       </c>
-      <c r="C114" s="15">
+      <c r="C115" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
         <v/>
       </c>
-      <c r="D114" s="16" t="inlineStr">
+      <c r="D115" s="16" t="inlineStr">
         <is>
           <t>- Review the project documentation for file types that are rejected by the system.
 - Verify that the unwelcomed file types are rejected and handled safely.
 - Verify that file batch uploads are secure and do not allow any bypass against the set security measures.</t>
         </is>
       </c>
-      <c r="E114" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F114" s="18" t="n"/>
-    </row>
-    <row r="115" ht="165" customHeight="1" s="82">
-      <c r="A115" s="19" t="n"/>
-      <c r="B115" s="34" t="inlineStr">
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F115" s="18" t="n"/>
+    </row>
+    <row r="116" ht="165" customHeight="1" s="82">
+      <c r="A116" s="19" t="n"/>
+      <c r="B116" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-09</t>
         </is>
       </c>
-      <c r="C115" s="15">
+      <c r="C116" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
         <v/>
       </c>
-      <c r="D115" s="16" t="inlineStr">
+      <c r="D116" s="16" t="inlineStr">
         <is>
           <t>- Identify the file upload functionality.
 - Review the project documentation to identify what file types are considered acceptable, and what types would be considered dangerous or malicious.
@@ -4065,114 +4093,91 @@
 - Try to upload the malicious files to the application and determine whether it is accepted and processed.</t>
         </is>
       </c>
-      <c r="E115" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F115" s="18" t="n"/>
-    </row>
-    <row r="116" ht="66" customHeight="1" s="82">
-      <c r="A116" s="19" t="n"/>
-      <c r="B116" s="34" t="inlineStr">
+      <c r="E116" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F116" s="18" t="n"/>
+    </row>
+    <row r="117" ht="66" customHeight="1" s="82">
+      <c r="A117" s="19" t="n"/>
+      <c r="B117" s="34" t="inlineStr">
         <is>
           <t>WSTG-BUSL-10</t>
         </is>
       </c>
-      <c r="C116" s="15">
+      <c r="C117" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
         <v/>
       </c>
-      <c r="D116" s="16" t="inlineStr">
+      <c r="D117" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the business logic for the e-commerce functionality is robust.
 - Understand how the payment functionality works.
 - Determine whether the payment functionality is secure.</t>
         </is>
       </c>
-      <c r="E116" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F116" s="18" t="n"/>
-    </row>
-    <row r="117" ht="15" customHeight="1" s="82">
-      <c r="A117" s="97" t="n"/>
-      <c r="B117" s="98" t="n"/>
-      <c r="C117" s="99" t="n"/>
-      <c r="D117" s="99" t="n"/>
-      <c r="E117" s="99" t="n"/>
-      <c r="F117" s="99" t="n"/>
-    </row>
-    <row r="118" ht="47.25" customHeight="1" s="82">
-      <c r="A118" s="9" t="n"/>
-      <c r="B118" s="100" t="inlineStr">
+      <c r="E117" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F117" s="18" t="n"/>
+    </row>
+    <row r="118" ht="15" customHeight="1" s="82">
+      <c r="A118" s="97" t="n"/>
+      <c r="B118" s="98" t="n"/>
+      <c r="C118" s="99" t="n"/>
+      <c r="D118" s="99" t="n"/>
+      <c r="E118" s="99" t="n"/>
+      <c r="F118" s="99" t="n"/>
+    </row>
+    <row r="119" ht="47.25" customHeight="1" s="82">
+      <c r="A119" s="9" t="n"/>
+      <c r="B119" s="100" t="inlineStr">
         <is>
           <t>Client-side Testing</t>
         </is>
       </c>
-      <c r="C118" s="101" t="inlineStr">
+      <c r="C119" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D118" s="101" t="inlineStr">
+      <c r="D119" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E118" s="101" t="inlineStr">
+      <c r="E119" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F118" s="101" t="inlineStr">
+      <c r="F119" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="119" ht="33" customHeight="1" s="82">
-      <c r="A119" s="19" t="n"/>
-      <c r="B119" s="34" t="inlineStr">
+    <row r="120" ht="33" customHeight="1" s="82">
+      <c r="A120" s="19" t="n"/>
+      <c r="B120" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-01</t>
         </is>
       </c>
-      <c r="C119" s="15">
+      <c r="C120" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
-      <c r="D119" s="16" t="inlineStr">
+      <c r="D120" s="16" t="inlineStr">
         <is>
           <t>- Identify DOM sinks.
 - Build payloads that pertain to every sink type.</t>
         </is>
       </c>
-      <c r="E119" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F119" s="18" t="n"/>
-    </row>
-    <row r="120" ht="16.5" customHeight="1" s="82">
-      <c r="A120" s="19" t="n"/>
-      <c r="B120" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-02</t>
-        </is>
-      </c>
-      <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
-        <v/>
-      </c>
-      <c r="D120" s="16" t="inlineStr">
-        <is>
-          <t>- Identify sinks and possible JavaScript injection points.</t>
-        </is>
-      </c>
       <c r="E120" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4180,20 +4185,20 @@
       </c>
       <c r="F120" s="18" t="n"/>
     </row>
-    <row r="121" ht="33" customHeight="1" s="82">
+    <row r="121" ht="16.5" customHeight="1" s="82">
       <c r="A121" s="19" t="n"/>
       <c r="B121" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-03</t>
+          <t>WSTG-CLNT-02</t>
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
+          <t>- Identify sinks and possible JavaScript injection points.</t>
         </is>
       </c>
       <c r="E121" s="18" t="inlineStr">
@@ -4207,17 +4212,16 @@
       <c r="A122" s="19" t="n"/>
       <c r="B122" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-04</t>
+          <t>WSTG-CLNT-03</t>
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
         <is>
-          <t>- Identify injection points that handle URLs or paths.
-- Assess the locations that the system could redirect to.</t>
+          <t>- Identify HTML injection points and assess the severity of the injected content.</t>
         </is>
       </c>
       <c r="E122" s="18" t="inlineStr">
@@ -4231,17 +4235,17 @@
       <c r="A123" s="19" t="n"/>
       <c r="B123" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-05</t>
+          <t>WSTG-CLNT-04</t>
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>- Identify CSS injection points.
-- Assess the impact of the injection.</t>
+          <t>- Identify injection points that handle URLs or paths.
+- Assess the locations that the system could redirect to.</t>
         </is>
       </c>
       <c r="E123" s="18" t="inlineStr">
@@ -4255,17 +4259,17 @@
       <c r="A124" s="19" t="n"/>
       <c r="B124" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-06</t>
+          <t>WSTG-CLNT-05</t>
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
         <is>
-          <t>- Identify sinks with weak input validation.
-- Assess the impact of the resource manipulation.</t>
+          <t>- Identify CSS injection points.
+- Assess the impact of the injection.</t>
         </is>
       </c>
       <c r="E124" s="18" t="inlineStr">
@@ -4279,42 +4283,43 @@
       <c r="A125" s="19" t="n"/>
       <c r="B125" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-06</t>
+        </is>
+      </c>
+      <c r="C125" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <v/>
+      </c>
+      <c r="D125" s="16" t="inlineStr">
+        <is>
+          <t>- Identify sinks with weak input validation.
+- Assess the impact of the resource manipulation.</t>
+        </is>
+      </c>
+      <c r="E125" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F125" s="18" t="n"/>
+    </row>
+    <row r="126" ht="33" customHeight="1" s="82">
+      <c r="A126" s="19" t="n"/>
+      <c r="B126" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-07</t>
         </is>
       </c>
-      <c r="C125" s="15">
+      <c r="C126" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
         <v/>
       </c>
-      <c r="D125" s="16" t="inlineStr">
+      <c r="D126" s="16" t="inlineStr">
         <is>
           <t>- Identify endpoints that implement CORS.
 - Ensure that the CORS configuration is secure or harmless.</t>
         </is>
       </c>
-      <c r="E125" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F125" s="18" t="n"/>
-    </row>
-    <row r="126" ht="16.5" customHeight="1" s="82">
-      <c r="A126" s="19" t="n"/>
-      <c r="B126" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-09</t>
-        </is>
-      </c>
-      <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
-        <v/>
-      </c>
-      <c r="D126" s="16" t="inlineStr">
-        <is>
-          <t>- Assess application vulnerability to clickjacking attacks.</t>
-        </is>
-      </c>
       <c r="E126" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4322,21 +4327,20 @@
       </c>
       <c r="F126" s="18" t="n"/>
     </row>
-    <row r="127" ht="49.5" customHeight="1" s="82">
+    <row r="127" ht="16.5" customHeight="1" s="82">
       <c r="A127" s="19" t="n"/>
       <c r="B127" s="34" t="inlineStr">
         <is>
-          <t>WSTG-CLNT-10</t>
+          <t>WSTG-CLNT-09</t>
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>- Identify the usage of WebSockets.
-- Assess its implementation by using the same tests on normal HTTP channels.</t>
+          <t>- Assess application vulnerability to clickjacking attacks.</t>
         </is>
       </c>
       <c r="E127" s="18" t="inlineStr">
@@ -4350,90 +4354,91 @@
       <c r="A128" s="19" t="n"/>
       <c r="B128" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-10</t>
+        </is>
+      </c>
+      <c r="C128" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <v/>
+      </c>
+      <c r="D128" s="16" t="inlineStr">
+        <is>
+          <t>- Identify the usage of WebSockets.
+- Assess its implementation by using the same tests on normal HTTP channels.</t>
+        </is>
+      </c>
+      <c r="E128" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F128" s="18" t="n"/>
+    </row>
+    <row r="129" ht="49.5" customHeight="1" s="82">
+      <c r="A129" s="19" t="n"/>
+      <c r="B129" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-11</t>
         </is>
       </c>
-      <c r="C128" s="15">
+      <c r="C129" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
         <v/>
       </c>
-      <c r="D128" s="16" t="inlineStr">
+      <c r="D129" s="16" t="inlineStr">
         <is>
           <t>- Assess the security of the message's origin.
 - Validate that it's using safe methods and validating its input.</t>
         </is>
       </c>
-      <c r="E128" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F128" s="18" t="n"/>
-    </row>
-    <row r="129" ht="82.5" customHeight="1" s="82">
-      <c r="A129" s="19" t="n"/>
-      <c r="B129" s="34" t="inlineStr">
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F129" s="18" t="n"/>
+    </row>
+    <row r="130" ht="82.5" customHeight="1" s="82">
+      <c r="A130" s="19" t="n"/>
+      <c r="B130" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-12</t>
         </is>
       </c>
-      <c r="C129" s="15">
+      <c r="C130" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
         <v/>
       </c>
-      <c r="D129" s="16" t="inlineStr">
+      <c r="D130" s="16" t="inlineStr">
         <is>
           <t>- Determine whether the site is storing sensitive data in client-side storage.
 - The code handling of the storage objects should be examined for possibilities of injection attacks, such as utilizing unvalidated input or vulnerable libraries.</t>
         </is>
       </c>
-      <c r="E129" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F129" s="18" t="n"/>
-    </row>
-    <row r="130" ht="49.5" customHeight="1" s="82">
-      <c r="A130" s="19" t="n"/>
-      <c r="B130" s="34" t="inlineStr">
+      <c r="E130" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F130" s="18" t="n"/>
+    </row>
+    <row r="131" ht="49.5" customHeight="1" s="82">
+      <c r="A131" s="19" t="n"/>
+      <c r="B131" s="34" t="inlineStr">
         <is>
           <t>WSTG-CLNT-13</t>
         </is>
       </c>
-      <c r="C130" s="15">
+      <c r="C131" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
         <v/>
       </c>
-      <c r="D130" s="16" t="inlineStr">
+      <c r="D131" s="16" t="inlineStr">
         <is>
           <t>- Locate sensitive data across the system.
 - Assess the leakage of sensitive data through various techniques.</t>
         </is>
       </c>
-      <c r="E130" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F130" s="18" t="n"/>
-    </row>
-    <row r="131" ht="16.5" customHeight="1" s="82">
-      <c r="A131" s="19" t="n"/>
-      <c r="B131" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-CLNT-14</t>
-        </is>
-      </c>
-      <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
-        <v/>
-      </c>
-      <c r="D131" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E131" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4441,108 +4446,108 @@
       </c>
       <c r="F131" s="18" t="n"/>
     </row>
-    <row r="132" ht="99" customHeight="1" s="82">
+    <row r="132" ht="16.5" customHeight="1" s="82">
       <c r="A132" s="19" t="n"/>
       <c r="B132" s="34" t="inlineStr">
         <is>
+          <t>WSTG-CLNT-14</t>
+        </is>
+      </c>
+      <c r="C132" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <v/>
+      </c>
+      <c r="D132" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E132" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F132" s="18" t="n"/>
+    </row>
+    <row r="133" ht="99" customHeight="1" s="82">
+      <c r="A133" s="19" t="n"/>
+      <c r="B133" s="34" t="inlineStr">
+        <is>
           <t>WSTG-CLNT-15</t>
         </is>
       </c>
-      <c r="C132" s="15">
+      <c r="C133" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
         <v/>
       </c>
-      <c r="D132" s="16" t="inlineStr">
+      <c r="D133" s="16" t="inlineStr">
         <is>
           <t>- Identify the client-side framework and its version used by the application.
 - Detect injection points where user input is reflected into the DOM and processed by the template engine.
 - Assess if the injection allows for arbitrary JavaScript execution (XSS) via the template syntax.</t>
         </is>
       </c>
-      <c r="E132" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F132" s="18" t="n"/>
-    </row>
-    <row r="133" ht="15" customHeight="1" s="82">
-      <c r="A133" s="97" t="n"/>
-      <c r="B133" s="98" t="n"/>
-      <c r="C133" s="99" t="n"/>
-      <c r="D133" s="99" t="n"/>
-      <c r="E133" s="99" t="n"/>
-      <c r="F133" s="99" t="n"/>
-    </row>
-    <row r="134" ht="47.25" customHeight="1" s="82">
-      <c r="A134" s="9" t="n"/>
-      <c r="B134" s="100" t="inlineStr">
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F133" s="18" t="n"/>
+    </row>
+    <row r="134" ht="15" customHeight="1" s="82">
+      <c r="A134" s="97" t="n"/>
+      <c r="B134" s="98" t="n"/>
+      <c r="C134" s="99" t="n"/>
+      <c r="D134" s="99" t="n"/>
+      <c r="E134" s="99" t="n"/>
+      <c r="F134" s="99" t="n"/>
+    </row>
+    <row r="135" ht="47.25" customHeight="1" s="82">
+      <c r="A135" s="9" t="n"/>
+      <c r="B135" s="100" t="inlineStr">
         <is>
           <t>API Testing</t>
         </is>
       </c>
-      <c r="C134" s="101" t="inlineStr">
+      <c r="C135" s="101" t="inlineStr">
         <is>
           <t>Test Name</t>
         </is>
       </c>
-      <c r="D134" s="101" t="inlineStr">
+      <c r="D135" s="101" t="inlineStr">
         <is>
           <t>Objectives</t>
         </is>
       </c>
-      <c r="E134" s="101" t="inlineStr">
+      <c r="E135" s="101" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F134" s="101" t="inlineStr">
+      <c r="F135" s="101" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="99" customHeight="1" s="82">
-      <c r="A135" s="19" t="n"/>
-      <c r="B135" s="34" t="inlineStr">
+    <row r="136" ht="99" customHeight="1" s="82">
+      <c r="A136" s="19" t="n"/>
+      <c r="B136" s="34" t="inlineStr">
         <is>
           <t>WSTG-APIT-01</t>
         </is>
       </c>
-      <c r="C135" s="15">
+      <c r="C136" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/01-API_Reconnaissance", "API Reconnaissance")</f>
         <v/>
       </c>
-      <c r="D135" s="16" t="inlineStr">
+      <c r="D136" s="16" t="inlineStr">
         <is>
           <t>- Find all API endpoints supported by the backend server code, documented or undocumented.
 - Find all parameters for each endpoint supported by the backend server, documented or undocumented.
 - Discover interesting data related to APIs in HTML and JavaScript sent to clients.</t>
         </is>
       </c>
-      <c r="E135" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F135" s="18" t="n"/>
-    </row>
-    <row r="136" ht="66" customHeight="1" s="82">
-      <c r="A136" s="19" t="n"/>
-      <c r="B136" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-02</t>
-        </is>
-      </c>
-      <c r="C136" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D136" s="16" t="inlineStr">
-        <is>
-          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
-        </is>
-      </c>
       <c r="E136" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4550,47 +4555,47 @@
       </c>
       <c r="F136" s="18" t="n"/>
     </row>
-    <row r="137" ht="132" customHeight="1" s="82">
+    <row r="137" ht="66" customHeight="1" s="82">
       <c r="A137" s="19" t="n"/>
       <c r="B137" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-02</t>
+        </is>
+      </c>
+      <c r="C137" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/02-API_Broken_Object_Level_Authorization", "API Broken Object Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D137" s="16" t="inlineStr">
+        <is>
+          <t>- The objective of this test is to identify whether the API enforces proper **object-level authorization** checks, ensuring that users can only access and manipulate objects they are authorized to interact with.</t>
+        </is>
+      </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F137" s="18" t="n"/>
+    </row>
+    <row r="138" ht="132" customHeight="1" s="82">
+      <c r="A138" s="19" t="n"/>
+      <c r="B138" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-03</t>
         </is>
       </c>
-      <c r="C137" s="15">
+      <c r="C138" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
         <v/>
       </c>
-      <c r="D137" s="16" t="inlineStr">
+      <c r="D138" s="16" t="inlineStr">
         <is>
           <t>- Identify API responses that contain more data than what the client application displays or requires.
 - Detect sensitive fields returned in API responses such as password hashes, authentication tokens, internal object IDs, PII, or infrastructure details.
 - Determine whether the API relies on client-side filtering rather than server-side field selection to control data exposure.</t>
         </is>
       </c>
-      <c r="E137" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F137" s="18" t="n"/>
-    </row>
-    <row r="138" ht="82.5" customHeight="1" s="82">
-      <c r="A138" s="19" t="n"/>
-      <c r="B138" s="34" t="inlineStr">
-        <is>
-          <t>WSTG-APIT-04</t>
-        </is>
-      </c>
-      <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
-        <v/>
-      </c>
-      <c r="D138" s="16" t="inlineStr">
-        <is>
-          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
-        </is>
-      </c>
       <c r="E138" s="18" t="inlineStr">
         <is>
           <t>Not Started</t>
@@ -4598,38 +4603,61 @@
       </c>
       <c r="F138" s="18" t="n"/>
     </row>
-    <row r="139" ht="66" customHeight="1" s="82">
+    <row r="139" ht="82.5" customHeight="1" s="82">
       <c r="A139" s="19" t="n"/>
       <c r="B139" s="34" t="inlineStr">
         <is>
+          <t>WSTG-APIT-04</t>
+        </is>
+      </c>
+      <c r="C139" s="15">
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/04-API_Broken_Function_Level_Authorization", "API Broken Function Level Authorization")</f>
+        <v/>
+      </c>
+      <c r="D139" s="16" t="inlineStr">
+        <is>
+          <t>- The goal of this test is to determine if the API enforces **role or privilege-based access control** to restrict users from accessing or executing functions they are not authorized to use. This ensures that function-level security boundaries are properly enforced.</t>
+        </is>
+      </c>
+      <c r="E139" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" s="18" t="n"/>
+    </row>
+    <row r="140" ht="66" customHeight="1" s="82">
+      <c r="A140" s="19" t="n"/>
+      <c r="B140" s="34" t="inlineStr">
+        <is>
           <t>WSTG-APIT-99</t>
         </is>
       </c>
-      <c r="C139" s="15">
+      <c r="C140" s="15">
         <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
         <v/>
       </c>
-      <c r="D139" s="16" t="inlineStr">
+      <c r="D140" s="16" t="inlineStr">
         <is>
           <t>- Assess that a secure and production-ready configuration is deployed.
 - Validate all input fields against generic attacks.
 - Ensure that proper access controls are applied.</t>
         </is>
       </c>
-      <c r="E139" s="18" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F139" s="18" t="n"/>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="82">
-      <c r="A140" s="97" t="n"/>
-      <c r="B140" s="98" t="n"/>
-      <c r="C140" s="99" t="n"/>
-      <c r="D140" s="99" t="n"/>
-      <c r="E140" s="99" t="n"/>
-      <c r="F140" s="99" t="n"/>
+      <c r="E140" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F140" s="18" t="n"/>
+    </row>
+    <row r="141" ht="15" customHeight="1" s="82">
+      <c r="A141" s="97" t="n"/>
+      <c r="B141" s="98" t="n"/>
+      <c r="C141" s="99" t="n"/>
+      <c r="D141" s="99" t="n"/>
+      <c r="E141" s="99" t="n"/>
+      <c r="F141" s="99" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4646,7 +4674,7 @@
       <formula>$E4="Issues"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F140">
+  <conditionalFormatting sqref="B4:F141">
     <cfRule type="expression" priority="1" dxfId="13">
       <formula>$E4="Pass"</formula>
     </cfRule>
@@ -4658,7 +4686,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E97 E98 E101 E102 E103 E104 E107 E108 E109 E110 E111 E112 E113 E114 E115 E116 E119 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E135 E136 E137 E138 E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E4 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E18 E19 E20 E21 E22 E23 E24 E25 E26 E27 E28 E29 E30 E33 E34 E35 E36 E37 E40 E41 E42 E43 E44 E45 E46 E47 E48 E49 E50 E53 E54 E55 E56 E57 E60 E61 E62 E63 E64 E65 E66 E67 E68 E69 E70 E73 E74 E75 E76 E77 E78 E79 E80 E81 E82 E83 E84 E85 E86 E87 E88 E89 E90 E91 E92 E93 E94 E95 E98 E99 E102 E103 E104 E105 E108 E109 E110 E111 E112 E113 E114 E115 E116 E117 E120 E121 E122 E123 E124 E125 E126 E127 E128 E129 E130 E131 E132 E133 E136 E137 E138 E139 E140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,Pass,Issues,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-01
Updates based on OWASP/wstg@d3a6bc1
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/01-Conduct_Search_Engine_Discovery_Reconnaissance_for_Information_Leakage", "Conduct Search Engine Discovery Reconnaissance for Information Leakage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/01-Conduct_Search_Engine_Reconnaissance_for_Information_Leakage", "Conduct Search Engine Reconnaissance for Information Leakage")</f>
         <v/>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="C28" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Testing for Content Security Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Test for Content Security Policy")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-01 (#1494)
Updates based on OWASP/wstg@d3a6bc1
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/01-Conduct_Search_Engine_Discovery_Reconnaissance_for_Information_Leakage", "Conduct Search Engine Discovery Reconnaissance for Information Leakage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/01-Information_Gathering/01-Conduct_Search_Engine_Reconnaissance_for_Information_Leakage", "Conduct Search Engine Reconnaissance for Information Leakage")</f>
         <v/>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="C28" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Testing for Content Security Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Test for Content Security Policy")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-08
Updates based on OWASP/wstg@1a22f2d
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -3035,7 +3035,7 @@
       <c r="A72" s="9" t="n"/>
       <c r="B72" s="100" t="inlineStr">
         <is>
-          <t>Input Validation Testing</t>
+          <t>Injection Testing</t>
         </is>
       </c>
       <c r="C72" s="101" t="inlineStr">
@@ -3063,11 +3063,11 @@
       <c r="A73" s="19" t="n"/>
       <c r="B73" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-01</t>
+          <t>WSTG-INJT-01</t>
         </is>
       </c>
       <c r="C73" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -3087,11 +3087,11 @@
       <c r="A74" s="19" t="n"/>
       <c r="B74" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-02</t>
+          <t>WSTG-INJT-02</t>
         </is>
       </c>
       <c r="C74" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D74" s="16" t="inlineStr">
@@ -3111,11 +3111,11 @@
       <c r="A75" s="19" t="n"/>
       <c r="B75" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-03</t>
+          <t>WSTG-INJT-03</t>
         </is>
       </c>
       <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -3134,11 +3134,11 @@
       <c r="A76" s="19" t="n"/>
       <c r="B76" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-04</t>
+          <t>WSTG-INJT-04</t>
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
@@ -3158,11 +3158,11 @@
       <c r="A77" s="19" t="n"/>
       <c r="B77" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-05</t>
+          <t>WSTG-INJT-05</t>
         </is>
       </c>
       <c r="C77" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
         <v/>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -3182,11 +3182,11 @@
       <c r="A78" s="19" t="n"/>
       <c r="B78" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-06</t>
+          <t>WSTG-INJT-06</t>
         </is>
       </c>
       <c r="C78" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
         <v/>
       </c>
       <c r="D78" s="16" t="inlineStr">
@@ -3206,11 +3206,11 @@
       <c r="A79" s="19" t="n"/>
       <c r="B79" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-07</t>
+          <t>WSTG-INJT-07</t>
         </is>
       </c>
       <c r="C79" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
         <v/>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -3230,11 +3230,11 @@
       <c r="A80" s="19" t="n"/>
       <c r="B80" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-08</t>
+          <t>WSTG-INJT-08</t>
         </is>
       </c>
       <c r="C80" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
         <v/>
       </c>
       <c r="D80" s="16" t="inlineStr">
@@ -3254,11 +3254,11 @@
       <c r="A81" s="19" t="n"/>
       <c r="B81" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-09</t>
+          <t>WSTG-INJT-09</t>
         </is>
       </c>
       <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
         <v/>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -3277,11 +3277,11 @@
       <c r="A82" s="19" t="n"/>
       <c r="B82" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-10</t>
+          <t>WSTG-INJT-10</t>
         </is>
       </c>
       <c r="C82" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
         <v/>
       </c>
       <c r="D82" s="16" t="inlineStr">
@@ -3302,11 +3302,11 @@
       <c r="A83" s="19" t="n"/>
       <c r="B83" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-11</t>
+          <t>WSTG-INJT-11</t>
         </is>
       </c>
       <c r="C83" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
         <v/>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -3326,11 +3326,11 @@
       <c r="A84" s="19" t="n"/>
       <c r="B84" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-12</t>
+          <t>WSTG-INJT-12</t>
         </is>
       </c>
       <c r="C84" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
         <v/>
       </c>
       <c r="D84" s="16" t="inlineStr">
@@ -3350,11 +3350,11 @@
       <c r="A85" s="19" t="n"/>
       <c r="B85" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-13</t>
+          <t>WSTG-INJT-13</t>
         </is>
       </c>
       <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
         <v/>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -3373,11 +3373,11 @@
       <c r="A86" s="19" t="n"/>
       <c r="B86" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-14</t>
+          <t>WSTG-INJT-14</t>
         </is>
       </c>
       <c r="C86" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
         <v/>
       </c>
       <c r="D86" s="16" t="inlineStr">
@@ -3398,11 +3398,11 @@
       <c r="A87" s="19" t="n"/>
       <c r="B87" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-15</t>
+          <t>WSTG-INJT-15</t>
         </is>
       </c>
       <c r="C87" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
         <v/>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -3423,11 +3423,11 @@
       <c r="A88" s="19" t="n"/>
       <c r="B88" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-16</t>
+          <t>WSTG-INJT-16</t>
         </is>
       </c>
       <c r="C88" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
         <v/>
       </c>
       <c r="D88" s="16" t="inlineStr">
@@ -3450,11 +3450,11 @@
       <c r="A89" s="19" t="n"/>
       <c r="B89" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-17</t>
+          <t>WSTG-INJT-17</t>
         </is>
       </c>
       <c r="C89" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
         <v/>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -3474,11 +3474,11 @@
       <c r="A90" s="19" t="n"/>
       <c r="B90" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-18</t>
+          <t>WSTG-INJT-18</t>
         </is>
       </c>
       <c r="C90" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
         <v/>
       </c>
       <c r="D90" s="16" t="inlineStr">
@@ -3499,11 +3499,11 @@
       <c r="A91" s="19" t="n"/>
       <c r="B91" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-19</t>
+          <t>WSTG-INJT-19</t>
         </is>
       </c>
       <c r="C91" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
         <v/>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -3524,11 +3524,11 @@
       <c r="A92" s="19" t="n"/>
       <c r="B92" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-20</t>
+          <t>WSTG-INJT-20</t>
         </is>
       </c>
       <c r="C92" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
         <v/>
       </c>
       <c r="D92" s="16" t="inlineStr">
@@ -3548,11 +3548,11 @@
       <c r="A93" s="19" t="n"/>
       <c r="B93" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-21</t>
+          <t>WSTG-INJT-21</t>
         </is>
       </c>
       <c r="C93" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
         <v/>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -3575,11 +3575,11 @@
       <c r="A94" s="19" t="n"/>
       <c r="B94" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-22</t>
+          <t>WSTG-INJT-22</t>
         </is>
       </c>
       <c r="C94" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
         <v/>
       </c>
       <c r="D94" s="16" t="inlineStr">
@@ -3600,11 +3600,11 @@
       <c r="A95" s="19" t="n"/>
       <c r="B95" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-23</t>
+          <t>WSTG-INJT-23</t>
         </is>
       </c>
       <c r="C95" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
         <v/>
       </c>
       <c r="D95" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-08 (#1514)
Updates based on OWASP/wstg@1a22f2d
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -3035,7 +3035,7 @@
       <c r="A72" s="9" t="n"/>
       <c r="B72" s="100" t="inlineStr">
         <is>
-          <t>Input Validation Testing</t>
+          <t>Injection Testing</t>
         </is>
       </c>
       <c r="C72" s="101" t="inlineStr">
@@ -3063,11 +3063,11 @@
       <c r="A73" s="19" t="n"/>
       <c r="B73" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-01</t>
+          <t>WSTG-INJT-01</t>
         </is>
       </c>
       <c r="C73" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -3087,11 +3087,11 @@
       <c r="A74" s="19" t="n"/>
       <c r="B74" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-02</t>
+          <t>WSTG-INJT-02</t>
         </is>
       </c>
       <c r="C74" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D74" s="16" t="inlineStr">
@@ -3111,11 +3111,11 @@
       <c r="A75" s="19" t="n"/>
       <c r="B75" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-03</t>
+          <t>WSTG-INJT-03</t>
         </is>
       </c>
       <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -3134,11 +3134,11 @@
       <c r="A76" s="19" t="n"/>
       <c r="B76" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-04</t>
+          <t>WSTG-INJT-04</t>
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
@@ -3158,11 +3158,11 @@
       <c r="A77" s="19" t="n"/>
       <c r="B77" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-05</t>
+          <t>WSTG-INJT-05</t>
         </is>
       </c>
       <c r="C77" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
         <v/>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -3182,11 +3182,11 @@
       <c r="A78" s="19" t="n"/>
       <c r="B78" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-06</t>
+          <t>WSTG-INJT-06</t>
         </is>
       </c>
       <c r="C78" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
         <v/>
       </c>
       <c r="D78" s="16" t="inlineStr">
@@ -3206,11 +3206,11 @@
       <c r="A79" s="19" t="n"/>
       <c r="B79" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-07</t>
+          <t>WSTG-INJT-07</t>
         </is>
       </c>
       <c r="C79" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
         <v/>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -3230,11 +3230,11 @@
       <c r="A80" s="19" t="n"/>
       <c r="B80" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-08</t>
+          <t>WSTG-INJT-08</t>
         </is>
       </c>
       <c r="C80" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
         <v/>
       </c>
       <c r="D80" s="16" t="inlineStr">
@@ -3254,11 +3254,11 @@
       <c r="A81" s="19" t="n"/>
       <c r="B81" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-09</t>
+          <t>WSTG-INJT-09</t>
         </is>
       </c>
       <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
         <v/>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -3277,11 +3277,11 @@
       <c r="A82" s="19" t="n"/>
       <c r="B82" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-10</t>
+          <t>WSTG-INJT-10</t>
         </is>
       </c>
       <c r="C82" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
         <v/>
       </c>
       <c r="D82" s="16" t="inlineStr">
@@ -3302,11 +3302,11 @@
       <c r="A83" s="19" t="n"/>
       <c r="B83" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-11</t>
+          <t>WSTG-INJT-11</t>
         </is>
       </c>
       <c r="C83" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
         <v/>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -3326,11 +3326,11 @@
       <c r="A84" s="19" t="n"/>
       <c r="B84" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-12</t>
+          <t>WSTG-INJT-12</t>
         </is>
       </c>
       <c r="C84" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
         <v/>
       </c>
       <c r="D84" s="16" t="inlineStr">
@@ -3350,11 +3350,11 @@
       <c r="A85" s="19" t="n"/>
       <c r="B85" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-13</t>
+          <t>WSTG-INJT-13</t>
         </is>
       </c>
       <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
         <v/>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -3373,11 +3373,11 @@
       <c r="A86" s="19" t="n"/>
       <c r="B86" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-14</t>
+          <t>WSTG-INJT-14</t>
         </is>
       </c>
       <c r="C86" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
         <v/>
       </c>
       <c r="D86" s="16" t="inlineStr">
@@ -3398,11 +3398,11 @@
       <c r="A87" s="19" t="n"/>
       <c r="B87" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-15</t>
+          <t>WSTG-INJT-15</t>
         </is>
       </c>
       <c r="C87" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
         <v/>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -3423,11 +3423,11 @@
       <c r="A88" s="19" t="n"/>
       <c r="B88" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-16</t>
+          <t>WSTG-INJT-16</t>
         </is>
       </c>
       <c r="C88" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
         <v/>
       </c>
       <c r="D88" s="16" t="inlineStr">
@@ -3450,11 +3450,11 @@
       <c r="A89" s="19" t="n"/>
       <c r="B89" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-17</t>
+          <t>WSTG-INJT-17</t>
         </is>
       </c>
       <c r="C89" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
         <v/>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -3474,11 +3474,11 @@
       <c r="A90" s="19" t="n"/>
       <c r="B90" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-18</t>
+          <t>WSTG-INJT-18</t>
         </is>
       </c>
       <c r="C90" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
         <v/>
       </c>
       <c r="D90" s="16" t="inlineStr">
@@ -3499,11 +3499,11 @@
       <c r="A91" s="19" t="n"/>
       <c r="B91" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-19</t>
+          <t>WSTG-INJT-19</t>
         </is>
       </c>
       <c r="C91" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
         <v/>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -3524,11 +3524,11 @@
       <c r="A92" s="19" t="n"/>
       <c r="B92" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-20</t>
+          <t>WSTG-INJT-20</t>
         </is>
       </c>
       <c r="C92" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
         <v/>
       </c>
       <c r="D92" s="16" t="inlineStr">
@@ -3548,11 +3548,11 @@
       <c r="A93" s="19" t="n"/>
       <c r="B93" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-21</t>
+          <t>WSTG-INJT-21</t>
         </is>
       </c>
       <c r="C93" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
         <v/>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -3575,11 +3575,11 @@
       <c r="A94" s="19" t="n"/>
       <c r="B94" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-22</t>
+          <t>WSTG-INJT-22</t>
         </is>
       </c>
       <c r="C94" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
         <v/>
       </c>
       <c r="D94" s="16" t="inlineStr">
@@ -3600,11 +3600,11 @@
       <c r="A95" s="19" t="n"/>
       <c r="B95" s="34" t="inlineStr">
         <is>
-          <t>WSTG-INPV-23</t>
+          <t>WSTG-INJT-23</t>
         </is>
       </c>
       <c r="C95" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Input_Validation_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
         <v/>
       </c>
       <c r="D95" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Publish Latest checklists 2026-09-10
Updates based on OWASP/wstg@0ec5295
</commit_message>
<xml_diff>
--- a/checklists/checklist.xlsx
+++ b/checklists/checklist.xlsx
@@ -1788,7 +1788,7 @@
       <c r="A17" s="9" t="n"/>
       <c r="B17" s="100" t="inlineStr">
         <is>
-          <t>Configuration and Deployment Management Testing</t>
+          <t>Configuration and Deployment Management</t>
         </is>
       </c>
       <c r="C17" s="101" t="inlineStr">
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="C18" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/01-Test_Network_Infrastructure_Configuration", "Test Network Infrastructure Configuration")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/01-Network_Infrastructure_Configuration", "Network Infrastructure Configuration")</f>
         <v/>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="C19" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/02-Test_Application_Platform_Configuration", "Test Application Platform Configuration")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/02-Application_Platform_Configuration", "Application Platform Configuration")</f>
         <v/>
       </c>
       <c r="D19" s="16" t="inlineStr">
@@ -1869,7 +1869,7 @@
         </is>
       </c>
       <c r="C20" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/03-Test_File_Extensions_Handling_for_Sensitive_Information", "Test File Extensions Handling for Sensitive Information")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/03-File_Extensions_Handling_for_Sensitive_Information", "File Extensions Handling for Sensitive Information")</f>
         <v/>
       </c>
       <c r="D20" s="16" t="inlineStr">
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="C21" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/04-Review_Old_Backup_and_Unreferenced_Files_for_Sensitive_Information", "Review Old Backup and Unreferenced Files for Sensitive Information")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/04-Review_Old_Backup_and_Unreferenced_Files_for_Sensitive_Information", "Review Old Backup and Unreferenced Files for Sensitive Information")</f>
         <v/>
       </c>
       <c r="D21" s="16" t="inlineStr">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="C22" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/05-Enumerate_Infrastructure_and_Application_Admin_Interfaces", "Enumerate Infrastructure and Application Admin Interfaces")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/05-Enumerate_Infrastructure_and_Application_Admin_Interfaces", "Enumerate Infrastructure and Application Admin Interfaces")</f>
         <v/>
       </c>
       <c r="D22" s="16" t="inlineStr">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="C23" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/06-Test_HTTP_Methods", "Test HTTP Methods")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/06-HTTP_Methods", "HTTP Methods")</f>
         <v/>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="C24" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/07-Test_HTTP_Strict_Transport_Security", "Test HTTP Strict Transport Security")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/07-HTTP_Strict_Transport_Security", "HTTP Strict Transport Security")</f>
         <v/>
       </c>
       <c r="D24" s="16" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="C25" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/09-Test_File_Permission", "Test File Permission")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/09-File_Permission", "File Permission")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="inlineStr">
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="C26" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/10-Test_for_Subdomain_Takeover", "Test for Subdomain Takeover")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/10-Subdomain_Takeover", "Subdomain Takeover")</f>
         <v/>
       </c>
       <c r="D26" s="16" t="inlineStr">
@@ -2034,7 +2034,7 @@
         </is>
       </c>
       <c r="C27" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/11-Test_Cloud_Storage", "Test Cloud Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/11-Cloud_Storage", "Cloud Storage")</f>
         <v/>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -2057,7 +2057,7 @@
         </is>
       </c>
       <c r="C28" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/12-Test_for_Content_Security_Policy", "Test for Content Security Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/12-Content_Security_Policy", "Content Security Policy")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="inlineStr">
@@ -2080,7 +2080,7 @@
         </is>
       </c>
       <c r="C29" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/13-Test_for_Path_Confusion", "Test Path Confusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/13-Path_Confusion", "Path Confusion")</f>
         <v/>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="C30" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management_Testing/14-Test_Other_HTTP_Security_Header_Misconfigurations", "Test Other HTTP Security Header Misconfigurations")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/02-Configuration_and_Deployment_Management/14-Other_HTTP_Security_Header_Misconfigurations", "Other HTTP Security Header Misconfigurations")</f>
         <v/>
       </c>
       <c r="D30" s="16" t="inlineStr">
@@ -2132,7 +2132,7 @@
       <c r="A32" s="9" t="n"/>
       <c r="B32" s="100" t="inlineStr">
         <is>
-          <t>Identity Management Testing</t>
+          <t>Identity Management</t>
         </is>
       </c>
       <c r="C32" s="101" t="inlineStr">
@@ -2164,7 +2164,7 @@
         </is>
       </c>
       <c r="C33" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/01-Test_Role_Definitions", "Test Role Definitions")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/01-Role_Definitions", "Role Definitions")</f>
         <v/>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="C34" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/02-Test_User_Registration_Process", "Test User Registration Process")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/02-User_Registration_Process", "User Registration Process")</f>
         <v/>
       </c>
       <c r="D34" s="16" t="inlineStr">
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="C35" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/03-Test_Account_Provisioning_Process", "Test Account Provisioning Process")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/03-Account_Provisioning_Process", "Account Provisioning Process")</f>
         <v/>
       </c>
       <c r="D35" s="16" t="inlineStr">
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="C36" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/04-Testing_for_Account_Enumeration_and_Guessable_User_Account", "Testing for Account Enumeration and Guessable User Account")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/04-Account_Enumeration_and_Guessable_User_Account", "Account Enumeration and Guessable User Account")</f>
         <v/>
       </c>
       <c r="D36" s="16" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="F36" s="18" t="n"/>
     </row>
-    <row r="37" ht="33" customHeight="1" s="82">
+    <row r="37" ht="16.5" customHeight="1" s="82">
       <c r="A37" s="19" t="n"/>
       <c r="B37" s="34" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="C37" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management_Testing/05-Testing_for_Weak_or_Unenforced_Username_Policy", "Testing for Weak or Unenforced Username Policy")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/03-Identity_Management/05-Weak_or_Unenforced_Username_Policy", "Weak or Unenforced Username Policy")</f>
         <v/>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -2287,7 +2287,7 @@
       <c r="A39" s="9" t="n"/>
       <c r="B39" s="100" t="inlineStr">
         <is>
-          <t>Authentication Testing</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C39" s="101" t="inlineStr">
@@ -2319,7 +2319,7 @@
         </is>
       </c>
       <c r="C40" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/01-Testing_for_Credentials_Transported_over_an_Encrypted_Channel", "Testing for Credentials Transported over an Encrypted Channel")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/01-Credentials_Transported_over_an_Encrypted_Channel", "Credentials Transported over an Encrypted Channel")</f>
         <v/>
       </c>
       <c r="D40" s="16" t="inlineStr">
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="C41" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/02-Testing_for_Default_Credentials", "Testing for Default Credentials")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/02-Default_Credentials", "Default Credentials")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="C42" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/03-Testing_for_Weak_Lock_Out_Mechanism", "Testing for Weak Lock Out Mechanism")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/03-Weak_Lock_Out_Mechanism", "Weak Lock Out Mechanism")</f>
         <v/>
       </c>
       <c r="D42" s="16" t="inlineStr">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="C43" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/04-Testing_for_Bypassing_Authentication_Schema", "Testing for Bypassing Authentication Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/04-Bypassing_Authentication_Schema", "Bypassing Authentication Schema")</f>
         <v/>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -2413,7 +2413,7 @@
         </is>
       </c>
       <c r="C44" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/05-Testing_for_Vulnerable_Remember_Password", "Testing for Vulnerable Remember Password")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/05-Vulnerable_Remember_Password", "Vulnerable Remember Password")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="inlineStr">
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="C45" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/06-Testing_for_Browser_Cache_Weaknesses", "Testing for Browser Cache Weaknesses")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/06-Browser_Cache_Weaknesses", "Browser Cache Weaknesses")</f>
         <v/>
       </c>
       <c r="D45" s="16" t="inlineStr">
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="C46" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/07-Testing_for_Weak_Authentication_Methods", "Testing for Weak Authentication Methods")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/07-Weak_Authentication_Methods", "Weak Authentication Methods")</f>
         <v/>
       </c>
       <c r="D46" s="16" t="inlineStr">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="C47" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/08-Testing_for_Weak_Security_Question_Answer", "Testing for Weak Security Question Answer")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/08-Weak_Security_Question_Answer", "Weak Security Question Answer")</f>
         <v/>
       </c>
       <c r="D47" s="16" t="inlineStr">
@@ -2507,7 +2507,7 @@
         </is>
       </c>
       <c r="C48" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/09-Testing_for_Weak_Password_Change_or_Reset_Functionalities", "Testing for Weak Password Change or Reset Functionalities")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/09-Weak_Password_Change_or_Reset_Functionalities", "Weak Password Change or Reset Functionalities")</f>
         <v/>
       </c>
       <c r="D48" s="16" t="inlineStr">
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="C49" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/10-Testing_for_Weaker_Authentication_in_Alternative_Channel", "Testing for Weaker Authentication in Alternative Channel")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/10-Weaker_Authentication_in_Alternative_Channel", "Weaker Authentication in Alternative Channel")</f>
         <v/>
       </c>
       <c r="D49" s="16" t="inlineStr">
@@ -2554,7 +2554,7 @@
         </is>
       </c>
       <c r="C50" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication_Testing/11-Testing_Multi-Factor_Authentication", "Testing Multi-Factor Authentication (MFA)")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/04-Authentication/11-Multi-Factor_Authentication", "Multi-Factor Authentication (MFA)")</f>
         <v/>
       </c>
       <c r="D50" s="16" t="inlineStr">
@@ -2583,7 +2583,7 @@
       <c r="A52" s="9" t="n"/>
       <c r="B52" s="100" t="inlineStr">
         <is>
-          <t>Authorization Testing</t>
+          <t>Authorization</t>
         </is>
       </c>
       <c r="C52" s="101" t="inlineStr">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="C53" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/01-Testing_Directory_Traversal_File_Include", "Testing Directory Traversal File Include")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/01-Directory_Traversal_File_Include", "Directory Traversal File Include")</f>
         <v/>
       </c>
       <c r="D53" s="16" t="inlineStr">
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="C54" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/02-Testing_for_Bypassing_Authorization_Schema", "Testing for Bypassing Authorization Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/02-Bypassing_Authorization_Schema", "Bypassing Authorization Schema")</f>
         <v/>
       </c>
       <c r="D54" s="16" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="C55" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/03-Testing_for_Privilege_Escalation", "Testing for Privilege Escalation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/03-Privilege_Escalation", "Privilege Escalation")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="inlineStr">
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="C56" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/04-Testing_for_Insecure_Direct_Object_References", "Testing for Insecure Direct Object References")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/04-Insecure_Direct_Object_References", "Insecure Direct Object References")</f>
         <v/>
       </c>
       <c r="D56" s="16" t="inlineStr">
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="C57" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization_Testing/05-Testing_for_OAuth_Weaknesses", "Testing for OAuth Weaknesses")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/05-Authorization/05-OAuth_Weaknesses", "OAuth Weaknesses")</f>
         <v/>
       </c>
       <c r="D57" s="16" t="inlineStr">
@@ -2737,7 +2737,7 @@
       <c r="A59" s="9" t="n"/>
       <c r="B59" s="100" t="inlineStr">
         <is>
-          <t>Session Management Testing</t>
+          <t>Session Management</t>
         </is>
       </c>
       <c r="C59" s="101" t="inlineStr">
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="C60" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/01-Testing_for_Session_Management_Schema", "Testing for Session Management Schema")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/01-Session_Management_Schema", "Session Management Schema")</f>
         <v/>
       </c>
       <c r="D60" s="16" t="inlineStr">
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="C61" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/02-Testing_for_Cookies_Attributes", "Testing for Cookies Attributes")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/02-Cookies_Attributes", "Cookies Attributes")</f>
         <v/>
       </c>
       <c r="D61" s="16" t="inlineStr">
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="C62" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/03-Testing_for_Session_Fixation", "Testing for Session Fixation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/03-Session_Fixation", "Session Fixation")</f>
         <v/>
       </c>
       <c r="D62" s="16" t="inlineStr">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="C63" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/04-Testing_for_Exposed_Session_Variables", "Testing for Exposed Session Variables")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/04-Exposed_Session_Variables", "Exposed Session Variables")</f>
         <v/>
       </c>
       <c r="D63" s="16" t="inlineStr">
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="C64" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/05-Testing_for_Cross_Site_Request_Forgery", "Testing for Cross Site Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/05-Cross_Site_Request_Forgery", "Cross Site Request Forgery")</f>
         <v/>
       </c>
       <c r="D64" s="16" t="inlineStr">
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="C65" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/06-Testing_for_Logout_Functionality", "Testing for Logout Functionality")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/06-Logout_Functionality", "Logout Functionality")</f>
         <v/>
       </c>
       <c r="D65" s="16" t="inlineStr">
@@ -2913,7 +2913,7 @@
         </is>
       </c>
       <c r="C66" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/07-Testing_Session_Timeout", "Testing Session Timeout")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/07-Session_Timeout", "Session Timeout")</f>
         <v/>
       </c>
       <c r="D66" s="16" t="inlineStr">
@@ -2936,7 +2936,7 @@
         </is>
       </c>
       <c r="C67" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/08-Testing_for_Session_Puzzling", "Testing for Session Puzzling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/08-Session_Puzzling", "Session Puzzling")</f>
         <v/>
       </c>
       <c r="D67" s="16" t="inlineStr">
@@ -2960,7 +2960,7 @@
         </is>
       </c>
       <c r="C68" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/09-Testing_for_Session_Hijacking", "Testing for Session Hijacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/09-Session_Hijacking", "Session Hijacking")</f>
         <v/>
       </c>
       <c r="D68" s="16" t="inlineStr">
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="C69" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/10-Testing_JSON_Web_Tokens", "Testing JSON Web Tokens")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/10-JSON_Web_Tokens", "JSON Web Tokens")</f>
         <v/>
       </c>
       <c r="D69" s="16" t="inlineStr">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="C70" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management_Testing/11-Testing_for_Concurrent_Sessions", "Testing for Concurrent Sessions")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/06-Session_Management/11-Concurrent_Sessions", "Concurrent Sessions")</f>
         <v/>
       </c>
       <c r="D70" s="16" t="inlineStr">
@@ -3035,7 +3035,7 @@
       <c r="A72" s="9" t="n"/>
       <c r="B72" s="100" t="inlineStr">
         <is>
-          <t>Injection Testing</t>
+          <t>Injection</t>
         </is>
       </c>
       <c r="C72" s="101" t="inlineStr">
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="C73" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/01-Testing_for_Reflected_Cross_Site_Scripting", "Testing for Reflected Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/01-Reflected_Cross_Site_Scripting", "Reflected Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D73" s="16" t="inlineStr">
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="C74" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/02-Testing_for_Stored_Cross_Site_Scripting", "Testing for Stored Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/02-Stored_Cross_Site_Scripting", "Stored Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D74" s="16" t="inlineStr">
@@ -3115,7 +3115,7 @@
         </is>
       </c>
       <c r="C75" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/03-Testing_for_HTTP_Verb_Tampering", "Testing for HTTP Verb Tampering")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/03-HTTP_Verb_Tampering", "HTTP Verb Tampering")</f>
         <v/>
       </c>
       <c r="D75" s="16" t="inlineStr">
@@ -3138,7 +3138,7 @@
         </is>
       </c>
       <c r="C76" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/04-Testing_for_HTTP_Parameter_Pollution", "Testing for HTTP Parameter Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/04-HTTP_Parameter_Pollution", "HTTP Parameter Pollution")</f>
         <v/>
       </c>
       <c r="D76" s="16" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="C77" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/05-Testing_for_SQL_Injection", "Testing for SQL Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/05-SQL_Injection", "SQL Injection")</f>
         <v/>
       </c>
       <c r="D77" s="16" t="inlineStr">
@@ -3186,7 +3186,7 @@
         </is>
       </c>
       <c r="C78" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/06-Testing_for_LDAP_Injection", "Testing for LDAP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/06-LDAP_Injection", "LDAP Injection")</f>
         <v/>
       </c>
       <c r="D78" s="16" t="inlineStr">
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="C79" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/07-Testing_for_XML_Injection", "Testing for XML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/07-XML_Injection", "XML Injection")</f>
         <v/>
       </c>
       <c r="D79" s="16" t="inlineStr">
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="C80" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/08-Testing_for_SSI_Injection", "Testing for SSI Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/08-SSI_Injection", "SSI Injection")</f>
         <v/>
       </c>
       <c r="D80" s="16" t="inlineStr">
@@ -3258,7 +3258,7 @@
         </is>
       </c>
       <c r="C81" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/09-Testing_for_XPath_Injection", "Testing for XPath Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/09-XPath_Injection", "XPath Injection")</f>
         <v/>
       </c>
       <c r="D81" s="16" t="inlineStr">
@@ -3281,7 +3281,7 @@
         </is>
       </c>
       <c r="C82" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/10-Testing_for_IMAP_SMTP_Injection", "Testing for IMAP SMTP Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/10-IMAP_SMTP_Injection", "IMAP SMTP Injection")</f>
         <v/>
       </c>
       <c r="D82" s="16" t="inlineStr">
@@ -3306,7 +3306,7 @@
         </is>
       </c>
       <c r="C83" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/11-Testing_for_Code_Injection", "Testing for Code Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/11-Code_Injection", "Code Injection")</f>
         <v/>
       </c>
       <c r="D83" s="16" t="inlineStr">
@@ -3330,7 +3330,7 @@
         </is>
       </c>
       <c r="C84" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/12-Testing_for_Command_Injection", "Testing for Command Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/12-Command_Injection", "Command Injection")</f>
         <v/>
       </c>
       <c r="D84" s="16" t="inlineStr">
@@ -3354,7 +3354,7 @@
         </is>
       </c>
       <c r="C85" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/13-Testing_for_Format_String_Injection", "Testing for Format String Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/13-Format_String_Injection", "Format String Injection")</f>
         <v/>
       </c>
       <c r="D85" s="16" t="inlineStr">
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="C86" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/14-Testing_for_Incubated_Vulnerability", "Testing for Incubated Vulnerability")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/14-Incubated_Vulnerability", "Incubated Vulnerability")</f>
         <v/>
       </c>
       <c r="D86" s="16" t="inlineStr">
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="C87" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/15-Testing_for_HTTP_Response_Splitting", "Testing for HTTP Response Splitting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/15-HTTP_Response_Splitting", "HTTP Response Splitting")</f>
         <v/>
       </c>
       <c r="D87" s="16" t="inlineStr">
@@ -3427,7 +3427,7 @@
         </is>
       </c>
       <c r="C88" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/16-Testing_for_HTTP_Request_Smuggling", "Testing for HTTP Request Smuggling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/16-HTTP_Request_Smuggling", "HTTP Request Smuggling")</f>
         <v/>
       </c>
       <c r="D88" s="16" t="inlineStr">
@@ -3454,7 +3454,7 @@
         </is>
       </c>
       <c r="C89" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/17-Testing_for_Host_Header_Injection", "Testing for Host Header Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/17-Host_Header_Injection", "Host Header Injection")</f>
         <v/>
       </c>
       <c r="D89" s="16" t="inlineStr">
@@ -3478,7 +3478,7 @@
         </is>
       </c>
       <c r="C90" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/18-Testing_for_Server-side_Template_Injection", "Testing for Server-side Template Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/18-Server-side_Template_Injection", "Server-side Template Injection")</f>
         <v/>
       </c>
       <c r="D90" s="16" t="inlineStr">
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="C91" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/19-Testing_for_Server-Side_Request_Forgery", "Testing for Server-Side Request Forgery")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/19-Server-Side_Request_Forgery", "Server-Side Request Forgery")</f>
         <v/>
       </c>
       <c r="D91" s="16" t="inlineStr">
@@ -3528,7 +3528,7 @@
         </is>
       </c>
       <c r="C92" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/20-Testing_for_Mass_Assignment", "Testing for Mass Assignment")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/20-Mass_Assignment", "Mass Assignment")</f>
         <v/>
       </c>
       <c r="D92" s="16" t="inlineStr">
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="C93" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/21-Testing_for_CSV_Injection", "Testing for CSV Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/21-CSV_Injection", "CSV Injection")</f>
         <v/>
       </c>
       <c r="D93" s="16" t="inlineStr">
@@ -3579,7 +3579,7 @@
         </is>
       </c>
       <c r="C94" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/22-Testing_for_Prototype_Pollution", "Testing for Prototype Pollution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/22-Prototype_Pollution", "Prototype Pollution")</f>
         <v/>
       </c>
       <c r="D94" s="16" t="inlineStr">
@@ -3604,7 +3604,7 @@
         </is>
       </c>
       <c r="C95" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection_Testing/23-Testing_for_Insecure_Deserialization", "Testing for Insecure Deserialization")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/07-Injection/23-Insecure_Deserialization", "Insecure Deserialization")</f>
         <v/>
       </c>
       <c r="D95" s="16" t="inlineStr">
@@ -3636,7 +3636,7 @@
       <c r="A97" s="9" t="n"/>
       <c r="B97" s="100" t="inlineStr">
         <is>
-          <t>Testing for Error Handling</t>
+          <t>Error Handling</t>
         </is>
       </c>
       <c r="C97" s="101" t="inlineStr">
@@ -3668,7 +3668,7 @@
         </is>
       </c>
       <c r="C98" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/01-Testing_For_Improper_Error_Handling", "Testing for Improper Error Handling")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/01-Improper_Error_Handling", "Improper Error Handling")</f>
         <v/>
       </c>
       <c r="D98" s="16" t="inlineStr">
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="C99" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Testing_for_Error_Handling/02-Testing_for_Stack_Traces", "Testing for Stack Traces")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/08-Error_Handling/02-Stack_Traces", "Stack Traces")</f>
         <v/>
       </c>
       <c r="D99" s="16" t="inlineStr">
@@ -3719,7 +3719,7 @@
       <c r="A101" s="9" t="n"/>
       <c r="B101" s="100" t="inlineStr">
         <is>
-          <t>Testing for Weak Cryptography</t>
+          <t>Weak Cryptography</t>
         </is>
       </c>
       <c r="C101" s="101" t="inlineStr">
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="C102" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/01-Testing_for_Weak_Transport_Layer_Security", "Testing for Weak Transport Layer Security")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/01-Weak_Transport_Layer_Security", "Weak Transport Layer Security")</f>
         <v/>
       </c>
       <c r="D102" s="16" t="inlineStr">
@@ -3776,7 +3776,7 @@
         </is>
       </c>
       <c r="C103" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/02-Testing_for_Padding_Oracle", "Testing for Padding Oracle")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/02-Padding_Oracle", "Padding Oracle")</f>
         <v/>
       </c>
       <c r="D103" s="16" t="inlineStr">
@@ -3800,7 +3800,7 @@
         </is>
       </c>
       <c r="C104" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/03-Testing_for_Sensitive_Information_Sent_via_Unencrypted_Channels", "Testing for Sensitive Information Sent via Unencrypted Channels")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/03-Sensitive_Information_Sent_via_Unencrypted_Channels", "Sensitive Information Sent via Unencrypted Channels")</f>
         <v/>
       </c>
       <c r="D104" s="16" t="inlineStr">
@@ -3824,7 +3824,7 @@
         </is>
       </c>
       <c r="C105" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Testing_for_Weak_Cryptography/04-Testing_for_Weak_Cryptographic_Primitives", "Testing for Weak Cryptographic Primitives")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/09-Weak_Cryptography/04-Weak_Cryptographic_Primitives", "Weak Cryptographic Primitives")</f>
         <v/>
       </c>
       <c r="D105" s="16" t="inlineStr">
@@ -3851,7 +3851,7 @@
       <c r="A107" s="9" t="n"/>
       <c r="B107" s="100" t="inlineStr">
         <is>
-          <t>Business Logic Testing</t>
+          <t>Business Logic</t>
         </is>
       </c>
       <c r="C107" s="101" t="inlineStr">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="C108" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/01-Test_Business_Logic_Data_Validation", "Test Business Logic Data Validation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/01-Business_Logic_Data_Validation", "Business Logic Data Validation")</f>
         <v/>
       </c>
       <c r="D108" s="16" t="inlineStr">
@@ -3908,7 +3908,7 @@
         </is>
       </c>
       <c r="C109" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/02-Test_Ability_to_Forge_Requests", "Test Ability to Forge Requests")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/02-Ability_to_Forge_Requests", "Ability to Forge Requests")</f>
         <v/>
       </c>
       <c r="D109" s="16" t="inlineStr">
@@ -3932,7 +3932,7 @@
         </is>
       </c>
       <c r="C110" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/03-Test_Integrity_Checks", "Test Integrity Checks")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/03-Integrity_Checks", "Integrity Checks")</f>
         <v/>
       </c>
       <c r="D110" s="16" t="inlineStr">
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="C111" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/04-Test_for_Process_Timing", "Test for Process Timing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/04-Process_Timing", "Process Timing")</f>
         <v/>
       </c>
       <c r="D111" s="16" t="inlineStr">
@@ -3982,7 +3982,7 @@
         </is>
       </c>
       <c r="C112" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/05-Test_Number_of_Times_a_Function_Can_Be_Used_Limits", "Test Number of Times a Function Can Be Used Limits")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/05-Number_of_Times_a_Function_Can_Be_Used_Limits", "Number of Times a Function Can Be Used Limits")</f>
         <v/>
       </c>
       <c r="D112" s="16" t="inlineStr">
@@ -4006,7 +4006,7 @@
         </is>
       </c>
       <c r="C113" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/06-Testing_for_the_Circumvention_of_Work_Flows", "Testing for the Circumvention of Work Flows")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/06-Circumvention_of_Work_Flows", "Circumvention of Work Flows")</f>
         <v/>
       </c>
       <c r="D113" s="16" t="inlineStr">
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="C114" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/07-Test_Defenses_Against_Application_Misuse", "Test Defenses Against Application Misuse")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/07-Defenses_Against_Application_Misuse", "Defenses Against Application Misuse")</f>
         <v/>
       </c>
       <c r="D114" s="16" t="inlineStr">
@@ -4055,7 +4055,7 @@
         </is>
       </c>
       <c r="C115" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/08-Test_Upload_of_Unexpected_File_Types", "Test Upload of Unexpected File Types")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/08-Upload_of_Unexpected_File_Types", "Upload of Unexpected File Types")</f>
         <v/>
       </c>
       <c r="D115" s="16" t="inlineStr">
@@ -4080,7 +4080,7 @@
         </is>
       </c>
       <c r="C116" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/09-Test_Upload_of_Malicious_Files", "Test Upload of Malicious Files")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/09-Upload_of_Malicious_Files", "Upload of Malicious Files")</f>
         <v/>
       </c>
       <c r="D116" s="16" t="inlineStr">
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="C117" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic_Testing/10-Test-Payment-Functionality", "Test Payment Functionality")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/10-Business_Logic/10-Payment_Functionality", "Payment Functionality")</f>
         <v/>
       </c>
       <c r="D117" s="16" t="inlineStr">
@@ -4137,7 +4137,7 @@
       <c r="A119" s="9" t="n"/>
       <c r="B119" s="100" t="inlineStr">
         <is>
-          <t>Client-side Testing</t>
+          <t>Client-side</t>
         </is>
       </c>
       <c r="C119" s="101" t="inlineStr">
@@ -4169,7 +4169,7 @@
         </is>
       </c>
       <c r="C120" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/01-Testing_for_DOM-based_Cross_Site_Scripting", "Testing for DOM-Based Cross Site Scripting")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/01-DOM-based_Cross_Site_Scripting", "DOM-Based Cross Site Scripting")</f>
         <v/>
       </c>
       <c r="D120" s="16" t="inlineStr">
@@ -4193,7 +4193,7 @@
         </is>
       </c>
       <c r="C121" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/02-Testing_for_JavaScript_Execution", "Testing for JavaScript Execution")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/02-JavaScript_Execution", "JavaScript Execution")</f>
         <v/>
       </c>
       <c r="D121" s="16" t="inlineStr">
@@ -4216,7 +4216,7 @@
         </is>
       </c>
       <c r="C122" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/03-Testing_for_HTML_Injection", "Testing for HTML Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/03-HTML_Injection", "HTML Injection")</f>
         <v/>
       </c>
       <c r="D122" s="16" t="inlineStr">
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="C123" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/04-Testing_for_Client-side_URL_Redirect", "Testing for Client-side URL Redirect")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/04-Client-side_URL_Redirect", "Client-side URL Redirect")</f>
         <v/>
       </c>
       <c r="D123" s="16" t="inlineStr">
@@ -4263,7 +4263,7 @@
         </is>
       </c>
       <c r="C124" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/05-Testing_for_CSS_Injection", "Testing for CSS Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/05-CSS_Injection", "CSS Injection")</f>
         <v/>
       </c>
       <c r="D124" s="16" t="inlineStr">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="C125" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/06-Testing_for_Client-side_Resource_Manipulation", "Testing for Client-side Resource Manipulation")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/06-Client-side_Resource_Manipulation", "Client-side Resource Manipulation")</f>
         <v/>
       </c>
       <c r="D125" s="16" t="inlineStr">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="C126" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/07-Testing_Cross_Origin_Resource_Sharing", "Testing Cross Origin Resource Sharing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/07-Cross_Origin_Resource_Sharing", "Cross Origin Resource Sharing")</f>
         <v/>
       </c>
       <c r="D126" s="16" t="inlineStr">
@@ -4335,7 +4335,7 @@
         </is>
       </c>
       <c r="C127" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/09-Testing_for_Clickjacking", "Testing for Clickjacking")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/09-Clickjacking", "Clickjacking")</f>
         <v/>
       </c>
       <c r="D127" s="16" t="inlineStr">
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="C128" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/10-Testing_WebSockets", "Testing WebSockets")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/10-WebSockets", "WebSockets")</f>
         <v/>
       </c>
       <c r="D128" s="16" t="inlineStr">
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="C129" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/11-Testing_Web_Messaging", "Testing Web Messaging")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/11-Web_Messaging", "Web Messaging")</f>
         <v/>
       </c>
       <c r="D129" s="16" t="inlineStr">
@@ -4406,7 +4406,7 @@
         </is>
       </c>
       <c r="C130" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/12-Testing_Browser_Storage", "Testing Browser Storage")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/12-Browser_Storage", "Browser Storage")</f>
         <v/>
       </c>
       <c r="D130" s="16" t="inlineStr">
@@ -4430,7 +4430,7 @@
         </is>
       </c>
       <c r="C131" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/13-Testing_for_Cross_Site_Script_Inclusion", "Testing for Cross Site Script Inclusion")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/13-Cross_Site_Script_Inclusion", "Cross Site Script Inclusion")</f>
         <v/>
       </c>
       <c r="D131" s="16" t="inlineStr">
@@ -4454,7 +4454,7 @@
         </is>
       </c>
       <c r="C132" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/14-Testing_for_Reverse_Tabnabbing", "Testing for Reverse Tabnabbing")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/14-Reverse_Tabnabbing", "Reverse Tabnabbing")</f>
         <v/>
       </c>
       <c r="D132" s="16" t="inlineStr">
@@ -4477,7 +4477,7 @@
         </is>
       </c>
       <c r="C133" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side_Testing/15-Testing_for_Client-Side_Template_Injection", "Testing for Client-side Template Injection")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/11-Client-side/15-Client-Side_Template_Injection", "Client-side Template Injection")</f>
         <v/>
       </c>
       <c r="D133" s="16" t="inlineStr">
@@ -4586,7 +4586,7 @@
         </is>
       </c>
       <c r="C138" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Testing_for_Excessive_Data_Exposure", "Testing for Excessive Data Exposure")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/03-Excessive_Data_Exposure", "Excessive Data Exposure")</f>
         <v/>
       </c>
       <c r="D138" s="16" t="inlineStr">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="C140" s="15">
-        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-Testing_GraphQL", "Testing GraphQL")</f>
+        <f>HYPERLINK("https://owasp.org/www-project-web-security-testing-guide/latest/4-Web_Application_Security_Testing/12-API_Testing/99-GraphQL", "GraphQL")</f>
         <v/>
       </c>
       <c r="D140" s="16" t="inlineStr">

</xml_diff>